<commit_message>
Refactor scouting and signability configurations in credentials. Introduce new parameters for scouting trust and signability penalties in the environment file. Update related functions to utilize these configurations, enhancing the flexibility and accuracy of player evaluation during the draft process.
</commit_message>
<xml_diff>
--- a/Season x amateur draft-template.xlsx
+++ b/Season x amateur draft-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13362ca80da55a94/Documents/hardball-dynasty-draft-optimizer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3BD80D3-44C8-45D2-AC5C-31D7F3876EE2}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4A6E41B-B920-4826-824B-E20F97D11AED}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hitters" sheetId="1" r:id="rId1"/>
@@ -1322,6 +1322,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1337,7 +1338,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -11403,6 +11403,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -11987,13 +11991,13 @@
         <v>2</v>
       </c>
       <c r="J1" s="1">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="K1" s="1">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="L1" s="1">
-        <v>2.2000000000000002</v>
+        <v>1.6</v>
       </c>
       <c r="M1" s="8">
         <v>1</v>
@@ -12043,13 +12047,13 @@
         <v>0.1</v>
       </c>
       <c r="AH1" s="1"/>
-      <c r="AI1" s="22" t="s">
+      <c r="AI1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="AJ1" s="23"/>
-      <c r="AK1" s="23"/>
-      <c r="AL1" s="23"/>
-      <c r="AM1" s="23"/>
+      <c r="AJ1" s="24"/>
+      <c r="AK1" s="24"/>
+      <c r="AL1" s="24"/>
+      <c r="AM1" s="24"/>
     </row>
     <row r="2" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2"/>
@@ -12101,18 +12105,18 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="24">
+      <c r="H3" s="25">
         <v>2.5</v>
       </c>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26">
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27">
         <v>0.6</v>
       </c>
-      <c r="N3" s="26"/>
-      <c r="O3" s="25"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="26"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
@@ -12120,23 +12124,23 @@
       <c r="T3" s="7"/>
       <c r="U3" s="7"/>
       <c r="V3" s="7"/>
-      <c r="W3" s="24">
+      <c r="W3" s="25">
         <v>2</v>
       </c>
-      <c r="X3" s="26"/>
-      <c r="Y3" s="26"/>
-      <c r="Z3" s="26"/>
-      <c r="AA3" s="25"/>
-      <c r="AB3" s="24">
+      <c r="X3" s="27"/>
+      <c r="Y3" s="27"/>
+      <c r="Z3" s="27"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="25">
         <v>1</v>
       </c>
-      <c r="AC3" s="25"/>
-      <c r="AD3" s="24">
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="25">
         <v>0.6</v>
       </c>
-      <c r="AE3" s="26"/>
-      <c r="AF3" s="26"/>
-      <c r="AG3" s="25"/>
+      <c r="AE3" s="27"/>
+      <c r="AF3" s="27"/>
+      <c r="AG3" s="26"/>
       <c r="AH3" s="1"/>
     </row>
     <row r="4" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -12255,7 +12259,7 @@
       <c r="AH5" s="1"/>
       <c r="AI5" s="6">
         <f>H$1*((-2*10^-6)*H5^3+0.00032*H5^2-0.0021*H5)+I$1*((-2*10^-6)*I5^3+0.00032*I5^2-0.0021*I5)+J$1*((-2*10^-6)*J5^3+0.00032*J5^2-0.0021*J5)+K$1*((-2*10^-6)*K5^3+0.00032*K5^2-0.0021*K5)+L$1*((-2*10^-6)*L5^3+0.00032*L5^2-0.0021*L5)</f>
-        <v>6.5340000000000025</v>
+        <v>6.5340000000000016</v>
       </c>
       <c r="AJ5" s="6">
         <f>(M$1*M5+N$1*N5+O$1*O5)/100</f>
@@ -12275,7 +12279,7 @@
       </c>
     </row>
     <row r="6" spans="1:39" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="22" t="s">
         <v>25</v>
       </c>
       <c r="B6" s="14" t="s">
@@ -12396,7 +12400,7 @@
     <row r="7" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
         <f t="shared" ref="A7:A70" si="0">(AI7*H$3+AJ7*M$3+AK7*W$3+AL7*AB$3+AM7*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>76.925821122683445</v>
+        <v>78.859066668656183</v>
       </c>
       <c r="B7" s="18">
         <v>1</v>
@@ -12499,7 +12503,7 @@
       </c>
       <c r="AI7" s="6">
         <f t="shared" ref="AI7:AI70" si="1">H$1*((-2*10^-6)*H7^3+0.00032*H7^2-0.0021*H7)+I$1*((-2*10^-6)*I7^3+0.00032*I7^2-0.0021*I7)+J$1*((-2*10^-6)*J7^3+0.00032*J7^2-0.0021*J7)+K$1*((-2*10^-6)*K7^3+0.00032*K7^2-0.0021*K7)+L$1*((-2*10^-6)*L7^3+0.00032*L7^2-0.0021*L7)</f>
-        <v>5.3988432000000017</v>
+        <v>5.6061428000000015</v>
       </c>
       <c r="AJ7" s="6">
         <f t="shared" ref="AJ7:AJ70" si="2">(M$1*M7+N$1*N7+O$1*O7)/100</f>
@@ -12521,7 +12525,7 @@
     <row r="8" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <f t="shared" si="0"/>
-        <v>72.014497896087605</v>
+        <v>72.690376018383105</v>
       </c>
       <c r="B8" s="20">
         <v>10</v>
@@ -12624,7 +12628,7 @@
       </c>
       <c r="AI8" s="6">
         <f t="shared" si="1"/>
-        <v>5.0953000000000008</v>
+        <v>5.1677736000000012</v>
       </c>
       <c r="AJ8" s="6">
         <f t="shared" si="2"/>
@@ -12646,7 +12650,7 @@
     <row r="9" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <f t="shared" si="0"/>
-        <v>70.83639126801755</v>
+        <v>71.279525948252711</v>
       </c>
       <c r="B9" s="20">
         <v>48</v>
@@ -12749,7 +12753,7 @@
       </c>
       <c r="AI9" s="6">
         <f t="shared" si="1"/>
-        <v>4.4520432000000021</v>
+        <v>4.4995600000000016</v>
       </c>
       <c r="AJ9" s="6">
         <f t="shared" si="2"/>
@@ -12771,7 +12775,7 @@
     <row r="10" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <f t="shared" si="0"/>
-        <v>69.296207287594356</v>
+        <v>68.248138112148965</v>
       </c>
       <c r="B10" s="20">
         <v>4</v>
@@ -12874,7 +12878,7 @@
       </c>
       <c r="AI10" s="6">
         <f t="shared" si="1"/>
-        <v>4.2209900000000014</v>
+        <v>4.1086068000000013</v>
       </c>
       <c r="AJ10" s="6">
         <f t="shared" si="2"/>
@@ -12896,7 +12900,7 @@
     <row r="11" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <f t="shared" si="0"/>
-        <v>68.02485108478318</v>
+        <v>67.103684383300006</v>
       </c>
       <c r="B11" s="18">
         <v>5</v>
@@ -12999,7 +13003,7 @@
       </c>
       <c r="AI11" s="6">
         <f t="shared" si="1"/>
-        <v>4.638036800000001</v>
+        <v>4.5392612000000012</v>
       </c>
       <c r="AJ11" s="6">
         <f t="shared" si="2"/>
@@ -13021,7 +13025,7 @@
     <row r="12" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <f t="shared" si="0"/>
-        <v>66.583922826703258</v>
+        <v>66.324026231758637</v>
       </c>
       <c r="B12" s="20">
         <v>8</v>
@@ -13124,7 +13128,7 @@
       </c>
       <c r="AI12" s="6">
         <f t="shared" si="1"/>
-        <v>3.9783404000000013</v>
+        <v>3.9504720000000013</v>
       </c>
       <c r="AJ12" s="6">
         <f t="shared" si="2"/>
@@ -13146,7 +13150,7 @@
     <row r="13" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <f t="shared" si="0"/>
-        <v>65.503265540601006</v>
+        <v>64.191908890148909</v>
       </c>
       <c r="B13" s="18">
         <v>13</v>
@@ -13249,7 +13253,7 @@
       </c>
       <c r="AI13" s="6">
         <f t="shared" si="1"/>
-        <v>4.4067404000000012</v>
+        <v>4.2661252000000012</v>
       </c>
       <c r="AJ13" s="6">
         <f t="shared" si="2"/>
@@ -13271,7 +13275,7 @@
     <row r="14" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <f t="shared" si="0"/>
-        <v>64.294691127756721</v>
+        <v>61.978574562057958</v>
       </c>
       <c r="B14" s="20">
         <v>18</v>
@@ -13374,7 +13378,7 @@
       </c>
       <c r="AI14" s="6">
         <f t="shared" si="1"/>
-        <v>3.4845964000000009</v>
+        <v>3.2362420000000007</v>
       </c>
       <c r="AJ14" s="6">
         <f t="shared" si="2"/>
@@ -13396,7 +13400,7 @@
     <row r="15" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <f t="shared" si="0"/>
-        <v>63.859374197976649</v>
+        <v>61.924449998507875</v>
       </c>
       <c r="B15" s="18">
         <v>15</v>
@@ -13499,7 +13503,7 @@
       </c>
       <c r="AI15" s="6">
         <f t="shared" si="1"/>
-        <v>3.225820800000001</v>
+        <v>3.0183412000000014</v>
       </c>
       <c r="AJ15" s="6">
         <f t="shared" si="2"/>
@@ -13521,7 +13525,7 @@
     <row r="16" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <f t="shared" si="0"/>
-        <v>63.652450386463315</v>
+        <v>63.02113118863587</v>
       </c>
       <c r="B16" s="20">
         <v>2</v>
@@ -13624,7 +13628,7 @@
       </c>
       <c r="AI16" s="6">
         <f t="shared" si="1"/>
-        <v>5.3107792000000016</v>
+        <v>5.2430836000000012</v>
       </c>
       <c r="AJ16" s="6">
         <f t="shared" si="2"/>
@@ -13646,7 +13650,7 @@
     <row r="17" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <f t="shared" si="0"/>
-        <v>63.012815661464082</v>
+        <v>62.613598287027358</v>
       </c>
       <c r="B17" s="18">
         <v>47</v>
@@ -13749,7 +13753,7 @@
       </c>
       <c r="AI17" s="6">
         <f t="shared" si="1"/>
-        <v>3.9934440000000011</v>
+        <v>3.9506364000000005</v>
       </c>
       <c r="AJ17" s="6">
         <f t="shared" si="2"/>
@@ -13771,7 +13775,7 @@
     <row r="18" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <f t="shared" si="0"/>
-        <v>61.679461338744808</v>
+        <v>61.872032737473518</v>
       </c>
       <c r="B18" s="18">
         <v>21</v>
@@ -13874,7 +13878,7 @@
       </c>
       <c r="AI18" s="6">
         <f t="shared" si="1"/>
-        <v>3.5196468000000007</v>
+        <v>3.540296000000001</v>
       </c>
       <c r="AJ18" s="6">
         <f t="shared" si="2"/>
@@ -13896,7 +13900,7 @@
     <row r="19" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <f t="shared" si="0"/>
-        <v>60.362514697543929</v>
+        <v>58.970004476409308</v>
       </c>
       <c r="B19" s="18">
         <v>27</v>
@@ -13999,7 +14003,7 @@
       </c>
       <c r="AI19" s="6">
         <f t="shared" si="1"/>
-        <v>5.0269036000000016</v>
+        <v>4.8775864000000011</v>
       </c>
       <c r="AJ19" s="6">
         <f t="shared" si="2"/>
@@ -14021,7 +14025,7 @@
     <row r="20" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <f t="shared" si="0"/>
-        <v>59.785335283058259</v>
+        <v>59.661036587185514</v>
       </c>
       <c r="B20" s="20">
         <v>12</v>
@@ -14124,7 +14128,7 @@
       </c>
       <c r="AI20" s="6">
         <f t="shared" si="1"/>
-        <v>4.9341756000000005</v>
+        <v>4.9208472000000008</v>
       </c>
       <c r="AJ20" s="6">
         <f t="shared" si="2"/>
@@ -14146,7 +14150,7 @@
     <row r="21" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
         <f t="shared" si="0"/>
-        <v>57.673585156226679</v>
+        <v>55.63346160732938</v>
       </c>
       <c r="B21" s="20">
         <v>34</v>
@@ -14249,7 +14253,7 @@
       </c>
       <c r="AI21" s="6">
         <f t="shared" si="1"/>
-        <v>2.7674884000000008</v>
+        <v>2.5487284000000008</v>
       </c>
       <c r="AJ21" s="6">
         <f t="shared" si="2"/>
@@ -14271,7 +14275,7 @@
     <row r="22" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
         <f t="shared" si="0"/>
-        <v>57.610538661255177</v>
+        <v>58.660293950878859</v>
       </c>
       <c r="B22" s="20">
         <v>28</v>
@@ -14374,7 +14378,7 @@
       </c>
       <c r="AI22" s="6">
         <f t="shared" si="1"/>
-        <v>3.2055264000000006</v>
+        <v>3.3180904000000004</v>
       </c>
       <c r="AJ22" s="6">
         <f t="shared" si="2"/>
@@ -14396,7 +14400,7 @@
     <row r="23" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
         <f t="shared" si="0"/>
-        <v>56.941244591005386</v>
+        <v>57.577431883971471</v>
       </c>
       <c r="B23" s="18">
         <v>43</v>
@@ -14499,7 +14503,7 @@
       </c>
       <c r="AI23" s="6">
         <f t="shared" si="1"/>
-        <v>3.2149504000000011</v>
+        <v>3.2831680000000012</v>
       </c>
       <c r="AJ23" s="6">
         <f t="shared" si="2"/>
@@ -14521,7 +14525,7 @@
     <row r="24" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
         <f t="shared" si="0"/>
-        <v>56.898373123638414</v>
+        <v>58.631276970366159</v>
       </c>
       <c r="B24" s="20">
         <v>30</v>
@@ -14624,7 +14628,7 @@
       </c>
       <c r="AI24" s="6">
         <f t="shared" si="1"/>
-        <v>3.3149880000000005</v>
+        <v>3.5008052000000007</v>
       </c>
       <c r="AJ24" s="6">
         <f t="shared" si="2"/>
@@ -14646,7 +14650,7 @@
     <row r="25" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6">
         <f t="shared" si="0"/>
-        <v>56.833674982840414</v>
+        <v>58.234936584201243</v>
       </c>
       <c r="B25" s="20">
         <v>36</v>
@@ -14749,7 +14753,7 @@
       </c>
       <c r="AI25" s="6">
         <f t="shared" si="1"/>
-        <v>3.2838300000000005</v>
+        <v>3.4340856000000008</v>
       </c>
       <c r="AJ25" s="6">
         <f t="shared" si="2"/>
@@ -14771,7 +14775,7 @@
     <row r="26" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6">
         <f t="shared" si="0"/>
-        <v>54.867016473186297</v>
+        <v>54.381740129517446</v>
       </c>
       <c r="B26" s="20">
         <v>72</v>
@@ -14874,7 +14878,7 @@
       </c>
       <c r="AI26" s="6">
         <f t="shared" si="1"/>
-        <v>3.1083524000000007</v>
+        <v>3.0563168000000007</v>
       </c>
       <c r="AJ26" s="6">
         <f t="shared" si="2"/>
@@ -14896,7 +14900,7 @@
     <row r="27" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
         <f t="shared" si="0"/>
-        <v>54.489312125100696</v>
+        <v>55.504994479095153</v>
       </c>
       <c r="B27" s="18">
         <v>49</v>
@@ -14999,7 +15003,7 @@
       </c>
       <c r="AI27" s="6">
         <f t="shared" si="1"/>
-        <v>3.1717320000000009</v>
+        <v>3.2806424000000005</v>
       </c>
       <c r="AJ27" s="6">
         <f t="shared" si="2"/>
@@ -15021,7 +15025,7 @@
     <row r="28" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
         <f t="shared" si="0"/>
-        <v>54.308466531379615</v>
+        <v>54.321302635112943</v>
       </c>
       <c r="B28" s="20">
         <v>32</v>
@@ -15124,7 +15128,7 @@
       </c>
       <c r="AI28" s="6">
         <f t="shared" si="1"/>
-        <v>2.4663196000000012</v>
+        <v>2.467696000000001</v>
       </c>
       <c r="AJ28" s="6">
         <f t="shared" si="2"/>
@@ -15146,7 +15150,7 @@
     <row r="29" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
         <f t="shared" si="0"/>
-        <v>54.070408994598452</v>
+        <v>50.731671640454806</v>
       </c>
       <c r="B29" s="20">
         <v>182</v>
@@ -15249,7 +15253,7 @@
       </c>
       <c r="AI29" s="6">
         <f t="shared" si="1"/>
-        <v>4.7145608000000019</v>
+        <v>4.3565520000000024</v>
       </c>
       <c r="AJ29" s="6">
         <f t="shared" si="2"/>
@@ -15271,7 +15275,7 @@
     <row r="30" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
         <f t="shared" si="0"/>
-        <v>52.273470709361654</v>
+        <v>50.948509504909126</v>
       </c>
       <c r="B30" s="20">
         <v>68</v>
@@ -15374,7 +15378,7 @@
       </c>
       <c r="AI30" s="6">
         <f t="shared" si="1"/>
-        <v>1.7815540000000003</v>
+        <v>1.6394800000000005</v>
       </c>
       <c r="AJ30" s="6">
         <f t="shared" si="2"/>
@@ -15396,7 +15400,7 @@
     <row r="31" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
         <f t="shared" si="0"/>
-        <v>51.973672744635756</v>
+        <v>48.384562356381863</v>
       </c>
       <c r="B31" s="20">
         <v>42</v>
@@ -15499,7 +15503,7 @@
       </c>
       <c r="AI31" s="6">
         <f t="shared" si="1"/>
-        <v>4.0954768000000019</v>
+        <v>3.7106208000000018</v>
       </c>
       <c r="AJ31" s="6">
         <f t="shared" si="2"/>
@@ -15521,7 +15525,7 @@
     <row r="32" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
         <f t="shared" si="0"/>
-        <v>50.661999313617223</v>
+        <v>48.543766152376953</v>
       </c>
       <c r="B32" s="20">
         <v>44</v>
@@ -15624,7 +15628,7 @@
       </c>
       <c r="AI32" s="6">
         <f t="shared" si="1"/>
-        <v>2.7303256000000014</v>
+        <v>2.5031900000000005</v>
       </c>
       <c r="AJ32" s="6">
         <f t="shared" si="2"/>
@@ -15646,7 +15650,7 @@
     <row r="33" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
         <f t="shared" si="0"/>
-        <v>50.029231997373827</v>
+        <v>51.296518398042316</v>
       </c>
       <c r="B33" s="20">
         <v>26</v>
@@ -15749,7 +15753,7 @@
       </c>
       <c r="AI33" s="6">
         <f t="shared" si="1"/>
-        <v>2.720829600000001</v>
+        <v>2.856719200000001</v>
       </c>
       <c r="AJ33" s="6">
         <f t="shared" si="2"/>
@@ -15771,7 +15775,7 @@
     <row r="34" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
         <f t="shared" si="0"/>
-        <v>49.585065952430682</v>
+        <v>48.440477931302041</v>
       </c>
       <c r="B34" s="20">
         <v>56</v>
@@ -15874,7 +15878,7 @@
       </c>
       <c r="AI34" s="6">
         <f t="shared" si="1"/>
-        <v>3.017719200000001</v>
+        <v>2.8949864000000005</v>
       </c>
       <c r="AJ34" s="6">
         <f t="shared" si="2"/>
@@ -15896,7 +15900,7 @@
     <row r="35" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
         <f t="shared" si="0"/>
-        <v>49.23671849353903</v>
+        <v>49.516531379629342</v>
       </c>
       <c r="B35" s="18">
         <v>55</v>
@@ -15999,7 +16003,7 @@
       </c>
       <c r="AI35" s="6">
         <f t="shared" si="1"/>
-        <v>3.8082652000000001</v>
+        <v>3.8382692000000005</v>
       </c>
       <c r="AJ35" s="6">
         <f t="shared" si="2"/>
@@ -16021,7 +16025,7 @@
     <row r="36" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
         <f t="shared" si="0"/>
-        <v>49.108510997045563</v>
+        <v>50.551895610134586</v>
       </c>
       <c r="B36" s="18">
         <v>31</v>
@@ -16124,7 +16128,7 @@
       </c>
       <c r="AI36" s="6">
         <f t="shared" si="1"/>
-        <v>1.4027864000000003</v>
+        <v>1.5575588000000002</v>
       </c>
       <c r="AJ36" s="6">
         <f t="shared" si="2"/>
@@ -16146,7 +16150,7 @@
     <row r="37" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6">
         <f t="shared" si="0"/>
-        <v>49.02679623384762</v>
+        <v>48.358580232176443</v>
       </c>
       <c r="B37" s="20">
         <v>190</v>
@@ -16249,7 +16253,7 @@
       </c>
       <c r="AI37" s="6">
         <f t="shared" si="1"/>
-        <v>4.0803032000000012</v>
+        <v>4.0086512000000019</v>
       </c>
       <c r="AJ37" s="6">
         <f t="shared" si="2"/>
@@ -16271,7 +16275,7 @@
     <row r="38" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6">
         <f t="shared" si="0"/>
-        <v>48.919184696648657</v>
+        <v>47.923541735056247</v>
       </c>
       <c r="B38" s="18">
         <v>183</v>
@@ -16374,7 +16378,7 @@
       </c>
       <c r="AI38" s="6">
         <f t="shared" si="1"/>
-        <v>3.7008572000000006</v>
+        <v>3.5940956000000006</v>
       </c>
       <c r="AJ38" s="6">
         <f t="shared" si="2"/>
@@ -16396,7 +16400,7 @@
     <row r="39" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
         <f t="shared" si="0"/>
-        <v>48.456150884836902</v>
+        <v>49.433175713987282</v>
       </c>
       <c r="B39" s="20">
         <v>40</v>
@@ -16499,7 +16503,7 @@
       </c>
       <c r="AI39" s="6">
         <f t="shared" si="1"/>
-        <v>2.1485816000000009</v>
+        <v>2.2533468000000005</v>
       </c>
       <c r="AJ39" s="6">
         <f t="shared" si="2"/>
@@ -16521,7 +16525,7 @@
     <row r="40" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6">
         <f t="shared" si="0"/>
-        <v>48.252199707541244</v>
+        <v>46.570726073592162</v>
       </c>
       <c r="B40" s="18">
         <v>85</v>
@@ -16624,7 +16628,7 @@
       </c>
       <c r="AI40" s="6">
         <f t="shared" si="1"/>
-        <v>2.1332748000000006</v>
+        <v>1.9529724000000006</v>
       </c>
       <c r="AJ40" s="6">
         <f t="shared" si="2"/>
@@ -16646,7 +16650,7 @@
     <row r="41" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6">
         <f t="shared" si="0"/>
-        <v>48.212002447103757</v>
+        <v>47.578959831687008</v>
       </c>
       <c r="B41" s="20">
         <v>60</v>
@@ -16749,7 +16753,7 @@
       </c>
       <c r="AI41" s="6">
         <f t="shared" si="1"/>
-        <v>3.2439052000000008</v>
+        <v>3.1760248000000009</v>
       </c>
       <c r="AJ41" s="6">
         <f t="shared" si="2"/>
@@ -16771,7 +16775,7 @@
     <row r="42" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6">
         <f t="shared" si="0"/>
-        <v>46.634080097884137</v>
+        <v>46.580777253872093</v>
       </c>
       <c r="B42" s="20">
         <v>184</v>
@@ -16874,7 +16878,7 @@
       </c>
       <c r="AI42" s="6">
         <f t="shared" si="1"/>
-        <v>2.4868360000000012</v>
+        <v>2.4811204000000009</v>
       </c>
       <c r="AJ42" s="6">
         <f t="shared" si="2"/>
@@ -16896,7 +16900,7 @@
     <row r="43" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6">
         <f t="shared" si="0"/>
-        <v>45.81955250828134</v>
+        <v>44.601916947685687</v>
       </c>
       <c r="B43" s="18">
         <v>91</v>
@@ -16999,7 +17003,7 @@
       </c>
       <c r="AI43" s="6">
         <f t="shared" si="1"/>
-        <v>3.2018820000000008</v>
+        <v>3.0713164000000011</v>
       </c>
       <c r="AJ43" s="6">
         <f t="shared" si="2"/>
@@ -17021,7 +17025,7 @@
     <row r="44" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6">
         <f t="shared" si="0"/>
-        <v>45.449370318421906</v>
+        <v>46.405658181384098</v>
       </c>
       <c r="B44" s="18">
         <v>69</v>
@@ -17124,7 +17128,7 @@
       </c>
       <c r="AI44" s="6">
         <f t="shared" si="1"/>
-        <v>2.2903028000000005</v>
+        <v>2.3928444000000004</v>
       </c>
       <c r="AJ44" s="6">
         <f t="shared" si="2"/>
@@ -17146,7 +17150,7 @@
     <row r="45" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
         <f t="shared" si="0"/>
-        <v>45.220889611746081</v>
+        <v>44.629787221343506</v>
       </c>
       <c r="B45" s="18">
         <v>161</v>
@@ -17249,7 +17253,7 @@
       </c>
       <c r="AI45" s="6">
         <f t="shared" si="1"/>
-        <v>1.8628236000000007</v>
+        <v>1.7994404000000004</v>
       </c>
       <c r="AJ45" s="6">
         <f t="shared" si="2"/>
@@ -17271,7 +17275,7 @@
     <row r="46" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6">
         <f t="shared" si="0"/>
-        <v>44.783743770330346</v>
+        <v>45.1574083082157</v>
       </c>
       <c r="B46" s="20">
         <v>66</v>
@@ -17374,7 +17378,7 @@
       </c>
       <c r="AI46" s="6">
         <f t="shared" si="1"/>
-        <v>3.3204124000000008</v>
+        <v>3.3604800000000008</v>
       </c>
       <c r="AJ46" s="6">
         <f t="shared" si="2"/>
@@ -17396,7 +17400,7 @@
     <row r="47" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6">
         <f t="shared" si="0"/>
-        <v>44.17548688412068</v>
+        <v>44.465297084365389</v>
       </c>
       <c r="B47" s="18">
         <v>39</v>
@@ -17499,7 +17503,7 @@
       </c>
       <c r="AI47" s="6">
         <f t="shared" si="1"/>
-        <v>2.921528400000001</v>
+        <v>2.9526044000000007</v>
       </c>
       <c r="AJ47" s="6">
         <f t="shared" si="2"/>
@@ -17521,7 +17525,7 @@
     <row r="48" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6">
         <f t="shared" si="0"/>
-        <v>43.932194037422768</v>
+        <v>42.865443313736598</v>
       </c>
       <c r="B48" s="18">
         <v>57</v>
@@ -17624,7 +17628,7 @@
       </c>
       <c r="AI48" s="6">
         <f t="shared" si="1"/>
-        <v>2.4100764000000008</v>
+        <v>2.2956900000000005</v>
       </c>
       <c r="AJ48" s="6">
         <f t="shared" si="2"/>
@@ -17646,7 +17650,7 @@
     <row r="49" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6">
         <f t="shared" si="0"/>
-        <v>43.543242710913475</v>
+        <v>42.17689710227102</v>
       </c>
       <c r="B49" s="18">
         <v>73</v>
@@ -17749,7 +17753,7 @@
       </c>
       <c r="AI49" s="6">
         <f t="shared" si="1"/>
-        <v>2.0355392000000005</v>
+        <v>1.8890276000000004</v>
       </c>
       <c r="AJ49" s="6">
         <f t="shared" si="2"/>
@@ -17771,7 +17775,7 @@
     <row r="50" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6">
         <f t="shared" si="0"/>
-        <v>43.524546688949222</v>
+        <v>42.947526336208171</v>
       </c>
       <c r="B50" s="18">
         <v>59</v>
@@ -17874,7 +17878,7 @@
       </c>
       <c r="AI50" s="6">
         <f t="shared" si="1"/>
-        <v>1.5855996000000003</v>
+        <v>1.5237264000000004</v>
       </c>
       <c r="AJ50" s="6">
         <f t="shared" si="2"/>
@@ -17896,7 +17900,7 @@
     <row r="51" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6">
         <f t="shared" si="0"/>
-        <v>42.469059655614906</v>
+        <v>41.987845653406545</v>
       </c>
       <c r="B51" s="20">
         <v>58</v>
@@ -17999,7 +18003,7 @@
       </c>
       <c r="AI51" s="6">
         <f t="shared" si="1"/>
-        <v>2.3861820000000007</v>
+        <v>2.3345820000000006</v>
       </c>
       <c r="AJ51" s="6">
         <f t="shared" si="2"/>
@@ -18021,7 +18025,7 @@
     <row r="52" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="6">
         <f t="shared" si="0"/>
-        <v>42.396658509654117</v>
+        <v>41.975607448745116</v>
       </c>
       <c r="B52" s="20">
         <v>176</v>
@@ -18124,7 +18128,7 @@
       </c>
       <c r="AI52" s="6">
         <f t="shared" si="1"/>
-        <v>1.3291584000000003</v>
+        <v>1.2840096000000003</v>
       </c>
       <c r="AJ52" s="6">
         <f t="shared" si="2"/>
@@ -18146,7 +18150,7 @@
     <row r="53" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="6">
         <f t="shared" si="0"/>
-        <v>41.880277089737071</v>
+        <v>41.172825360350942</v>
       </c>
       <c r="B53" s="20">
         <v>120</v>
@@ -18249,7 +18253,7 @@
       </c>
       <c r="AI53" s="6">
         <f t="shared" si="1"/>
-        <v>2.5424896000000006</v>
+        <v>2.4666304000000006</v>
       </c>
       <c r="AJ53" s="6">
         <f t="shared" si="2"/>
@@ -18271,7 +18275,7 @@
     <row r="54" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="6">
         <f t="shared" si="0"/>
-        <v>41.747568563669446</v>
+        <v>41.347325345429574</v>
       </c>
       <c r="B54" s="18">
         <v>81</v>
@@ -18374,7 +18378,7 @@
       </c>
       <c r="AI54" s="6">
         <f t="shared" si="1"/>
-        <v>1.2991772000000004</v>
+        <v>1.2562596000000001</v>
       </c>
       <c r="AJ54" s="6">
         <f t="shared" si="2"/>
@@ -18396,7 +18400,7 @@
     <row r="55" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="6">
         <f t="shared" si="0"/>
-        <v>41.116026589871367</v>
+        <v>40.916363812707033</v>
       </c>
       <c r="B55" s="20">
         <v>84</v>
@@ -18499,7 +18503,7 @@
       </c>
       <c r="AI55" s="6">
         <f t="shared" si="1"/>
-        <v>1.2081592000000003</v>
+        <v>1.1867496000000002</v>
       </c>
       <c r="AJ55" s="6">
         <f t="shared" si="2"/>
@@ -18521,7 +18525,7 @@
     <row r="56" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6">
         <f t="shared" si="0"/>
-        <v>40.485485391984234</v>
+        <v>41.209320779492074</v>
       </c>
       <c r="B56" s="18">
         <v>67</v>
@@ -18624,7 +18628,7 @@
       </c>
       <c r="AI56" s="6">
         <f t="shared" si="1"/>
-        <v>2.177256400000001</v>
+        <v>2.2548724000000009</v>
       </c>
       <c r="AJ56" s="6">
         <f t="shared" si="2"/>
@@ -18646,7 +18650,7 @@
     <row r="57" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="6">
         <f t="shared" si="0"/>
-        <v>40.131846817272958</v>
+        <v>38.179837655555211</v>
       </c>
       <c r="B57" s="18">
         <v>71</v>
@@ -18749,7 +18753,7 @@
       </c>
       <c r="AI57" s="6">
         <f t="shared" si="1"/>
-        <v>2.0148148000000008</v>
+        <v>1.8055032000000004</v>
       </c>
       <c r="AJ57" s="6">
         <f t="shared" si="2"/>
@@ -18771,7 +18775,7 @@
     <row r="58" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="6">
         <f t="shared" si="0"/>
-        <v>40.115499418066783</v>
+        <v>40.605121609119934</v>
       </c>
       <c r="B58" s="20">
         <v>90</v>
@@ -18874,7 +18878,7 @@
       </c>
       <c r="AI58" s="6">
         <f t="shared" si="1"/>
-        <v>1.4227400000000003</v>
+        <v>1.4752416000000004</v>
       </c>
       <c r="AJ58" s="6">
         <f t="shared" si="2"/>
@@ -18896,7 +18900,7 @@
     <row r="59" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6">
         <f t="shared" si="0"/>
-        <v>38.419132173445938</v>
+        <v>37.905743979229456</v>
       </c>
       <c r="B59" s="20">
         <v>78</v>
@@ -18999,7 +19003,7 @@
       </c>
       <c r="AI59" s="6">
         <f t="shared" si="1"/>
-        <v>1.3423908000000004</v>
+        <v>1.2873408000000004</v>
       </c>
       <c r="AJ59" s="6">
         <f t="shared" si="2"/>
@@ -19021,7 +19025,7 @@
     <row r="60" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6">
         <f t="shared" si="0"/>
-        <v>38.25248440717418</v>
+        <v>35.481799665761429</v>
       </c>
       <c r="B60" s="18">
         <v>105</v>
@@ -19124,7 +19128,7 @@
       </c>
       <c r="AI60" s="6">
         <f t="shared" si="1"/>
-        <v>1.5768984000000004</v>
+        <v>1.2798012000000001</v>
       </c>
       <c r="AJ60" s="6">
         <f t="shared" si="2"/>
@@ -19146,7 +19150,7 @@
     <row r="61" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="6">
         <f t="shared" si="0"/>
-        <v>37.464895998090057</v>
+        <v>37.975464054433132</v>
       </c>
       <c r="B61" s="20">
         <v>196</v>
@@ -19249,7 +19253,7 @@
       </c>
       <c r="AI61" s="6">
         <f t="shared" si="1"/>
-        <v>1.3631048000000003</v>
+        <v>1.4178524000000003</v>
       </c>
       <c r="AJ61" s="6">
         <f t="shared" si="2"/>
@@ -19271,7 +19275,7 @@
     <row r="62" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6">
         <f t="shared" si="0"/>
-        <v>36.621701333969973</v>
+        <v>33.352366976036279</v>
       </c>
       <c r="B62" s="18">
         <v>167</v>
@@ -19374,7 +19378,7 @@
       </c>
       <c r="AI62" s="6">
         <f t="shared" si="1"/>
-        <v>1.7940040000000006</v>
+        <v>1.4434372000000004</v>
       </c>
       <c r="AJ62" s="6">
         <f t="shared" si="2"/>
@@ -19396,7 +19400,7 @@
     <row r="63" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6">
         <f t="shared" si="0"/>
-        <v>36.546765943477865</v>
+        <v>34.693909248261654</v>
       </c>
       <c r="B63" s="20">
         <v>108</v>
@@ -19499,7 +19503,7 @@
       </c>
       <c r="AI63" s="6">
         <f t="shared" si="1"/>
-        <v>1.2626472000000004</v>
+        <v>1.0639676000000002</v>
       </c>
       <c r="AJ63" s="6">
         <f t="shared" si="2"/>
@@ -19521,7 +19525,7 @@
     <row r="64" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6">
         <f t="shared" si="0"/>
-        <v>36.390019397773727</v>
+        <v>37.201614790056396</v>
       </c>
       <c r="B64" s="18">
         <v>191</v>
@@ -19624,7 +19628,7 @@
       </c>
       <c r="AI64" s="6">
         <f t="shared" si="1"/>
-        <v>2.7765300000000006</v>
+        <v>2.8635564000000002</v>
       </c>
       <c r="AJ64" s="6">
         <f t="shared" si="2"/>
@@ -19646,7 +19650,7 @@
     <row r="65" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="6">
         <f t="shared" si="0"/>
-        <v>36.163722432779245</v>
+        <v>34.704095914530427</v>
       </c>
       <c r="B65" s="20">
         <v>188</v>
@@ -19749,7 +19753,7 @@
       </c>
       <c r="AI65" s="6">
         <f t="shared" si="1"/>
-        <v>2.3597292000000007</v>
+        <v>2.2032152000000007</v>
       </c>
       <c r="AJ65" s="6">
         <f t="shared" si="2"/>
@@ -19771,7 +19775,7 @@
     <row r="66" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="6">
         <f t="shared" si="0"/>
-        <v>35.580217105852149</v>
+        <v>36.152817004386876</v>
       </c>
       <c r="B66" s="20">
         <v>80</v>
@@ -19874,7 +19878,7 @@
       </c>
       <c r="AI66" s="6">
         <f t="shared" si="1"/>
-        <v>2.1212144000000004</v>
+        <v>2.1826136000000003</v>
       </c>
       <c r="AJ66" s="6">
         <f t="shared" si="2"/>
@@ -19896,7 +19900,7 @@
     <row r="67" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="6">
         <f t="shared" si="0"/>
-        <v>35.324870930197847</v>
+        <v>35.444357486048517</v>
       </c>
       <c r="B67" s="20">
         <v>128</v>
@@ -19999,7 +20003,7 @@
       </c>
       <c r="AI67" s="6">
         <f t="shared" si="1"/>
-        <v>1.5657844000000003</v>
+        <v>1.5785968000000004</v>
       </c>
       <c r="AJ67" s="6">
         <f t="shared" si="2"/>
@@ -20021,7 +20025,7 @@
     <row r="68" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6">
         <f t="shared" si="0"/>
-        <v>34.524010116685055</v>
+        <v>34.865537765973308</v>
       </c>
       <c r="B68" s="20">
         <v>86</v>
@@ -20124,7 +20128,7 @@
       </c>
       <c r="AI68" s="6">
         <f t="shared" si="1"/>
-        <v>0.98924800000000024</v>
+        <v>1.0258696000000003</v>
       </c>
       <c r="AJ68" s="6">
         <f t="shared" si="2"/>
@@ -20146,7 +20150,7 @@
     <row r="69" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="6">
         <f t="shared" si="0"/>
-        <v>34.49691306813093</v>
+        <v>32.941741323226594</v>
       </c>
       <c r="B69" s="18">
         <v>185</v>
@@ -20249,7 +20253,7 @@
       </c>
       <c r="AI69" s="6">
         <f t="shared" si="1"/>
-        <v>2.4248988000000002</v>
+        <v>2.2581396000000007</v>
       </c>
       <c r="AJ69" s="6">
         <f t="shared" si="2"/>
@@ -20271,7 +20275,7 @@
     <row r="70" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="6">
         <f t="shared" si="0"/>
-        <v>34.368702438150933</v>
+        <v>34.905998388492634</v>
       </c>
       <c r="B70" s="20">
         <v>94</v>
@@ -20374,7 +20378,7 @@
       </c>
       <c r="AI70" s="6">
         <f t="shared" si="1"/>
-        <v>0.90036920000000031</v>
+        <v>0.95798280000000013</v>
       </c>
       <c r="AJ70" s="6">
         <f t="shared" si="2"/>
@@ -20396,7 +20400,7 @@
     <row r="71" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A71" s="6">
         <f t="shared" ref="A71:A134" si="6">(AI71*H$3+AJ71*M$3+AK71*W$3+AL71*AB$3+AM71*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>34.103655435853049</v>
+        <v>31.95039064132024</v>
       </c>
       <c r="B71" s="18">
         <v>187</v>
@@ -20499,7 +20503,7 @@
       </c>
       <c r="AI71" s="6">
         <f t="shared" ref="AI71:AI134" si="7">H$1*((-2*10^-6)*H71^3+0.00032*H71^2-0.0021*H71)+I$1*((-2*10^-6)*I71^3+0.00032*I71^2-0.0021*I71)+J$1*((-2*10^-6)*J71^3+0.00032*J71^2-0.0021*J71)+K$1*((-2*10^-6)*K71^3+0.00032*K71^2-0.0021*K71)+L$1*((-2*10^-6)*L71^3+0.00032*L71^2-0.0021*L71)</f>
-        <v>2.4124004000000006</v>
+        <v>2.1815084000000007</v>
       </c>
       <c r="AJ71" s="6">
         <f t="shared" ref="AJ71:AJ134" si="8">(M$1*M71+N$1*N71+O$1*O71)/100</f>
@@ -20521,7 +20525,7 @@
     <row r="72" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A72" s="6">
         <f t="shared" si="6"/>
-        <v>34.001690292160312</v>
+        <v>31.414101883076182</v>
       </c>
       <c r="B72" s="20">
         <v>98</v>
@@ -20624,7 +20628,7 @@
       </c>
       <c r="AI72" s="6">
         <f t="shared" si="7"/>
-        <v>1.9474044000000008</v>
+        <v>1.6699404000000002</v>
       </c>
       <c r="AJ72" s="6">
         <f t="shared" si="8"/>
@@ -20646,7 +20650,7 @@
     <row r="73" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="6">
         <f t="shared" si="6"/>
-        <v>33.906723865230234</v>
+        <v>33.69168835238294</v>
       </c>
       <c r="B73" s="18">
         <v>97</v>
@@ -20749,7 +20753,7 @@
       </c>
       <c r="AI73" s="6">
         <f t="shared" si="7"/>
-        <v>0.87482960000000021</v>
+        <v>0.85177160000000007</v>
       </c>
       <c r="AJ73" s="6">
         <f t="shared" si="8"/>
@@ -20771,7 +20775,7 @@
     <row r="74" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="6">
         <f t="shared" si="6"/>
-        <v>33.838489808708097</v>
+        <v>33.26619206780267</v>
       </c>
       <c r="B74" s="20">
         <v>170</v>
@@ -20874,7 +20878,7 @@
       </c>
       <c r="AI74" s="6">
         <f t="shared" si="7"/>
-        <v>0.5704184000000001</v>
+        <v>0.50905160000000005</v>
       </c>
       <c r="AJ74" s="6">
         <f t="shared" si="8"/>
@@ -20896,7 +20900,7 @@
     <row r="75" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="6">
         <f t="shared" si="6"/>
-        <v>33.737730311259654</v>
+        <v>33.841638962666742</v>
       </c>
       <c r="B75" s="20">
         <v>130</v>
@@ -20999,7 +21003,7 @@
       </c>
       <c r="AI75" s="6">
         <f t="shared" si="7"/>
-        <v>1.5156216000000005</v>
+        <v>1.5267636000000007</v>
       </c>
       <c r="AJ75" s="6">
         <f t="shared" si="8"/>
@@ -21021,7 +21025,7 @@
     <row r="76" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="6">
         <f t="shared" si="6"/>
-        <v>33.611411561073133</v>
+        <v>34.253149601599567</v>
       </c>
       <c r="B76" s="18">
         <v>197</v>
@@ -21124,7 +21128,7 @@
       </c>
       <c r="AI76" s="6">
         <f t="shared" si="7"/>
-        <v>1.4626816000000002</v>
+        <v>1.5314944000000006</v>
       </c>
       <c r="AJ76" s="6">
         <f t="shared" si="8"/>
@@ -21146,7 +21150,7 @@
     <row r="77" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="6">
         <f t="shared" si="6"/>
-        <v>33.484845713091993</v>
+        <v>31.870965859918229</v>
       </c>
       <c r="B77" s="18">
         <v>201</v>
@@ -21249,7 +21253,7 @@
       </c>
       <c r="AI77" s="6">
         <f t="shared" si="7"/>
-        <v>1.8024392000000002</v>
+        <v>1.6293848000000004</v>
       </c>
       <c r="AJ77" s="6">
         <f t="shared" si="8"/>
@@ -21271,7 +21275,7 @@
     <row r="78" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="6">
         <f t="shared" si="6"/>
-        <v>33.220867528126767</v>
+        <v>29.978660210689664</v>
       </c>
       <c r="B78" s="20">
         <v>200</v>
@@ -21374,7 +21378,7 @@
       </c>
       <c r="AI78" s="6">
         <f t="shared" si="7"/>
-        <v>1.6526304000000005</v>
+        <v>1.3049724000000005</v>
       </c>
       <c r="AJ78" s="6">
         <f t="shared" si="8"/>
@@ -21396,7 +21400,7 @@
     <row r="79" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A79" s="6">
         <f t="shared" si="6"/>
-        <v>32.925160852308316</v>
+        <v>32.997932346533759</v>
       </c>
       <c r="B79" s="18">
         <v>103</v>
@@ -21499,7 +21503,7 @@
       </c>
       <c r="AI79" s="6">
         <f t="shared" si="7"/>
-        <v>1.2945756000000004</v>
+        <v>1.3023788000000003</v>
       </c>
       <c r="AJ79" s="6">
         <f t="shared" si="8"/>
@@ -21521,7 +21525,7 @@
     <row r="80" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="6">
         <f t="shared" si="6"/>
-        <v>32.81943985198005</v>
+        <v>32.095201587633163</v>
       </c>
       <c r="B80" s="18">
         <v>189</v>
@@ -21624,7 +21628,7 @@
       </c>
       <c r="AI80" s="6">
         <f t="shared" si="7"/>
-        <v>1.8385267999999999</v>
+        <v>1.7608676000000001</v>
       </c>
       <c r="AJ80" s="6">
         <f t="shared" si="8"/>
@@ -21646,7 +21650,7 @@
     <row r="81" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="6">
         <f t="shared" si="6"/>
-        <v>32.628401921871735</v>
+        <v>34.144793040675637</v>
       </c>
       <c r="B81" s="18">
         <v>145</v>
@@ -21749,7 +21753,7 @@
       </c>
       <c r="AI81" s="6">
         <f t="shared" si="7"/>
-        <v>0.9843120000000003</v>
+        <v>1.1469128000000004</v>
       </c>
       <c r="AJ81" s="6">
         <f t="shared" si="8"/>
@@ -21771,7 +21775,7 @@
     <row r="82" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="6">
         <f t="shared" si="6"/>
-        <v>32.41240786057476</v>
+        <v>31.235067444567125</v>
       </c>
       <c r="B82" s="20">
         <v>124</v>
@@ -21874,7 +21878,7 @@
       </c>
       <c r="AI82" s="6">
         <f t="shared" si="7"/>
-        <v>0.81462760000000012</v>
+        <v>0.68838280000000007</v>
       </c>
       <c r="AJ82" s="6">
         <f t="shared" si="8"/>
@@ -21896,7 +21900,7 @@
     <row r="83" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A83" s="6">
         <f t="shared" si="6"/>
-        <v>32.362329971052553</v>
+        <v>32.355324390462258</v>
       </c>
       <c r="B83" s="18">
         <v>175</v>
@@ -21999,7 +22003,7 @@
       </c>
       <c r="AI83" s="6">
         <f t="shared" si="7"/>
-        <v>0.41216240000000015</v>
+        <v>0.41141120000000009</v>
       </c>
       <c r="AJ83" s="6">
         <f t="shared" si="8"/>
@@ -22021,7 +22025,7 @@
     <row r="84" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="6">
         <f t="shared" si="6"/>
-        <v>32.103083649168873</v>
+        <v>30.912291623146018</v>
       </c>
       <c r="B84" s="18">
         <v>129</v>
@@ -22124,7 +22128,7 @@
       </c>
       <c r="AI84" s="6">
         <f t="shared" si="7"/>
-        <v>0.77334000000000014</v>
+        <v>0.64565280000000014</v>
       </c>
       <c r="AJ84" s="6">
         <f t="shared" si="8"/>
@@ -22146,7 +22150,7 @@
     <row r="85" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A85" s="6">
         <f t="shared" si="6"/>
-        <v>31.749693664388662</v>
+        <v>32.560699662777168</v>
       </c>
       <c r="B85" s="20">
         <v>104</v>
@@ -22249,7 +22253,7 @@
       </c>
       <c r="AI85" s="6">
         <f t="shared" si="7"/>
-        <v>0.73227680000000017</v>
+        <v>0.8192400000000003</v>
       </c>
       <c r="AJ85" s="6">
         <f t="shared" si="8"/>
@@ -22271,7 +22275,7 @@
     <row r="86" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A86" s="6">
         <f t="shared" si="6"/>
-        <v>31.312862365334681</v>
+        <v>30.821583902832074</v>
       </c>
       <c r="B86" s="20">
         <v>140</v>
@@ -22374,7 +22378,7 @@
       </c>
       <c r="AI86" s="6">
         <f t="shared" si="7"/>
-        <v>0.95011560000000017</v>
+        <v>0.89743640000000013</v>
       </c>
       <c r="AJ86" s="6">
         <f t="shared" si="8"/>
@@ -22396,7 +22400,7 @@
     <row r="87" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A87" s="6">
         <f t="shared" si="6"/>
-        <v>30.931057178668411</v>
+        <v>30.575216210570293</v>
       </c>
       <c r="B87" s="20">
         <v>180</v>
@@ -22499,7 +22503,7 @@
       </c>
       <c r="AI87" s="6">
         <f t="shared" si="7"/>
-        <v>0.9940956000000003</v>
+        <v>0.95593920000000021</v>
       </c>
       <c r="AJ87" s="6">
         <f t="shared" si="8"/>
@@ -22521,7 +22525,7 @@
     <row r="88" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A88" s="6">
         <f t="shared" si="6"/>
-        <v>30.686061804291377</v>
+        <v>30.201106269957322</v>
       </c>
       <c r="B88" s="18">
         <v>139</v>
@@ -22624,7 +22628,7 @@
       </c>
       <c r="AI88" s="6">
         <f t="shared" si="7"/>
-        <v>0.52157960000000014</v>
+        <v>0.46957840000000017</v>
       </c>
       <c r="AJ88" s="6">
         <f t="shared" si="8"/>
@@ -22646,7 +22650,7 @@
     <row r="89" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A89" s="6">
         <f t="shared" si="6"/>
-        <v>30.684697842370696</v>
+        <v>29.295112208660353</v>
       </c>
       <c r="B89" s="20">
         <v>186</v>
@@ -22749,7 +22753,7 @@
       </c>
       <c r="AI89" s="6">
         <f t="shared" si="7"/>
-        <v>1.6627680000000002</v>
+        <v>1.5137644000000001</v>
       </c>
       <c r="AJ89" s="6">
         <f t="shared" si="8"/>
@@ -22771,7 +22775,7 @@
     <row r="90" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A90" s="6">
         <f t="shared" si="6"/>
-        <v>29.976402906681777</v>
+        <v>29.502574979856156</v>
       </c>
       <c r="B90" s="18">
         <v>109</v>
@@ -22874,7 +22878,7 @@
       </c>
       <c r="AI90" s="6">
         <f t="shared" si="7"/>
-        <v>0.63089120000000021</v>
+        <v>0.58008320000000013</v>
       </c>
       <c r="AJ90" s="6">
         <f t="shared" si="8"/>
@@ -22896,7 +22900,7 @@
     <row r="91" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="6">
         <f t="shared" si="6"/>
-        <v>29.68968978483392</v>
+        <v>29.236296666567185</v>
       </c>
       <c r="B91" s="20">
         <v>198</v>
@@ -22999,7 +23003,7 @@
       </c>
       <c r="AI91" s="6">
         <f t="shared" si="7"/>
-        <v>1.2886768000000004</v>
+        <v>1.2400600000000002</v>
       </c>
       <c r="AJ91" s="6">
         <f t="shared" si="8"/>
@@ -23021,7 +23025,7 @@
     <row r="92" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="6">
         <f t="shared" si="6"/>
-        <v>29.072248052761939</v>
+        <v>29.015543137664501</v>
       </c>
       <c r="B92" s="20">
         <v>150</v>
@@ -23124,7 +23128,7 @@
       </c>
       <c r="AI92" s="6">
         <f t="shared" si="7"/>
-        <v>1.0831020000000002</v>
+        <v>1.0770216000000004</v>
       </c>
       <c r="AJ92" s="6">
         <f t="shared" si="8"/>
@@ -23146,7 +23150,7 @@
     <row r="93" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A93" s="6">
         <f t="shared" si="6"/>
-        <v>28.973263750037297</v>
+        <v>27.682017368468166</v>
       </c>
       <c r="B93" s="20">
         <v>192</v>
@@ -23249,7 +23253,7 @@
       </c>
       <c r="AI93" s="6">
         <f t="shared" si="7"/>
-        <v>1.8737916000000001</v>
+        <v>1.7353328000000001</v>
       </c>
       <c r="AJ93" s="6">
         <f t="shared" si="8"/>
@@ -23271,7 +23275,7 @@
     <row r="94" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A94" s="6">
         <f t="shared" si="6"/>
-        <v>28.288871049568762</v>
+        <v>26.778284341520184</v>
       </c>
       <c r="B94" s="20">
         <v>142</v>
@@ -23374,7 +23378,7 @@
       </c>
       <c r="AI94" s="6">
         <f t="shared" si="7"/>
-        <v>0.78958160000000033</v>
+        <v>0.62760320000000025</v>
       </c>
       <c r="AJ94" s="6">
         <f t="shared" si="8"/>
@@ -23396,7 +23400,7 @@
     <row r="95" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A95" s="6">
         <f t="shared" si="6"/>
-        <v>27.064454027276248</v>
+        <v>27.409372556626575</v>
       </c>
       <c r="B95" s="20">
         <v>144</v>
@@ -23499,7 +23503,7 @@
       </c>
       <c r="AI95" s="6">
         <f t="shared" si="7"/>
-        <v>0.49478960000000016</v>
+        <v>0.53177480000000021</v>
       </c>
       <c r="AJ95" s="6">
         <f t="shared" si="8"/>
@@ -23521,7 +23525,7 @@
     <row r="96" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A96" s="6">
         <f t="shared" si="6"/>
-        <v>25.859922558118708</v>
+        <v>25.468169596227874</v>
       </c>
       <c r="B96" s="18">
         <v>147</v>
@@ -23624,7 +23628,7 @@
       </c>
       <c r="AI96" s="6">
         <f t="shared" si="7"/>
-        <v>0.33374440000000005</v>
+        <v>0.29173720000000003</v>
       </c>
       <c r="AJ96" s="6">
         <f t="shared" si="8"/>
@@ -23646,7 +23650,7 @@
     <row r="97" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A97" s="6">
         <f t="shared" si="6"/>
-        <v>25.787922349219603</v>
+        <v>26.116848906263982</v>
       </c>
       <c r="B97" s="20">
         <v>138</v>
@@ -23749,7 +23753,7 @@
       </c>
       <c r="AI97" s="6">
         <f t="shared" si="7"/>
-        <v>1.4132488000000003</v>
+        <v>1.4485192000000005</v>
       </c>
       <c r="AJ97" s="6">
         <f t="shared" si="8"/>
@@ -23771,7 +23775,7 @@
     <row r="98" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A98" s="6">
         <f t="shared" si="6"/>
-        <v>25.651122981885457</v>
+        <v>23.411881285624755</v>
       </c>
       <c r="B98" s="18">
         <v>195</v>
@@ -23874,7 +23878,7 @@
       </c>
       <c r="AI98" s="6">
         <f t="shared" si="7"/>
-        <v>1.9647848000000008</v>
+        <v>1.7246736000000005</v>
       </c>
       <c r="AJ98" s="6">
         <f t="shared" si="8"/>
@@ -23896,7 +23900,7 @@
     <row r="99" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="6">
         <f t="shared" si="6"/>
-        <v>25.563287027365771</v>
+        <v>24.824992837745082</v>
       </c>
       <c r="B99" s="20">
         <v>148</v>
@@ -23999,7 +24003,7 @@
       </c>
       <c r="AI99" s="6">
         <f t="shared" si="7"/>
-        <v>0.67017080000000018</v>
+        <v>0.5910044000000001</v>
       </c>
       <c r="AJ99" s="6">
         <f t="shared" si="8"/>
@@ -24021,7 +24025,7 @@
     <row r="100" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
         <f t="shared" si="6"/>
-        <v>25.387204930018793</v>
+        <v>24.298918947148525</v>
       </c>
       <c r="B100" s="18">
         <v>141</v>
@@ -24124,7 +24128,7 @@
       </c>
       <c r="AI100" s="6">
         <f t="shared" si="7"/>
-        <v>0.92597880000000021</v>
+        <v>0.8092832000000002</v>
       </c>
       <c r="AJ100" s="6">
         <f t="shared" si="8"/>
@@ -24146,7 +24150,7 @@
     <row r="101" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="6">
         <f t="shared" si="6"/>
-        <v>25.320263660509113</v>
+        <v>24.659780655943173</v>
       </c>
       <c r="B101" s="18">
         <v>171</v>
@@ -24249,7 +24253,7 @@
       </c>
       <c r="AI101" s="6">
         <f t="shared" si="7"/>
-        <v>0.84891160000000032</v>
+        <v>0.77808880000000025</v>
       </c>
       <c r="AJ101" s="6">
         <f t="shared" si="8"/>
@@ -24271,7 +24275,7 @@
     <row r="102" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="6">
         <f t="shared" si="6"/>
-        <v>24.093379838252403</v>
+        <v>23.803424154704704</v>
       </c>
       <c r="B102" s="18">
         <v>169</v>
@@ -24374,7 +24378,7 @@
       </c>
       <c r="AI102" s="6">
         <f t="shared" si="7"/>
-        <v>0.61924880000000015</v>
+        <v>0.58815720000000016</v>
       </c>
       <c r="AJ102" s="6">
         <f t="shared" si="8"/>
@@ -24396,7 +24400,7 @@
     <row r="103" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="6">
         <f t="shared" si="6"/>
-        <v>24.020866483631252</v>
+        <v>23.28365036258915</v>
       </c>
       <c r="B103" s="18">
         <v>143</v>
@@ -24499,7 +24503,7 @@
       </c>
       <c r="AI103" s="6">
         <f t="shared" si="7"/>
-        <v>0.79728680000000007</v>
+        <v>0.7182360000000001</v>
       </c>
       <c r="AJ103" s="6">
         <f t="shared" si="8"/>
@@ -24521,7 +24525,7 @@
     <row r="104" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="6">
         <f t="shared" si="6"/>
-        <v>23.760556417678828</v>
+        <v>25.135343788235996</v>
       </c>
       <c r="B104" s="20">
         <v>114</v>
@@ -24624,7 +24628,7 @@
       </c>
       <c r="AI104" s="6">
         <f t="shared" si="7"/>
-        <v>0.77083160000000028</v>
+        <v>0.91824840000000041</v>
       </c>
       <c r="AJ104" s="6">
         <f t="shared" si="8"/>
@@ -24646,7 +24650,7 @@
     <row r="105" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A105" s="6">
         <f t="shared" si="6"/>
-        <v>23.696345310215165</v>
+        <v>23.927712256408725</v>
       </c>
       <c r="B105" s="20">
         <v>156</v>
@@ -24749,7 +24753,7 @@
       </c>
       <c r="AI105" s="6">
         <f t="shared" si="7"/>
-        <v>0.57145800000000013</v>
+        <v>0.59626720000000011</v>
       </c>
       <c r="AJ105" s="6">
         <f t="shared" si="8"/>
@@ -24771,7 +24775,7 @@
     <row r="106" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A106" s="6">
         <f t="shared" si="6"/>
-        <v>23.655091766391113</v>
+        <v>23.708954161568531</v>
       </c>
       <c r="B106" s="18">
         <v>7</v>
@@ -24874,7 +24878,7 @@
       </c>
       <c r="AI106" s="6">
         <f t="shared" si="7"/>
-        <v>0.40974600000000011</v>
+        <v>0.41552160000000005</v>
       </c>
       <c r="AJ106" s="6">
         <f t="shared" si="8"/>
@@ -24896,7 +24900,7 @@
     <row r="107" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A107" s="6">
         <f t="shared" si="6"/>
-        <v>23.140520755617889</v>
+        <v>23.142632128681846</v>
       </c>
       <c r="B107" s="18">
         <v>155</v>
@@ -24999,7 +25003,7 @@
       </c>
       <c r="AI107" s="6">
         <f t="shared" si="7"/>
-        <v>0.15113480000000004</v>
+        <v>0.15136120000000006</v>
       </c>
       <c r="AJ107" s="6">
         <f t="shared" si="8"/>
@@ -25021,7 +25025,7 @@
     <row r="108" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="6">
         <f t="shared" si="6"/>
-        <v>22.727945029693508</v>
+        <v>23.568480408248522</v>
       </c>
       <c r="B108" s="20">
         <v>102</v>
@@ -25124,7 +25128,7 @@
       </c>
       <c r="AI108" s="6">
         <f t="shared" si="7"/>
-        <v>0.33194520000000005</v>
+        <v>0.42207480000000003</v>
       </c>
       <c r="AJ108" s="6">
         <f t="shared" si="8"/>
@@ -25146,7 +25150,7 @@
     <row r="109" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A109" s="6">
         <f t="shared" si="6"/>
-        <v>22.283925363335221</v>
+        <v>22.445803515473457</v>
       </c>
       <c r="B109" s="18">
         <v>83</v>
@@ -25249,7 +25253,7 @@
       </c>
       <c r="AI109" s="6">
         <f t="shared" si="7"/>
-        <v>0.16579920000000004</v>
+        <v>0.18315720000000008</v>
       </c>
       <c r="AJ109" s="6">
         <f t="shared" si="8"/>
@@ -25271,7 +25275,7 @@
     <row r="110" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A110" s="6">
         <f t="shared" si="6"/>
-        <v>21.920072667044671</v>
+        <v>21.723200185024918</v>
       </c>
       <c r="B110" s="20">
         <v>24</v>
@@ -25374,7 +25378,7 @@
       </c>
       <c r="AI110" s="6">
         <f t="shared" si="7"/>
-        <v>0.79414320000000016</v>
+        <v>0.77303280000000008</v>
       </c>
       <c r="AJ110" s="6">
         <f t="shared" si="8"/>
@@ -25396,7 +25400,7 @@
     <row r="111" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A111" s="6">
         <f t="shared" si="6"/>
-        <v>21.837197469336591</v>
+        <v>21.547383538750783</v>
       </c>
       <c r="B111" s="20">
         <v>194</v>
@@ -25499,7 +25503,7 @@
       </c>
       <c r="AI111" s="6">
         <f t="shared" si="7"/>
-        <v>1.1343352000000002</v>
+        <v>1.1032588000000003</v>
       </c>
       <c r="AJ111" s="6">
         <f t="shared" si="8"/>
@@ -25521,7 +25525,7 @@
     <row r="112" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A112" s="6">
         <f t="shared" si="6"/>
-        <v>21.653593810618037</v>
+        <v>22.140750246202515</v>
       </c>
       <c r="B112" s="18">
         <v>9</v>
@@ -25624,7 +25628,7 @@
       </c>
       <c r="AI112" s="6">
         <f t="shared" si="7"/>
-        <v>0.42928320000000009</v>
+        <v>0.48152040000000007</v>
       </c>
       <c r="AJ112" s="6">
         <f t="shared" si="8"/>
@@ -25646,7 +25650,7 @@
     <row r="113" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A113" s="6">
         <f t="shared" si="6"/>
-        <v>21.263497567817595</v>
+        <v>21.817464412545881</v>
       </c>
       <c r="B113" s="18">
         <v>75</v>
@@ -25749,7 +25753,7 @@
       </c>
       <c r="AI113" s="6">
         <f t="shared" si="7"/>
-        <v>0.33230440000000006</v>
+        <v>0.39170560000000004</v>
       </c>
       <c r="AJ113" s="6">
         <f t="shared" si="8"/>
@@ -25771,7 +25775,7 @@
     <row r="114" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A114" s="6">
         <f t="shared" si="6"/>
-        <v>20.955300367065558</v>
+        <v>21.48115536124623</v>
       </c>
       <c r="B114" s="18">
         <v>33</v>
@@ -25874,7 +25878,7 @@
       </c>
       <c r="AI114" s="6">
         <f t="shared" si="7"/>
-        <v>0.87521360000000026</v>
+        <v>0.93160040000000033</v>
       </c>
       <c r="AJ114" s="6">
         <f t="shared" si="8"/>
@@ -25896,7 +25900,7 @@
     <row r="115" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A115" s="6">
         <f t="shared" si="6"/>
-        <v>20.71254021307708</v>
+        <v>21.462887134799605</v>
       </c>
       <c r="B115" s="18">
         <v>29</v>
@@ -25999,7 +26003,7 @@
       </c>
       <c r="AI115" s="6">
         <f t="shared" si="7"/>
-        <v>0.41397760000000017</v>
+        <v>0.49443640000000016</v>
       </c>
       <c r="AJ115" s="6">
         <f t="shared" si="8"/>
@@ -26021,7 +26025,7 @@
     <row r="116" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="6">
         <f t="shared" si="6"/>
-        <v>20.541906055089676</v>
+        <v>20.926567638544867</v>
       </c>
       <c r="B116" s="20">
         <v>54</v>
@@ -26124,7 +26128,7 @@
       </c>
       <c r="AI116" s="6">
         <f t="shared" si="7"/>
-        <v>0.5378248000000001</v>
+        <v>0.57907160000000013</v>
       </c>
       <c r="AJ116" s="6">
         <f t="shared" si="8"/>
@@ -26146,7 +26150,7 @@
     <row r="117" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="6">
         <f t="shared" si="6"/>
-        <v>20.438523381778019</v>
+        <v>19.612148378047685</v>
       </c>
       <c r="B117" s="18">
         <v>199</v>
@@ -26249,7 +26253,7 @@
       </c>
       <c r="AI117" s="6">
         <f t="shared" si="7"/>
-        <v>0.69950600000000018</v>
+        <v>0.61089480000000018</v>
       </c>
       <c r="AJ117" s="6">
         <f t="shared" si="8"/>
@@ -26271,7 +26275,7 @@
     <row r="118" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="6">
         <f t="shared" si="6"/>
-        <v>20.370367960846337</v>
+        <v>20.429120833208991</v>
       </c>
       <c r="B118" s="20">
         <v>46</v>
@@ -26374,7 +26378,7 @@
       </c>
       <c r="AI118" s="6">
         <f t="shared" si="7"/>
-        <v>0.31937600000000005</v>
+        <v>0.32567600000000008</v>
       </c>
       <c r="AJ118" s="6">
         <f t="shared" si="8"/>
@@ -26396,7 +26400,7 @@
     <row r="119" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A119" s="6">
         <f t="shared" si="6"/>
-        <v>20.227004983735707</v>
+        <v>20.248017995165473</v>
       </c>
       <c r="B119" s="18">
         <v>25</v>
@@ -26499,7 +26503,7 @@
       </c>
       <c r="AI119" s="6">
         <f t="shared" si="7"/>
-        <v>0.58506720000000023</v>
+        <v>0.58732040000000019</v>
       </c>
       <c r="AJ119" s="6">
         <f t="shared" si="8"/>
@@ -26521,7 +26525,7 @@
     <row r="120" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A120" s="6">
         <f t="shared" si="6"/>
-        <v>19.98019173953266</v>
+        <v>19.634224984332558</v>
       </c>
       <c r="B120" s="20">
         <v>160</v>
@@ -26624,7 +26628,7 @@
       </c>
       <c r="AI120" s="6">
         <f t="shared" si="7"/>
-        <v>0.56781720000000013</v>
+        <v>0.53071960000000007</v>
       </c>
       <c r="AJ120" s="6">
         <f t="shared" si="8"/>
@@ -26646,7 +26650,7 @@
     <row r="121" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A121" s="6">
         <f t="shared" si="6"/>
-        <v>19.893617237160157</v>
+        <v>20.090288280760387</v>
       </c>
       <c r="B121" s="20">
         <v>62</v>
@@ -26749,7 +26753,7 @@
       </c>
       <c r="AI121" s="6">
         <f t="shared" si="7"/>
-        <v>0.59076760000000017</v>
+        <v>0.61185640000000008</v>
       </c>
       <c r="AJ121" s="6">
         <f t="shared" si="8"/>
@@ -26771,7 +26775,7 @@
     <row r="122" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A122" s="6">
         <f t="shared" si="6"/>
-        <v>19.826884419111277</v>
+        <v>18.576597182846395</v>
       </c>
       <c r="B122" s="18">
         <v>157</v>
@@ -26874,7 +26878,7 @@
       </c>
       <c r="AI122" s="6">
         <f t="shared" si="7"/>
-        <v>1.0696576000000002</v>
+        <v>0.93559080000000017</v>
       </c>
       <c r="AJ122" s="6">
         <f t="shared" si="8"/>
@@ -26896,7 +26900,7 @@
     <row r="123" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A123" s="6">
         <f t="shared" si="6"/>
-        <v>19.557985168163768</v>
+        <v>19.664758721537488</v>
       </c>
       <c r="B123" s="20">
         <v>92</v>
@@ -26999,7 +27003,7 @@
       </c>
       <c r="AI123" s="6">
         <f t="shared" si="7"/>
-        <v>0.20326360000000004</v>
+        <v>0.21471280000000004</v>
       </c>
       <c r="AJ123" s="6">
         <f t="shared" si="8"/>
@@ -27021,7 +27025,7 @@
     <row r="124" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A124" s="6">
         <f t="shared" si="6"/>
-        <v>19.402617953385654</v>
+        <v>19.731164015637589</v>
       </c>
       <c r="B124" s="18">
         <v>11</v>
@@ -27124,7 +27128,7 @@
       </c>
       <c r="AI124" s="6">
         <f t="shared" si="7"/>
-        <v>0.46129320000000013</v>
+        <v>0.49652280000000015</v>
       </c>
       <c r="AJ124" s="6">
         <f t="shared" si="8"/>
@@ -27146,7 +27150,7 @@
     <row r="125" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A125" s="6">
         <f t="shared" si="6"/>
-        <v>19.371807275657286</v>
+        <v>19.0267917574383</v>
       </c>
       <c r="B125" s="18">
         <v>193</v>
@@ -27249,7 +27253,7 @@
       </c>
       <c r="AI125" s="6">
         <f t="shared" si="7"/>
-        <v>0.53212040000000016</v>
+        <v>0.49512480000000014</v>
       </c>
       <c r="AJ125" s="6">
         <f t="shared" si="8"/>
@@ -27271,7 +27275,7 @@
     <row r="126" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="6">
         <f t="shared" si="6"/>
-        <v>19.262521859798856</v>
+        <v>19.010634307201048</v>
       </c>
       <c r="B126" s="18">
         <v>61</v>
@@ -27374,7 +27378,7 @@
       </c>
       <c r="AI126" s="6">
         <f t="shared" si="7"/>
-        <v>0.46020360000000005</v>
+        <v>0.43319400000000008</v>
       </c>
       <c r="AJ126" s="6">
         <f t="shared" si="8"/>
@@ -27396,7 +27400,7 @@
     <row r="127" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A127" s="6">
         <f t="shared" si="6"/>
-        <v>19.261994837207908</v>
+        <v>17.015352144200062</v>
       </c>
       <c r="B127" s="18">
         <v>179</v>
@@ -27499,7 +27503,7 @@
       </c>
       <c r="AI127" s="6">
         <f t="shared" si="7"/>
-        <v>0.95734720000000029</v>
+        <v>0.71644240000000026</v>
       </c>
       <c r="AJ127" s="6">
         <f t="shared" si="8"/>
@@ -27521,7 +27525,7 @@
     <row r="128" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="6">
         <f t="shared" si="6"/>
-        <v>19.130191291891727</v>
+        <v>18.900312751798019</v>
       </c>
       <c r="B128" s="20">
         <v>52</v>
@@ -27624,7 +27628,7 @@
       </c>
       <c r="AI128" s="6">
         <f t="shared" si="7"/>
-        <v>0.38925840000000012</v>
+        <v>0.36460880000000007</v>
       </c>
       <c r="AJ128" s="6">
         <f t="shared" si="8"/>
@@ -27646,7 +27650,7 @@
     <row r="129" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A129" s="6">
         <f t="shared" si="6"/>
-        <v>19.011471246530778</v>
+        <v>18.949831090154881</v>
       </c>
       <c r="B129" s="18">
         <v>125</v>
@@ -27749,7 +27753,7 @@
       </c>
       <c r="AI129" s="6">
         <f t="shared" si="7"/>
-        <v>0.71732640000000014</v>
+        <v>0.71071680000000015</v>
       </c>
       <c r="AJ129" s="6">
         <f t="shared" si="8"/>
@@ -27771,7 +27775,7 @@
     <row r="130" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A130" s="6">
         <f t="shared" si="6"/>
-        <v>19.002621534513114</v>
+        <v>18.547702706735507</v>
       </c>
       <c r="B130" s="18">
         <v>17</v>
@@ -27874,7 +27878,7 @@
       </c>
       <c r="AI130" s="6">
         <f t="shared" si="7"/>
-        <v>0.52463320000000013</v>
+        <v>0.47585280000000013</v>
       </c>
       <c r="AJ130" s="6">
         <f t="shared" si="8"/>
@@ -27896,7 +27900,7 @@
     <row r="131" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A131" s="6">
         <f t="shared" si="6"/>
-        <v>18.822738518010084</v>
+        <v>20.359881524366585</v>
       </c>
       <c r="B131" s="20">
         <v>178</v>
@@ -27999,7 +28003,7 @@
       </c>
       <c r="AI131" s="6">
         <f t="shared" si="7"/>
-        <v>0.92539320000000025</v>
+        <v>1.0902192000000004</v>
       </c>
       <c r="AJ131" s="6">
         <f t="shared" si="8"/>
@@ -28021,7 +28025,7 @@
     <row r="132" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A132" s="6">
         <f t="shared" si="6"/>
-        <v>18.807586320093101</v>
+        <v>17.940330508221667</v>
       </c>
       <c r="B132" s="18">
         <v>93</v>
@@ -28124,7 +28128,7 @@
       </c>
       <c r="AI132" s="6">
         <f t="shared" si="7"/>
-        <v>0.88954880000000025</v>
+        <v>0.79655400000000021</v>
       </c>
       <c r="AJ132" s="6">
         <f t="shared" si="8"/>
@@ -28146,7 +28150,7 @@
     <row r="133" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A133" s="6">
         <f t="shared" si="6"/>
-        <v>18.664792443821057</v>
+        <v>19.207620490017607</v>
       </c>
       <c r="B133" s="18">
         <v>95</v>
@@ -28249,7 +28253,7 @@
       </c>
       <c r="AI133" s="6">
         <f t="shared" si="7"/>
-        <v>0.20912800000000006</v>
+        <v>0.26733480000000009</v>
       </c>
       <c r="AJ133" s="6">
         <f t="shared" si="8"/>
@@ -28271,7 +28275,7 @@
     <row r="134" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A134" s="6">
         <f t="shared" si="6"/>
-        <v>18.645210540451814</v>
+        <v>18.53377779104121</v>
       </c>
       <c r="B134" s="18">
         <v>151</v>
@@ -28374,7 +28378,7 @@
       </c>
       <c r="AI134" s="6">
         <f t="shared" si="7"/>
-        <v>0.25882840000000007</v>
+        <v>0.24687960000000003</v>
       </c>
       <c r="AJ134" s="6">
         <f t="shared" si="8"/>
@@ -28396,7 +28400,7 @@
     <row r="135" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A135" s="6">
         <f t="shared" ref="A135:A198" si="12">(AI135*H$3+AJ135*M$3+AK135*W$3+AL135*AB$3+AM135*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>18.169363753021571</v>
+        <v>18.629672923692141</v>
       </c>
       <c r="B135" s="18">
         <v>133</v>
@@ -28499,7 +28503,7 @@
       </c>
       <c r="AI135" s="6">
         <f t="shared" ref="AI135:AI198" si="13">H$1*((-2*10^-6)*H135^3+0.00032*H135^2-0.0021*H135)+I$1*((-2*10^-6)*I135^3+0.00032*I135^2-0.0021*I135)+J$1*((-2*10^-6)*J135^3+0.00032*J135^2-0.0021*J135)+K$1*((-2*10^-6)*K135^3+0.00032*K135^2-0.0021*K135)+L$1*((-2*10^-6)*L135^3+0.00032*L135^2-0.0021*L135)</f>
-        <v>0.24287560000000005</v>
+        <v>0.2922340000000001</v>
       </c>
       <c r="AJ135" s="6">
         <f t="shared" ref="AJ135:AJ198" si="14">(M$1*M135+N$1*N135+O$1*O135)/100</f>
@@ -28521,7 +28525,7 @@
     <row r="136" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A136" s="6">
         <f t="shared" si="12"/>
-        <v>18.045394222447694</v>
+        <v>17.889171267420689</v>
       </c>
       <c r="B136" s="20">
         <v>96</v>
@@ -28624,7 +28628,7 @@
       </c>
       <c r="AI136" s="6">
         <f t="shared" si="13"/>
-        <v>0.48991040000000013</v>
+        <v>0.4731588000000001</v>
       </c>
       <c r="AJ136" s="6">
         <f t="shared" si="14"/>
@@ -28646,7 +28650,7 @@
     <row r="137" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A137" s="6">
         <f t="shared" si="12"/>
-        <v>17.839010116685067</v>
+        <v>17.854923751827865</v>
       </c>
       <c r="B137" s="18">
         <v>63</v>
@@ -28749,7 +28753,7 @@
       </c>
       <c r="AI137" s="6">
         <f t="shared" si="13"/>
-        <v>0.65684400000000021</v>
+        <v>0.6585504000000002</v>
       </c>
       <c r="AJ137" s="6">
         <f t="shared" si="14"/>
@@ -28771,7 +28775,7 @@
     <row r="138" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="6">
         <f t="shared" si="12"/>
-        <v>17.735876630159058</v>
+        <v>17.163295383329846</v>
       </c>
       <c r="B138" s="18">
         <v>101</v>
@@ -28874,7 +28878,7 @@
       </c>
       <c r="AI138" s="6">
         <f t="shared" si="13"/>
-        <v>0.47925000000000012</v>
+        <v>0.41785280000000002</v>
       </c>
       <c r="AJ138" s="6">
         <f t="shared" si="14"/>
@@ -28896,7 +28900,7 @@
     <row r="139" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A139" s="6">
         <f t="shared" si="12"/>
-        <v>17.585528663941027</v>
+        <v>17.651764600555072</v>
       </c>
       <c r="B139" s="20">
         <v>22</v>
@@ -28999,7 +29003,7 @@
       </c>
       <c r="AI139" s="6">
         <f t="shared" si="13"/>
-        <v>0.14113440000000005</v>
+        <v>0.14823680000000006</v>
       </c>
       <c r="AJ139" s="6">
         <f t="shared" si="14"/>
@@ -29021,7 +29025,7 @@
     <row r="140" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A140" s="6">
         <f t="shared" si="12"/>
-        <v>17.48939240204124</v>
+        <v>17.19819451490644</v>
       </c>
       <c r="B140" s="20">
         <v>110</v>
@@ -29124,7 +29128,7 @@
       </c>
       <c r="AI140" s="6">
         <f t="shared" si="13"/>
-        <v>0.77669960000000016</v>
+        <v>0.74547479999999999</v>
       </c>
       <c r="AJ140" s="6">
         <f t="shared" si="14"/>
@@ -29146,7 +29150,7 @@
     <row r="141" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="6">
         <f t="shared" si="12"/>
-        <v>17.186662687636154</v>
+        <v>17.281182070488523</v>
       </c>
       <c r="B141" s="20">
         <v>136</v>
@@ -29249,7 +29253,7 @@
       </c>
       <c r="AI141" s="6">
         <f t="shared" si="13"/>
-        <v>0.58540040000000015</v>
+        <v>0.59553560000000016</v>
       </c>
       <c r="AJ141" s="6">
         <f t="shared" si="14"/>
@@ -29271,7 +29275,7 @@
     <row r="142" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="6">
         <f t="shared" si="12"/>
-        <v>17.016012265361539</v>
+        <v>16.242026172073171</v>
       </c>
       <c r="B142" s="20">
         <v>88</v>
@@ -29374,7 +29378,7 @@
       </c>
       <c r="AI142" s="6">
         <f t="shared" si="13"/>
-        <v>0.71035960000000009</v>
+        <v>0.62736600000000009</v>
       </c>
       <c r="AJ142" s="6">
         <f t="shared" si="14"/>
@@ -29396,7 +29400,7 @@
     <row r="143" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="6">
         <f t="shared" si="12"/>
-        <v>16.999865409293019</v>
+        <v>17.066101345907065</v>
       </c>
       <c r="B143" s="20">
         <v>158</v>
@@ -29499,7 +29503,7 @@
       </c>
       <c r="AI143" s="6">
         <f t="shared" si="13"/>
-        <v>0.14242040000000006</v>
+        <v>0.14952280000000007</v>
       </c>
       <c r="AJ143" s="6">
         <f t="shared" si="14"/>
@@ -29521,7 +29525,7 @@
     <row r="144" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A144" s="6">
         <f t="shared" si="12"/>
-        <v>16.968170939150671</v>
+        <v>16.188242412486193</v>
       </c>
       <c r="B144" s="20">
         <v>74</v>
@@ -29624,7 +29628,7 @@
       </c>
       <c r="AI144" s="6">
         <f t="shared" si="13"/>
-        <v>0.81437760000000015</v>
+        <v>0.73074680000000014</v>
       </c>
       <c r="AJ144" s="6">
         <f t="shared" si="14"/>
@@ -29646,7 +29650,7 @@
     <row r="145" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A145" s="6">
         <f t="shared" si="12"/>
-        <v>16.835678922080632</v>
+        <v>16.481303978035754</v>
       </c>
       <c r="B145" s="20">
         <v>126</v>
@@ -29749,7 +29753,7 @@
       </c>
       <c r="AI145" s="6">
         <f t="shared" si="13"/>
-        <v>0.54002920000000021</v>
+        <v>0.5020300000000002</v>
       </c>
       <c r="AJ145" s="6">
         <f t="shared" si="14"/>
@@ -29771,7 +29775,7 @@
     <row r="146" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A146" s="6">
         <f t="shared" si="12"/>
-        <v>16.818072458145569</v>
+        <v>16.620946312930851</v>
       </c>
       <c r="B146" s="18">
         <v>173</v>
@@ -29874,7 +29878,7 @@
       </c>
       <c r="AI146" s="6">
         <f t="shared" si="13"/>
-        <v>0.63623160000000023</v>
+        <v>0.61509400000000014</v>
       </c>
       <c r="AJ146" s="6">
         <f t="shared" si="14"/>
@@ -29896,7 +29900,7 @@
     <row r="147" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6">
         <f t="shared" si="12"/>
-        <v>16.609993882240584</v>
+        <v>16.826596138350887</v>
       </c>
       <c r="B147" s="18">
         <v>35</v>
@@ -29999,7 +30003,7 @@
       </c>
       <c r="AI147" s="6">
         <f t="shared" si="13"/>
-        <v>0.12004120000000003</v>
+        <v>0.14326720000000001</v>
       </c>
       <c r="AJ147" s="6">
         <f t="shared" si="14"/>
@@ -30021,7 +30025,7 @@
     <row r="148" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A148" s="6">
         <f t="shared" si="12"/>
-        <v>16.234811990808439</v>
+        <v>16.634447163448623</v>
       </c>
       <c r="B148" s="18">
         <v>159</v>
@@ -30124,7 +30128,7 @@
       </c>
       <c r="AI148" s="6">
         <f t="shared" si="13"/>
-        <v>0.12976200000000004</v>
+        <v>0.17261440000000003</v>
       </c>
       <c r="AJ148" s="6">
         <f t="shared" si="14"/>
@@ -30146,7 +30150,7 @@
     <row r="149" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A149" s="6">
         <f t="shared" si="12"/>
-        <v>16.164498492942194</v>
+        <v>16.307627950699811</v>
       </c>
       <c r="B149" s="20">
         <v>20</v>
@@ -30249,7 +30253,7 @@
       </c>
       <c r="AI149" s="6">
         <f t="shared" si="13"/>
-        <v>0.33436680000000008</v>
+        <v>0.34971440000000015</v>
       </c>
       <c r="AJ149" s="6">
         <f t="shared" si="14"/>
@@ -30271,7 +30275,7 @@
     <row r="150" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A150" s="6">
         <f t="shared" si="12"/>
-        <v>16.010437643618125</v>
+        <v>17.04584231102092</v>
       </c>
       <c r="B150" s="18">
         <v>177</v>
@@ -30374,7 +30378,7 @@
       </c>
       <c r="AI150" s="6">
         <f t="shared" si="13"/>
-        <v>0.39046960000000014</v>
+        <v>0.50149480000000024</v>
       </c>
       <c r="AJ150" s="6">
         <f t="shared" si="14"/>
@@ -30396,7 +30400,7 @@
     <row r="151" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A151" s="6">
         <f t="shared" si="12"/>
-        <v>15.394803187203436</v>
+        <v>15.813078874332271</v>
       </c>
       <c r="B151" s="18">
         <v>3</v>
@@ -30499,7 +30503,7 @@
       </c>
       <c r="AI151" s="6">
         <f t="shared" si="13"/>
-        <v>0.15668640000000003</v>
+        <v>0.20153760000000001</v>
       </c>
       <c r="AJ151" s="6">
         <f t="shared" si="14"/>
@@ -30521,7 +30525,7 @@
     <row r="152" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A152" s="6">
         <f t="shared" si="12"/>
-        <v>15.164503416992448</v>
+        <v>15.025219940911395</v>
       </c>
       <c r="B152" s="18">
         <v>53</v>
@@ -30624,7 +30628,7 @@
       </c>
       <c r="AI152" s="6">
         <f t="shared" si="13"/>
-        <v>0.28516680000000005</v>
+        <v>0.27023160000000013</v>
       </c>
       <c r="AJ152" s="6">
         <f t="shared" si="14"/>
@@ -30646,7 +30650,7 @@
     <row r="153" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A153" s="6">
         <f t="shared" si="12"/>
-        <v>15.161188635888864</v>
+        <v>14.997102121818017</v>
       </c>
       <c r="B153" s="20">
         <v>76</v>
@@ -30749,7 +30753,7 @@
       </c>
       <c r="AI153" s="6">
         <f t="shared" si="13"/>
-        <v>0.51240880000000022</v>
+        <v>0.4948140000000002</v>
       </c>
       <c r="AJ153" s="6">
         <f t="shared" si="14"/>
@@ -30771,7 +30775,7 @@
     <row r="154" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A154" s="6">
         <f t="shared" si="12"/>
-        <v>15.039203795995103</v>
+        <v>15.286872332806109</v>
       </c>
       <c r="B154" s="20">
         <v>146</v>
@@ -30874,7 +30878,7 @@
       </c>
       <c r="AI154" s="6">
         <f t="shared" si="13"/>
-        <v>0.15047840000000007</v>
+        <v>0.17703560000000004</v>
       </c>
       <c r="AJ154" s="6">
         <f t="shared" si="14"/>
@@ -30896,7 +30900,7 @@
     <row r="155" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A155" s="6">
         <f t="shared" si="12"/>
-        <v>15.009654271986626</v>
+        <v>14.978774508341036</v>
       </c>
       <c r="B155" s="20">
         <v>82</v>
@@ -30999,7 +31003,7 @@
       </c>
       <c r="AI155" s="6">
         <f t="shared" si="13"/>
-        <v>0.39099480000000009</v>
+        <v>0.38768360000000002</v>
       </c>
       <c r="AJ155" s="6">
         <f t="shared" si="14"/>
@@ -31021,7 +31025,7 @@
     <row r="156" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A156" s="6">
         <f t="shared" si="12"/>
-        <v>14.96248589931063</v>
+        <v>14.918303739293917</v>
       </c>
       <c r="B156" s="18">
         <v>121</v>
@@ -31124,7 +31128,7 @@
       </c>
       <c r="AI156" s="6">
         <f t="shared" si="13"/>
-        <v>0.43028520000000015</v>
+        <v>0.42554760000000008</v>
       </c>
       <c r="AJ156" s="6">
         <f t="shared" si="14"/>
@@ -31146,7 +31150,7 @@
     <row r="157" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A157" s="6">
         <f t="shared" si="12"/>
-        <v>14.925705482109279</v>
+        <v>14.751632844907336</v>
       </c>
       <c r="B157" s="20">
         <v>70</v>
@@ -31249,7 +31253,7 @@
       </c>
       <c r="AI157" s="6">
         <f t="shared" si="13"/>
-        <v>0.31471400000000005</v>
+        <v>0.2960484000000001</v>
       </c>
       <c r="AJ157" s="6">
         <f t="shared" si="14"/>
@@ -31271,7 +31275,7 @@
     <row r="158" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="6">
         <f t="shared" si="12"/>
-        <v>14.782664209615325</v>
+        <v>15.056213852994714</v>
       </c>
       <c r="B158" s="20">
         <v>116</v>
@@ -31374,7 +31378,7 @@
       </c>
       <c r="AI158" s="6">
         <f t="shared" si="13"/>
-        <v>0.26247680000000012</v>
+        <v>0.2918092000000001</v>
       </c>
       <c r="AJ158" s="6">
         <f t="shared" si="14"/>
@@ -31396,7 +31400,7 @@
     <row r="159" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="6">
         <f t="shared" si="12"/>
-        <v>14.666987674952994</v>
+        <v>14.630422871467363</v>
       </c>
       <c r="B159" s="20">
         <v>16</v>
@@ -31499,7 +31503,7 @@
       </c>
       <c r="AI159" s="6">
         <f t="shared" si="13"/>
-        <v>0.57471360000000016</v>
+        <v>0.5707928000000001</v>
       </c>
       <c r="AJ159" s="6">
         <f t="shared" si="14"/>
@@ -31521,7 +31525,7 @@
     <row r="160" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="6">
         <f t="shared" si="12"/>
-        <v>14.630638037542148</v>
+        <v>13.43037094511922</v>
       </c>
       <c r="B160" s="18">
         <v>181</v>
@@ -31624,7 +31628,7 @@
       </c>
       <c r="AI160" s="6">
         <f t="shared" si="13"/>
-        <v>0.61209080000000005</v>
+        <v>0.48338760000000003</v>
       </c>
       <c r="AJ160" s="6">
         <f t="shared" si="14"/>
@@ -31646,7 +31650,7 @@
     <row r="161" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A161" s="6">
         <f t="shared" si="12"/>
-        <v>14.62335447193291</v>
+        <v>15.28738503088722</v>
       </c>
       <c r="B161" s="18">
         <v>65</v>
@@ -31749,7 +31753,7 @@
       </c>
       <c r="AI161" s="6">
         <f t="shared" si="13"/>
-        <v>0.35785200000000006</v>
+        <v>0.42905520000000003</v>
       </c>
       <c r="AJ161" s="6">
         <f t="shared" si="14"/>
@@ -31771,7 +31775,7 @@
     <row r="162" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="6">
         <f t="shared" si="12"/>
-        <v>14.621931421409171</v>
+        <v>15.127650034319135</v>
       </c>
       <c r="B162" s="20">
         <v>64</v>
@@ -31874,7 +31878,7 @@
       </c>
       <c r="AI162" s="6">
         <f t="shared" si="13"/>
-        <v>0.28559880000000004</v>
+        <v>0.33982640000000008</v>
       </c>
       <c r="AJ162" s="6">
         <f t="shared" si="14"/>
@@ -31896,7 +31900,7 @@
     <row r="163" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A163" s="6">
         <f t="shared" si="12"/>
-        <v>14.519725297681216</v>
+        <v>13.986965442120026</v>
       </c>
       <c r="B163" s="20">
         <v>168</v>
@@ -31999,7 +32003,7 @@
       </c>
       <c r="AI163" s="6">
         <f t="shared" si="13"/>
-        <v>0.25775200000000004</v>
+        <v>0.20062480000000005</v>
       </c>
       <c r="AJ163" s="6">
         <f t="shared" si="14"/>
@@ -32021,7 +32025,7 @@
     <row r="164" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A164" s="6">
         <f t="shared" si="12"/>
-        <v>14.490950192485595</v>
+        <v>14.694966277716432</v>
       </c>
       <c r="B164" s="20">
         <v>38</v>
@@ -32124,7 +32128,7 @@
       </c>
       <c r="AI164" s="6">
         <f t="shared" si="13"/>
-        <v>0.36772640000000006</v>
+        <v>0.38960280000000003</v>
       </c>
       <c r="AJ164" s="6">
         <f t="shared" si="14"/>
@@ -32146,7 +32150,7 @@
     <row r="165" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="6">
         <f t="shared" si="12"/>
-        <v>14.45868557700916</v>
+        <v>14.274481333373124</v>
       </c>
       <c r="B165" s="18">
         <v>163</v>
@@ -32249,7 +32253,7 @@
       </c>
       <c r="AI165" s="6">
         <f t="shared" si="13"/>
-        <v>0.62415840000000022</v>
+        <v>0.60440640000000023</v>
       </c>
       <c r="AJ165" s="6">
         <f t="shared" si="14"/>
@@ -32271,7 +32275,7 @@
     <row r="166" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A166" s="6">
         <f t="shared" si="12"/>
-        <v>13.95048583962517</v>
+        <v>14.567267898176606</v>
       </c>
       <c r="B166" s="20">
         <v>100</v>
@@ -32374,7 +32378,7 @@
       </c>
       <c r="AI166" s="6">
         <f t="shared" si="13"/>
-        <v>0.40261040000000009</v>
+        <v>0.46874720000000009</v>
       </c>
       <c r="AJ166" s="6">
         <f t="shared" si="14"/>
@@ -32396,7 +32400,7 @@
     <row r="167" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A167" s="6">
         <f t="shared" si="12"/>
-        <v>13.893948342236412</v>
+        <v>14.441133426840548</v>
       </c>
       <c r="B167" s="18">
         <v>115</v>
@@ -32499,7 +32503,7 @@
       </c>
       <c r="AI167" s="6">
         <f t="shared" si="13"/>
-        <v>0.65945080000000011</v>
+        <v>0.71812480000000012</v>
       </c>
       <c r="AJ167" s="6">
         <f t="shared" si="14"/>
@@ -32521,7 +32525,7 @@
     <row r="168" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="6">
         <f t="shared" si="12"/>
-        <v>13.762901608523078</v>
+        <v>14.097046912769699</v>
       </c>
       <c r="B168" s="20">
         <v>122</v>
@@ -32624,7 +32628,7 @@
       </c>
       <c r="AI168" s="6">
         <f t="shared" si="13"/>
-        <v>0.76787840000000007</v>
+        <v>0.8037084000000001</v>
       </c>
       <c r="AJ168" s="6">
         <f t="shared" si="14"/>
@@ -32646,7 +32650,7 @@
     <row r="169" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A169" s="6">
         <f t="shared" si="12"/>
-        <v>13.745751141484373</v>
+        <v>14.28922080635053</v>
       </c>
       <c r="B169" s="18">
         <v>37</v>
@@ -32749,7 +32753,7 @@
       </c>
       <c r="AI169" s="6">
         <f t="shared" si="13"/>
-        <v>0.6408948000000001</v>
+        <v>0.69917040000000008</v>
       </c>
       <c r="AJ169" s="6">
         <f t="shared" si="14"/>
@@ -32771,7 +32775,7 @@
     <row r="170" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A170" s="6">
         <f t="shared" si="12"/>
-        <v>13.71120385568056</v>
+        <v>14.18821376346653</v>
       </c>
       <c r="B170" s="20">
         <v>6</v>
@@ -32874,7 +32878,7 @@
       </c>
       <c r="AI170" s="6">
         <f t="shared" si="13"/>
-        <v>0.34530120000000003</v>
+        <v>0.39645040000000004</v>
       </c>
       <c r="AJ170" s="6">
         <f t="shared" si="14"/>
@@ -32896,7 +32900,7 @@
     <row r="171" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="6">
         <f t="shared" si="12"/>
-        <v>13.612518726312331</v>
+        <v>13.854752156137156</v>
       </c>
       <c r="B171" s="18">
         <v>19</v>
@@ -32999,7 +33003,7 @@
       </c>
       <c r="AI171" s="6">
         <f t="shared" si="13"/>
-        <v>0.33666760000000007</v>
+        <v>0.36264200000000008</v>
       </c>
       <c r="AJ171" s="6">
         <f t="shared" si="14"/>
@@ -33021,7 +33025,7 @@
     <row r="172" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="6">
         <f t="shared" si="12"/>
-        <v>13.507382792682559</v>
+        <v>13.426288907457696</v>
       </c>
       <c r="B172" s="18">
         <v>137</v>
@@ -33124,7 +33128,7 @@
       </c>
       <c r="AI172" s="6">
         <f t="shared" si="13"/>
-        <v>0.7572732000000002</v>
+        <v>0.74857760000000018</v>
       </c>
       <c r="AJ172" s="6">
         <f t="shared" si="14"/>
@@ -33146,7 +33150,7 @@
     <row r="173" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A173" s="6">
         <f t="shared" si="12"/>
-        <v>13.396426333223904</v>
+        <v>13.642244620848128</v>
       </c>
       <c r="B173" s="20">
         <v>154</v>
@@ -33249,7 +33253,7 @@
       </c>
       <c r="AI173" s="6">
         <f t="shared" si="13"/>
-        <v>0.1604072</v>
+        <v>0.18676600000000007</v>
       </c>
       <c r="AJ173" s="6">
         <f t="shared" si="14"/>
@@ -33271,7 +33275,7 @@
     <row r="174" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A174" s="6">
         <f t="shared" si="12"/>
-        <v>13.391150437195975</v>
+        <v>13.951376794294067</v>
       </c>
       <c r="B174" s="18">
         <v>135</v>
@@ -33374,7 +33378,7 @@
       </c>
       <c r="AI174" s="6">
         <f t="shared" si="13"/>
-        <v>0.31270440000000005</v>
+        <v>0.37277680000000007</v>
       </c>
       <c r="AJ174" s="6">
         <f t="shared" si="14"/>
@@ -33396,7 +33400,7 @@
     <row r="175" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A175" s="6">
         <f t="shared" si="12"/>
-        <v>13.364551463785842</v>
+        <v>13.194436718493536</v>
       </c>
       <c r="B175" s="18">
         <v>79</v>
@@ -33499,7 +33503,7 @@
       </c>
       <c r="AI175" s="6">
         <f t="shared" si="13"/>
-        <v>0.58191000000000004</v>
+        <v>0.56366880000000008</v>
       </c>
       <c r="AJ175" s="6">
         <f t="shared" si="14"/>
@@ -33521,7 +33525,7 @@
     <row r="176" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A176" s="6">
         <f t="shared" si="12"/>
-        <v>13.307043331642241</v>
+        <v>13.47523322092572</v>
       </c>
       <c r="B176" s="20">
         <v>166</v>
@@ -33624,7 +33628,7 @@
       </c>
       <c r="AI176" s="6">
         <f t="shared" si="13"/>
-        <v>0.15680280000000002</v>
+        <v>0.17483760000000004</v>
       </c>
       <c r="AJ176" s="6">
         <f t="shared" si="14"/>
@@ -33646,7 +33650,7 @@
     <row r="177" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="6">
         <f t="shared" si="12"/>
-        <v>13.183442060341992</v>
+        <v>13.2499279298099</v>
       </c>
       <c r="B177" s="20">
         <v>50</v>
@@ -33749,7 +33753,7 @@
       </c>
       <c r="AI177" s="6">
         <f t="shared" si="13"/>
-        <v>0.45813320000000013</v>
+        <v>0.46526240000000008</v>
       </c>
       <c r="AJ177" s="6">
         <f t="shared" si="14"/>
@@ -33771,7 +33775,7 @@
     <row r="178" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="6">
         <f t="shared" si="12"/>
-        <v>13.142328180488819</v>
+        <v>12.75139216329941</v>
       </c>
       <c r="B178" s="20">
         <v>112</v>
@@ -33874,7 +33878,7 @@
       </c>
       <c r="AI178" s="6">
         <f t="shared" si="13"/>
-        <v>0.44924440000000015</v>
+        <v>0.40732480000000015</v>
       </c>
       <c r="AJ178" s="6">
         <f t="shared" si="14"/>
@@ -33896,7 +33900,7 @@
     <row r="179" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="6">
         <f t="shared" si="12"/>
-        <v>12.944730818586049</v>
+        <v>13.513182577814913</v>
       </c>
       <c r="B179" s="18">
         <v>45</v>
@@ -33999,7 +34003,7 @@
       </c>
       <c r="AI179" s="6">
         <f t="shared" si="13"/>
-        <v>0.32105240000000002</v>
+        <v>0.38200680000000004</v>
       </c>
       <c r="AJ179" s="6">
         <f t="shared" si="14"/>
@@ -34021,7 +34025,7 @@
     <row r="180" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A180" s="6">
         <f t="shared" si="12"/>
-        <v>12.821681488555308</v>
+        <v>12.199195738458322</v>
       </c>
       <c r="B180" s="18">
         <v>119</v>
@@ -34124,7 +34128,7 @@
       </c>
       <c r="AI180" s="6">
         <f t="shared" si="13"/>
-        <v>0.65472680000000016</v>
+        <v>0.58797840000000012</v>
       </c>
       <c r="AJ180" s="6">
         <f t="shared" si="14"/>
@@ -34146,7 +34150,7 @@
     <row r="181" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A181" s="6">
         <f t="shared" si="12"/>
-        <v>12.78934689187979</v>
+        <v>12.654398072159717</v>
       </c>
       <c r="B181" s="18">
         <v>107</v>
@@ -34249,7 +34253,7 @@
       </c>
       <c r="AI181" s="6">
         <f t="shared" si="13"/>
-        <v>0.45368760000000008</v>
+        <v>0.43921720000000009</v>
       </c>
       <c r="AJ181" s="6">
         <f t="shared" si="14"/>
@@ -34271,7 +34275,7 @@
     <row r="182" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A182" s="6">
         <f t="shared" si="12"/>
-        <v>12.547403085738157</v>
+        <v>12.615742934733952</v>
       </c>
       <c r="B182" s="18">
         <v>131</v>
@@ -34374,7 +34378,7 @@
       </c>
       <c r="AI182" s="6">
         <f t="shared" si="13"/>
-        <v>1.024000000000001E-2</v>
+        <v>1.7568000000000011E-2</v>
       </c>
       <c r="AJ182" s="6">
         <f t="shared" si="14"/>
@@ -34396,7 +34400,7 @@
     <row r="183" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A183" s="6">
         <f t="shared" si="12"/>
-        <v>12.499511772956515</v>
+        <v>12.599458802112862</v>
       </c>
       <c r="B183" s="18">
         <v>99</v>
@@ -34499,7 +34503,7 @@
       </c>
       <c r="AI183" s="6">
         <f t="shared" si="13"/>
-        <v>0.51104520000000009</v>
+        <v>0.52176240000000007</v>
       </c>
       <c r="AJ183" s="6">
         <f t="shared" si="14"/>
@@ -34521,7 +34525,7 @@
     <row r="184" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A184" s="6">
         <f t="shared" si="12"/>
-        <v>12.409808558894623</v>
+        <v>11.809287057208511</v>
       </c>
       <c r="B184" s="18">
         <v>87</v>
@@ -34624,7 +34628,7 @@
       </c>
       <c r="AI184" s="6">
         <f t="shared" si="13"/>
-        <v>0.52000520000000017</v>
+        <v>0.45561200000000013</v>
       </c>
       <c r="AJ184" s="6">
         <f t="shared" si="14"/>
@@ -34646,7 +34650,7 @@
     <row r="185" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A185" s="6">
         <f t="shared" si="12"/>
-        <v>11.916678056641492</v>
+        <v>11.367810588200184</v>
       </c>
       <c r="B185" s="18">
         <v>23</v>
@@ -34749,7 +34753,7 @@
       </c>
       <c r="AI185" s="6">
         <f t="shared" si="13"/>
-        <v>0.52746360000000014</v>
+        <v>0.46860920000000017</v>
       </c>
       <c r="AJ185" s="6">
         <f t="shared" si="14"/>
@@ -34771,7 +34775,7 @@
     <row r="186" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A186" s="6">
         <f t="shared" si="12"/>
-        <v>11.830812169864808</v>
+        <v>12.263833895371389</v>
       </c>
       <c r="B186" s="20">
         <v>152</v>
@@ -34874,7 +34878,7 @@
       </c>
       <c r="AI186" s="6">
         <f t="shared" si="13"/>
-        <v>0.4550224000000001</v>
+        <v>0.50145480000000009</v>
       </c>
       <c r="AJ186" s="6">
         <f t="shared" si="14"/>
@@ -34896,7 +34900,7 @@
     <row r="187" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A187" s="6">
         <f t="shared" si="12"/>
-        <v>11.820535378555013</v>
+        <v>11.90084962248948</v>
       </c>
       <c r="B187" s="20">
         <v>164</v>
@@ -34999,7 +35003,7 @@
       </c>
       <c r="AI187" s="6">
         <f t="shared" si="13"/>
-        <v>0.16193400000000005</v>
+        <v>0.17054600000000003</v>
       </c>
       <c r="AJ187" s="6">
         <f t="shared" si="14"/>
@@ -35021,7 +35025,7 @@
     <row r="188" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A188" s="6">
         <f t="shared" si="12"/>
-        <v>11.729282580799184</v>
+        <v>11.750657435315883</v>
       </c>
       <c r="B188" s="20">
         <v>172</v>
@@ -35124,7 +35128,7 @@
       </c>
       <c r="AI188" s="6">
         <f t="shared" si="13"/>
-        <v>0.13757160000000004</v>
+        <v>0.13986360000000006</v>
       </c>
       <c r="AJ188" s="6">
         <f t="shared" si="14"/>
@@ -35146,7 +35150,7 @@
     <row r="189" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A189" s="6">
         <f t="shared" si="12"/>
-        <v>11.631831746694916</v>
+        <v>12.316603002178519</v>
       </c>
       <c r="B189" s="18">
         <v>111</v>
@@ -35249,7 +35253,7 @@
       </c>
       <c r="AI189" s="6">
         <f t="shared" si="13"/>
-        <v>0.35580200000000017</v>
+        <v>0.42922920000000009</v>
       </c>
       <c r="AJ189" s="6">
         <f t="shared" si="14"/>
@@ -35271,7 +35275,7 @@
     <row r="190" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A190" s="6">
         <f t="shared" si="12"/>
-        <v>11.33811065683846</v>
+        <v>11.79908382822525</v>
       </c>
       <c r="B190" s="18">
         <v>165</v>
@@ -35374,7 +35378,7 @@
       </c>
       <c r="AI190" s="6">
         <f t="shared" si="13"/>
-        <v>0.4000028000000001</v>
+        <v>0.44943240000000012</v>
       </c>
       <c r="AJ190" s="6">
         <f t="shared" si="14"/>
@@ -35396,7 +35400,7 @@
     <row r="191" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A191" s="6">
         <f t="shared" si="12"/>
-        <v>11.111714166343365</v>
+        <v>11.455953773613059</v>
       </c>
       <c r="B191" s="20">
         <v>132</v>
@@ -35499,7 +35503,7 @@
       </c>
       <c r="AI191" s="6">
         <f t="shared" si="13"/>
-        <v>0.13181880000000004</v>
+        <v>0.16873120000000005</v>
       </c>
       <c r="AJ191" s="6">
         <f t="shared" si="14"/>
@@ -35521,7 +35525,7 @@
     <row r="192" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A192" s="6">
         <f t="shared" si="12"/>
-        <v>10.945352591840996</v>
+        <v>10.992880867826553</v>
       </c>
       <c r="B192" s="18">
         <v>41</v>
@@ -35624,7 +35628,7 @@
       </c>
       <c r="AI192" s="6">
         <f t="shared" si="13"/>
-        <v>0.33890840000000011</v>
+        <v>0.34400480000000011</v>
       </c>
       <c r="AJ192" s="6">
         <f t="shared" si="14"/>
@@ -35646,7 +35650,7 @@
     <row r="193" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A193" s="6">
         <f t="shared" si="12"/>
-        <v>10.870741293383865</v>
+        <v>11.328554865856933</v>
       </c>
       <c r="B193" s="18">
         <v>89</v>
@@ -35749,7 +35753,7 @@
       </c>
       <c r="AI193" s="6">
         <f t="shared" si="13"/>
-        <v>0.14127840000000003</v>
+        <v>0.19036920000000004</v>
       </c>
       <c r="AJ193" s="6">
         <f t="shared" si="14"/>
@@ -35771,7 +35775,7 @@
     <row r="194" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A194" s="6">
         <f t="shared" si="12"/>
-        <v>10.760244113521736</v>
+        <v>10.594728878808677</v>
       </c>
       <c r="B194" s="18">
         <v>123</v>
@@ -35874,7 +35878,7 @@
       </c>
       <c r="AI194" s="6">
         <f t="shared" si="13"/>
-        <v>0.34796520000000009</v>
+        <v>0.3302172000000001</v>
       </c>
       <c r="AJ194" s="6">
         <f t="shared" si="14"/>
@@ -35896,7 +35900,7 @@
     <row r="195" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A195" s="6">
         <f t="shared" si="12"/>
-        <v>10.697541257572587</v>
+        <v>11.312678235697868</v>
       </c>
       <c r="B195" s="18">
         <v>51</v>
@@ -35999,7 +36003,7 @@
       </c>
       <c r="AI195" s="6">
         <f t="shared" si="13"/>
-        <v>0.32059560000000004</v>
+        <v>0.38655600000000012</v>
       </c>
       <c r="AJ195" s="6">
         <f t="shared" si="14"/>
@@ -36021,7 +36025,7 @@
     <row r="196" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A196" s="6">
         <f t="shared" si="12"/>
-        <v>10.567915783819268</v>
+        <v>10.706393506222206</v>
       </c>
       <c r="B196" s="20">
         <v>14</v>
@@ -36124,7 +36128,7 @@
       </c>
       <c r="AI196" s="6">
         <f t="shared" si="13"/>
-        <v>0.59917720000000019</v>
+        <v>0.61402600000000007</v>
       </c>
       <c r="AJ196" s="6">
         <f t="shared" si="14"/>
@@ -36146,7 +36150,7 @@
     <row r="197" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A197" s="6">
         <f t="shared" si="12"/>
-        <v>10.549448655585064</v>
+        <v>10.970096839655017</v>
       </c>
       <c r="B197" s="20">
         <v>162</v>
@@ -36249,7 +36253,7 @@
       </c>
       <c r="AI197" s="6">
         <f t="shared" si="13"/>
-        <v>0.19019000000000003</v>
+        <v>0.23529560000000008</v>
       </c>
       <c r="AJ197" s="6">
         <f t="shared" si="14"/>
@@ -36271,7 +36275,7 @@
     <row r="198" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A198" s="6">
         <f t="shared" si="12"/>
-        <v>10.354193201826373</v>
+        <v>10.862664806469903</v>
       </c>
       <c r="B198" s="20">
         <v>134</v>
@@ -36374,7 +36378,7 @@
       </c>
       <c r="AI198" s="6">
         <f t="shared" si="13"/>
-        <v>0.26187400000000005</v>
+        <v>0.31639680000000009</v>
       </c>
       <c r="AJ198" s="6">
         <f t="shared" si="14"/>
@@ -36396,7 +36400,7 @@
     <row r="199" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A199" s="6">
         <f t="shared" ref="A199:A207" si="18">(AI199*H$3+AJ199*M$3+AK199*W$3+AL199*AB$3+AM199*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>10.186447372347725</v>
+        <v>10.244364648303439</v>
       </c>
       <c r="B199" s="18">
         <v>127</v>
@@ -36499,7 +36503,7 @@
       </c>
       <c r="AI199" s="6">
         <f t="shared" ref="AI199:AI207" si="19">H$1*((-2*10^-6)*H199^3+0.00032*H199^2-0.0021*H199)+I$1*((-2*10^-6)*I199^3+0.00032*I199^2-0.0021*I199)+J$1*((-2*10^-6)*J199^3+0.00032*J199^2-0.0021*J199)+K$1*((-2*10^-6)*K199^3+0.00032*K199^2-0.0021*K199)+L$1*((-2*10^-6)*L199^3+0.00032*L199^2-0.0021*L199)</f>
-        <v>0.51517440000000003</v>
+        <v>0.52138480000000009</v>
       </c>
       <c r="AJ199" s="6">
         <f t="shared" ref="AJ199:AJ207" si="20">(M$1*M199+N$1*N199+O$1*O199)/100</f>
@@ -36521,7 +36525,7 @@
     <row r="200" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A200" s="6">
         <f t="shared" si="18"/>
-        <v>10.143006654928525</v>
+        <v>10.688792861619266</v>
       </c>
       <c r="B200" s="20">
         <v>106</v>
@@ -36624,7 +36628,7 @@
       </c>
       <c r="AI200" s="6">
         <f t="shared" si="19"/>
-        <v>0.37682720000000014</v>
+        <v>0.4353512000000001</v>
       </c>
       <c r="AJ200" s="6">
         <f t="shared" si="20"/>
@@ -36646,7 +36650,7 @@
     <row r="201" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A201" s="6">
         <f t="shared" si="18"/>
-        <v>9.9350847533498428</v>
+        <v>10.493818974006981</v>
       </c>
       <c r="B201" s="18">
         <v>113</v>
@@ -36749,7 +36753,7 @@
       </c>
       <c r="AI201" s="6">
         <f t="shared" si="19"/>
-        <v>0.37468040000000008</v>
+        <v>0.43459280000000006</v>
       </c>
       <c r="AJ201" s="6">
         <f t="shared" si="20"/>
@@ -36771,7 +36775,7 @@
     <row r="202" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A202" s="6">
         <f t="shared" si="18"/>
-        <v>9.9190935271121141</v>
+        <v>10.676501984541463</v>
       </c>
       <c r="B202" s="18">
         <v>153</v>
@@ -36874,7 +36878,7 @@
       </c>
       <c r="AI202" s="6">
         <f t="shared" si="19"/>
-        <v>0.31778920000000005</v>
+        <v>0.39900520000000012</v>
       </c>
       <c r="AJ202" s="6">
         <f t="shared" si="20"/>
@@ -36896,7 +36900,7 @@
     <row r="203" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A203" s="6">
         <f t="shared" si="18"/>
-        <v>9.6941693276433174</v>
+        <v>9.7371204750962406</v>
       </c>
       <c r="B203" s="20">
         <v>118</v>
@@ -36999,7 +37003,7 @@
       </c>
       <c r="AI203" s="6">
         <f t="shared" si="19"/>
-        <v>6.3866800000000029E-2</v>
+        <v>6.847240000000003E-2</v>
       </c>
       <c r="AJ203" s="6">
         <f t="shared" si="20"/>
@@ -37021,7 +37025,7 @@
     <row r="204" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A204" s="6">
         <f t="shared" si="18"/>
-        <v>9.394698290011636</v>
+        <v>10.106443642006621</v>
       </c>
       <c r="B204" s="18">
         <v>77</v>
@@ -37124,7 +37128,7 @@
       </c>
       <c r="AI204" s="6">
         <f t="shared" si="19"/>
-        <v>0.28389720000000007</v>
+        <v>0.36021680000000006</v>
       </c>
       <c r="AJ204" s="6">
         <f t="shared" si="20"/>
@@ -37146,7 +37150,7 @@
     <row r="205" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A205" s="6">
         <f t="shared" si="18"/>
-        <v>9.294189471485268</v>
+        <v>9.684640544331371</v>
       </c>
       <c r="B205" s="18">
         <v>149</v>
@@ -37249,7 +37253,7 @@
       </c>
       <c r="AI205" s="6">
         <f t="shared" si="19"/>
-        <v>0.33370800000000006</v>
+        <v>0.37557560000000006</v>
       </c>
       <c r="AJ205" s="6">
         <f t="shared" si="20"/>
@@ -37271,7 +37275,7 @@
     <row r="206" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="6">
         <f t="shared" si="18"/>
-        <v>8.7456738488167343</v>
+        <v>9.1882228654988189</v>
       </c>
       <c r="B206" s="18">
         <v>117</v>
@@ -37374,7 +37378,7 @@
       </c>
       <c r="AI206" s="6">
         <f t="shared" si="19"/>
-        <v>0.51253120000000019</v>
+        <v>0.55998520000000007</v>
       </c>
       <c r="AJ206" s="6">
         <f t="shared" si="20"/>
@@ -37396,7 +37400,7 @@
     <row r="207" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A207" s="6">
         <f t="shared" si="18"/>
-        <v>8.4095126682383814</v>
+        <v>8.6968869557432313</v>
       </c>
       <c r="B207" s="20">
         <v>174</v>
@@ -37499,7 +37503,7 @@
       </c>
       <c r="AI207" s="6">
         <f t="shared" si="19"/>
-        <v>0.27989000000000008</v>
+        <v>0.31070480000000011</v>
       </c>
       <c r="AJ207" s="6">
         <f t="shared" si="20"/>
@@ -49982,12 +49986,12 @@
         <v>0.3</v>
       </c>
       <c r="T1" s="4"/>
-      <c r="U1" s="22" t="s">
+      <c r="U1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
     </row>
     <row r="2" spans="1:25" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="C2" s="2"/>
@@ -49995,24 +49999,24 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="24">
+      <c r="H2" s="25">
         <v>1</v>
       </c>
-      <c r="I2" s="25"/>
-      <c r="J2" s="24">
+      <c r="I2" s="26"/>
+      <c r="J2" s="25">
         <v>4</v>
       </c>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="25"/>
-      <c r="O2" s="26">
+      <c r="K2" s="27"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="27">
         <v>2</v>
       </c>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="25"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="26"/>
       <c r="T2" s="9"/>
     </row>
     <row r="3" spans="1:25" s="11" customFormat="1" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -50078,7 +50082,7 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="22" t="s">
         <v>25</v>
       </c>
       <c r="B5" s="14" t="s">
@@ -66162,7 +66166,7 @@
         <v>1.25</v>
       </c>
       <c r="X198">
-        <f t="shared" ref="X198:X261" si="21">U198*J$2+V198*O$2+W198*H$2</f>
+        <f t="shared" ref="X198:X206" si="21">U198*J$2+V198*O$2+W198*H$2</f>
         <v>3.9174104000000005</v>
       </c>
       <c r="Y198" t="str">

</xml_diff>

<commit_message>
Update configuration management by introducing config.json for scouting budgets and signability penalties. Refactor credentials handling to load login details from credentials.env. Enhance README to reflect these changes and provide clearer setup instructions for users.
</commit_message>
<xml_diff>
--- a/Season x amateur draft-template.xlsx
+++ b/Season x amateur draft-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13362ca80da55a94/Documents/hardball-dynasty-draft-optimizer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4A6E41B-B920-4826-824B-E20F97D11AED}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F4D1FAA-7EEC-4AD7-A890-F7367C1FBE05}"/>
   <bookViews>
     <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11981,17 +11981,15 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="1">
-        <v>0</v>
-      </c>
+      <c r="G1" s="1"/>
       <c r="H1" s="1">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="I1" s="1">
         <v>2</v>
       </c>
       <c r="J1" s="1">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="K1" s="1">
         <v>1.2</v>
@@ -12259,7 +12257,7 @@
       <c r="AH5" s="1"/>
       <c r="AI5" s="6">
         <f>H$1*((-2*10^-6)*H5^3+0.00032*H5^2-0.0021*H5)+I$1*((-2*10^-6)*I5^3+0.00032*I5^2-0.0021*I5)+J$1*((-2*10^-6)*J5^3+0.00032*J5^2-0.0021*J5)+K$1*((-2*10^-6)*K5^3+0.00032*K5^2-0.0021*K5)+L$1*((-2*10^-6)*L5^3+0.00032*L5^2-0.0021*L5)</f>
-        <v>6.5340000000000016</v>
+        <v>6.9300000000000024</v>
       </c>
       <c r="AJ5" s="6">
         <f>(M$1*M5+N$1*N5+O$1*O5)/100</f>
@@ -12400,7 +12398,7 @@
     <row r="7" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
         <f t="shared" ref="A7:A70" si="0">(AI7*H$3+AJ7*M$3+AK7*W$3+AL7*AB$3+AM7*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>78.859066668656183</v>
+        <v>79.360697192522977</v>
       </c>
       <c r="B7" s="18">
         <v>1</v>
@@ -12503,7 +12501,7 @@
       </c>
       <c r="AI7" s="6">
         <f t="shared" ref="AI7:AI70" si="1">H$1*((-2*10^-6)*H7^3+0.00032*H7^2-0.0021*H7)+I$1*((-2*10^-6)*I7^3+0.00032*I7^2-0.0021*I7)+J$1*((-2*10^-6)*J7^3+0.00032*J7^2-0.0021*J7)+K$1*((-2*10^-6)*K7^3+0.00032*K7^2-0.0021*K7)+L$1*((-2*10^-6)*L7^3+0.00032*L7^2-0.0021*L7)</f>
-        <v>5.6061428000000015</v>
+        <v>5.9742004000000009</v>
       </c>
       <c r="AJ7" s="6">
         <f t="shared" ref="AJ7:AJ70" si="2">(M$1*M7+N$1*N7+O$1*O7)/100</f>
@@ -12525,7 +12523,7 @@
     <row r="8" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <f t="shared" si="0"/>
-        <v>72.690376018383105</v>
+        <v>72.49605888362855</v>
       </c>
       <c r="B8" s="20">
         <v>10</v>
@@ -12628,7 +12626,7 @@
       </c>
       <c r="AI8" s="6">
         <f t="shared" si="1"/>
-        <v>5.1677736000000012</v>
+        <v>5.4340216000000012</v>
       </c>
       <c r="AJ8" s="6">
         <f t="shared" si="2"/>
@@ -12650,7 +12648,7 @@
     <row r="9" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <f t="shared" si="0"/>
-        <v>71.279525948252711</v>
+        <v>71.499806023628267</v>
       </c>
       <c r="B9" s="20">
         <v>48</v>
@@ -12753,7 +12751,7 @@
       </c>
       <c r="AI9" s="6">
         <f t="shared" si="1"/>
-        <v>4.4995600000000016</v>
+        <v>4.8063196000000019</v>
       </c>
       <c r="AJ9" s="6">
         <f t="shared" si="2"/>
@@ -12775,7 +12773,7 @@
     <row r="10" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <f t="shared" si="0"/>
-        <v>68.248138112148965</v>
+        <v>67.927841221417964</v>
       </c>
       <c r="B10" s="20">
         <v>4</v>
@@ -12878,7 +12876,7 @@
       </c>
       <c r="AI10" s="6">
         <f t="shared" si="1"/>
-        <v>4.1086068000000013</v>
+        <v>4.3432560000000011</v>
       </c>
       <c r="AJ10" s="6">
         <f t="shared" si="2"/>
@@ -12900,7 +12898,7 @@
     <row r="11" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <f t="shared" si="0"/>
-        <v>67.103684383300006</v>
+        <v>67.348937590836485</v>
       </c>
       <c r="B11" s="18">
         <v>5</v>
@@ -13003,7 +13001,7 @@
       </c>
       <c r="AI11" s="6">
         <f t="shared" si="1"/>
-        <v>4.5392612000000012</v>
+        <v>4.8322612000000014</v>
       </c>
       <c r="AJ11" s="6">
         <f t="shared" si="2"/>
@@ -13025,7 +13023,7 @@
     <row r="12" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <f t="shared" si="0"/>
-        <v>66.324026231758637</v>
+        <v>66.170324205315637</v>
       </c>
       <c r="B12" s="20">
         <v>8</v>
@@ -13128,7 +13126,7 @@
       </c>
       <c r="AI12" s="6">
         <f t="shared" si="1"/>
-        <v>3.9504720000000013</v>
+        <v>4.1960252000000011</v>
       </c>
       <c r="AJ12" s="6">
         <f t="shared" si="2"/>
@@ -13150,7 +13148,7 @@
     <row r="13" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <f t="shared" si="0"/>
-        <v>64.191908890148909</v>
+        <v>64.196434892722991</v>
       </c>
       <c r="B13" s="18">
         <v>13</v>
@@ -13253,7 +13251,7 @@
       </c>
       <c r="AI13" s="6">
         <f t="shared" si="1"/>
-        <v>4.2661252000000012</v>
+        <v>4.520828400000001</v>
       </c>
       <c r="AJ13" s="6">
         <f t="shared" si="2"/>
@@ -13275,7 +13273,7 @@
     <row r="14" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="6">
         <f t="shared" si="0"/>
-        <v>61.978574562057958</v>
+        <v>60.853037140431404</v>
       </c>
       <c r="B14" s="20">
         <v>18</v>
@@ -13378,7 +13376,7 @@
       </c>
       <c r="AI14" s="6">
         <f t="shared" si="1"/>
-        <v>3.2362420000000007</v>
+        <v>3.3565300000000007</v>
       </c>
       <c r="AJ14" s="6">
         <f t="shared" si="2"/>
@@ -13400,7 +13398,7 @@
     <row r="15" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="6">
         <f t="shared" si="0"/>
-        <v>61.924449998507875</v>
+        <v>61.963144345473637</v>
       </c>
       <c r="B15" s="18">
         <v>15</v>
@@ -13503,7 +13501,7 @@
       </c>
       <c r="AI15" s="6">
         <f t="shared" si="1"/>
-        <v>3.0183412000000014</v>
+        <v>3.2678644000000014</v>
       </c>
       <c r="AJ15" s="6">
         <f t="shared" si="2"/>
@@ -13525,7 +13523,7 @@
     <row r="16" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="6">
         <f t="shared" si="0"/>
-        <v>63.02113118863587</v>
+        <v>63.712419524268626</v>
       </c>
       <c r="B16" s="20">
         <v>2</v>
@@ -13628,7 +13626,7 @@
       </c>
       <c r="AI16" s="6">
         <f t="shared" si="1"/>
-        <v>5.2430836000000012</v>
+        <v>5.5695108000000015</v>
       </c>
       <c r="AJ16" s="6">
         <f t="shared" si="2"/>
@@ -13650,7 +13648,7 @@
     <row r="17" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="6">
         <f t="shared" si="0"/>
-        <v>62.613598287027358</v>
+        <v>60.867844675003226</v>
       </c>
       <c r="B17" s="18">
         <v>47</v>
@@ -13753,7 +13751,7 @@
       </c>
       <c r="AI17" s="6">
         <f t="shared" si="1"/>
-        <v>3.9506364000000005</v>
+        <v>4.0044780000000006</v>
       </c>
       <c r="AJ17" s="6">
         <f t="shared" si="2"/>
@@ -13775,7 +13773,7 @@
     <row r="18" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="6">
         <f t="shared" si="0"/>
-        <v>61.872032737473518</v>
+        <v>60.849781848531499</v>
       </c>
       <c r="B18" s="18">
         <v>21</v>
@@ -13878,7 +13876,7 @@
       </c>
       <c r="AI18" s="6">
         <f t="shared" si="1"/>
-        <v>3.540296000000001</v>
+        <v>3.6716464000000011</v>
       </c>
       <c r="AJ18" s="6">
         <f t="shared" si="2"/>
@@ -13900,7 +13898,7 @@
     <row r="19" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="6">
         <f t="shared" si="0"/>
-        <v>58.970004476409308</v>
+        <v>59.290353129092132</v>
       </c>
       <c r="B19" s="18">
         <v>27</v>
@@ -14003,7 +14001,7 @@
       </c>
       <c r="AI19" s="6">
         <f t="shared" si="1"/>
-        <v>4.8775864000000011</v>
+        <v>5.1467268000000024</v>
       </c>
       <c r="AJ19" s="6">
         <f t="shared" si="2"/>
@@ -14025,7 +14023,7 @@
     <row r="20" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="6">
         <f t="shared" si="0"/>
-        <v>59.661036587185514</v>
+        <v>60.779205819291136</v>
       </c>
       <c r="B20" s="20">
         <v>12</v>
@@ -14128,7 +14126,7 @@
       </c>
       <c r="AI20" s="6">
         <f t="shared" si="1"/>
-        <v>4.9208472000000008</v>
+        <v>5.281432800000001</v>
       </c>
       <c r="AJ20" s="6">
         <f t="shared" si="2"/>
@@ -14150,7 +14148,7 @@
     <row r="21" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="6">
         <f t="shared" si="0"/>
-        <v>55.63346160732938</v>
+        <v>54.975286431726936</v>
       </c>
       <c r="B21" s="20">
         <v>34</v>
@@ -14253,7 +14251,7 @@
       </c>
       <c r="AI21" s="6">
         <f t="shared" si="1"/>
-        <v>2.5487284000000008</v>
+        <v>2.6958552000000009</v>
       </c>
       <c r="AJ21" s="6">
         <f t="shared" si="2"/>
@@ -14275,7 +14273,7 @@
     <row r="22" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="6">
         <f t="shared" si="0"/>
-        <v>58.660293950878859</v>
+        <v>57.986485401407329</v>
       </c>
       <c r="B22" s="20">
         <v>28</v>
@@ -14378,7 +14376,7 @@
       </c>
       <c r="AI22" s="6">
         <f t="shared" si="1"/>
-        <v>3.3180904000000004</v>
+        <v>3.4754652000000008</v>
       </c>
       <c r="AJ22" s="6">
         <f t="shared" si="2"/>
@@ -14400,7 +14398,7 @@
     <row r="23" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="6">
         <f t="shared" si="0"/>
-        <v>57.577431883971471</v>
+        <v>56.308136502957126</v>
       </c>
       <c r="B23" s="18">
         <v>43</v>
@@ -14503,7 +14501,7 @@
       </c>
       <c r="AI23" s="6">
         <f t="shared" si="1"/>
-        <v>3.2831680000000012</v>
+        <v>3.3700432000000009</v>
       </c>
       <c r="AJ23" s="6">
         <f t="shared" si="2"/>
@@ -14525,7 +14523,7 @@
     <row r="24" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="6">
         <f t="shared" si="0"/>
-        <v>58.631276970366159</v>
+        <v>58.286657217273657</v>
       </c>
       <c r="B24" s="20">
         <v>30</v>
@@ -14628,7 +14626,7 @@
       </c>
       <c r="AI24" s="6">
         <f t="shared" si="1"/>
-        <v>3.5008052000000007</v>
+        <v>3.6946672000000009</v>
       </c>
       <c r="AJ24" s="6">
         <f t="shared" si="2"/>
@@ -14650,7 +14648,7 @@
     <row r="25" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="6">
         <f t="shared" si="0"/>
-        <v>58.234936584201243</v>
+        <v>58.030650281323275</v>
       </c>
       <c r="B25" s="20">
         <v>36</v>
@@ -14753,7 +14751,7 @@
       </c>
       <c r="AI25" s="6">
         <f t="shared" si="1"/>
-        <v>3.4340856000000008</v>
+        <v>3.6419816000000007</v>
       </c>
       <c r="AJ25" s="6">
         <f t="shared" si="2"/>
@@ -14775,7 +14773,7 @@
     <row r="26" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="6">
         <f t="shared" si="0"/>
-        <v>54.381740129517446</v>
+        <v>53.403975364425186</v>
       </c>
       <c r="B26" s="20">
         <v>72</v>
@@ -14878,7 +14876,7 @@
       </c>
       <c r="AI26" s="6">
         <f t="shared" si="1"/>
-        <v>3.0563168000000007</v>
+        <v>3.1629520000000007</v>
       </c>
       <c r="AJ26" s="6">
         <f t="shared" si="2"/>
@@ -14900,7 +14898,7 @@
     <row r="27" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="6">
         <f t="shared" si="0"/>
-        <v>55.504994479095153</v>
+        <v>56.084720331544162</v>
       </c>
       <c r="B27" s="18">
         <v>49</v>
@@ -15003,7 +15001,7 @@
       </c>
       <c r="AI27" s="6">
         <f t="shared" si="1"/>
-        <v>3.2806424000000005</v>
+        <v>3.5649012000000009</v>
       </c>
       <c r="AJ27" s="6">
         <f t="shared" si="2"/>
@@ -15025,7 +15023,7 @@
     <row r="28" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="6">
         <f t="shared" si="0"/>
-        <v>54.321302635112943</v>
+        <v>52.898692098484723</v>
       </c>
       <c r="B28" s="20">
         <v>32</v>
@@ -15128,7 +15126,7 @@
       </c>
       <c r="AI28" s="6">
         <f t="shared" si="1"/>
-        <v>2.467696000000001</v>
+        <v>2.5246300000000006</v>
       </c>
       <c r="AJ28" s="6">
         <f t="shared" si="2"/>
@@ -15150,7 +15148,7 @@
     <row r="29" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="6">
         <f t="shared" si="0"/>
-        <v>50.731671640454806</v>
+        <v>49.752132157195675</v>
       </c>
       <c r="B29" s="20">
         <v>182</v>
@@ -15253,7 +15251,7 @@
       </c>
       <c r="AI29" s="6">
         <f t="shared" si="1"/>
-        <v>4.3565520000000024</v>
+        <v>4.4485356000000014</v>
       </c>
       <c r="AJ29" s="6">
         <f t="shared" si="2"/>
@@ -15275,7 +15273,7 @@
     <row r="30" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="6">
         <f t="shared" si="0"/>
-        <v>50.948509504909126</v>
+        <v>50.521523174996041</v>
       </c>
       <c r="B30" s="20">
         <v>68</v>
@@ -15378,7 +15376,7 @@
       </c>
       <c r="AI30" s="6">
         <f t="shared" si="1"/>
-        <v>1.6394800000000005</v>
+        <v>1.7937600000000005</v>
       </c>
       <c r="AJ30" s="6">
         <f t="shared" si="2"/>
@@ -15400,7 +15398,7 @@
     <row r="31" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="6">
         <f t="shared" si="0"/>
-        <v>48.384562356381863</v>
+        <v>48.717706819391871</v>
       </c>
       <c r="B31" s="20">
         <v>42</v>
@@ -15503,7 +15501,7 @@
       </c>
       <c r="AI31" s="6">
         <f t="shared" si="1"/>
-        <v>3.7106208000000018</v>
+        <v>3.9392656000000015</v>
       </c>
       <c r="AJ31" s="6">
         <f t="shared" si="2"/>
@@ -15525,7 +15523,7 @@
     <row r="32" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="6">
         <f t="shared" si="0"/>
-        <v>48.543766152376953</v>
+        <v>47.998015915272028</v>
       </c>
       <c r="B32" s="20">
         <v>44</v>
@@ -15628,7 +15626,7 @@
       </c>
       <c r="AI32" s="6">
         <f t="shared" si="1"/>
-        <v>2.5031900000000005</v>
+        <v>2.6347420000000006</v>
       </c>
       <c r="AJ32" s="6">
         <f t="shared" si="2"/>
@@ -15650,7 +15648,7 @@
     <row r="33" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="6">
         <f t="shared" si="0"/>
-        <v>51.296518398042316</v>
+        <v>51.440333127077544</v>
       </c>
       <c r="B33" s="20">
         <v>26</v>
@@ -15753,7 +15751,7 @@
       </c>
       <c r="AI33" s="6">
         <f t="shared" si="1"/>
-        <v>2.856719200000001</v>
+        <v>3.0758440000000009</v>
       </c>
       <c r="AJ33" s="6">
         <f t="shared" si="2"/>
@@ -15775,7 +15773,7 @@
     <row r="34" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="6">
         <f t="shared" si="0"/>
-        <v>48.440477931302041</v>
+        <v>48.665199372598671</v>
       </c>
       <c r="B34" s="20">
         <v>56</v>
@@ -15878,7 +15876,7 @@
       </c>
       <c r="AI34" s="6">
         <f t="shared" si="1"/>
-        <v>2.8949864000000005</v>
+        <v>3.1117972000000007</v>
       </c>
       <c r="AJ34" s="6">
         <f t="shared" si="2"/>
@@ -15900,7 +15898,7 @@
     <row r="35" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="6">
         <f t="shared" si="0"/>
-        <v>49.516531379629342</v>
+        <v>49.66956240196852</v>
       </c>
       <c r="B35" s="18">
         <v>55</v>
@@ -16003,7 +16001,7 @@
       </c>
       <c r="AI35" s="6">
         <f t="shared" si="1"/>
-        <v>3.8382692000000005</v>
+        <v>4.0513700000000004</v>
       </c>
       <c r="AJ35" s="6">
         <f t="shared" si="2"/>
@@ -16025,7 +16023,7 @@
     <row r="36" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="6">
         <f t="shared" si="0"/>
-        <v>50.551895610134586</v>
+        <v>49.413771027297713</v>
       </c>
       <c r="B36" s="18">
         <v>31</v>
@@ -16128,7 +16126,7 @@
       </c>
       <c r="AI36" s="6">
         <f t="shared" si="1"/>
-        <v>1.5575588000000002</v>
+        <v>1.6311976000000001</v>
       </c>
       <c r="AJ36" s="6">
         <f t="shared" si="2"/>
@@ -16150,7 +16148,7 @@
     <row r="37" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="6">
         <f t="shared" si="0"/>
-        <v>48.358580232176443</v>
+        <v>48.505753529132434</v>
       </c>
       <c r="B37" s="20">
         <v>190</v>
@@ -16253,7 +16251,7 @@
       </c>
       <c r="AI37" s="6">
         <f t="shared" si="1"/>
-        <v>4.0086512000000019</v>
+        <v>4.2165152000000017</v>
       </c>
       <c r="AJ37" s="6">
         <f t="shared" si="2"/>
@@ -16275,7 +16273,7 @@
     <row r="38" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="6">
         <f t="shared" si="0"/>
-        <v>47.923541735056247</v>
+        <v>47.770083605543</v>
       </c>
       <c r="B38" s="18">
         <v>183</v>
@@ -16378,7 +16376,7 @@
       </c>
       <c r="AI38" s="6">
         <f t="shared" si="1"/>
-        <v>3.5940956000000006</v>
+        <v>3.7668100000000009</v>
       </c>
       <c r="AJ38" s="6">
         <f t="shared" si="2"/>
@@ -16400,7 +16398,7 @@
     <row r="39" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="6">
         <f t="shared" si="0"/>
-        <v>49.433175713987282</v>
+        <v>49.968702890938644</v>
       </c>
       <c r="B39" s="20">
         <v>40</v>
@@ -16503,7 +16501,7 @@
       </c>
       <c r="AI39" s="6">
         <f t="shared" si="1"/>
-        <v>2.2533468000000005</v>
+        <v>2.5086468000000011</v>
       </c>
       <c r="AJ39" s="6">
         <f t="shared" si="2"/>
@@ -16525,7 +16523,7 @@
     <row r="40" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="6">
         <f t="shared" si="0"/>
-        <v>46.570726073592162</v>
+        <v>45.424153080166334</v>
       </c>
       <c r="B40" s="18">
         <v>85</v>
@@ -16628,7 +16626,7 @@
       </c>
       <c r="AI40" s="6">
         <f t="shared" si="1"/>
-        <v>1.9529724000000006</v>
+        <v>2.0099064000000006</v>
       </c>
       <c r="AJ40" s="6">
         <f t="shared" si="2"/>
@@ -16650,7 +16648,7 @@
     <row r="41" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="6">
         <f t="shared" si="0"/>
-        <v>47.578959831687008</v>
+        <v>47.168646194580745</v>
       </c>
       <c r="B41" s="20">
         <v>60</v>
@@ -16753,7 +16751,7 @@
       </c>
       <c r="AI41" s="6">
         <f t="shared" si="1"/>
-        <v>3.1760248000000009</v>
+        <v>3.3188152000000009</v>
       </c>
       <c r="AJ41" s="6">
         <f t="shared" si="2"/>
@@ -16775,7 +16773,7 @@
     <row r="42" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="6">
         <f t="shared" si="0"/>
-        <v>46.580777253872093</v>
+        <v>47.879488293784981</v>
       </c>
       <c r="B42" s="20">
         <v>184</v>
@@ -16878,7 +16876,7 @@
       </c>
       <c r="AI42" s="6">
         <f t="shared" si="1"/>
-        <v>2.4811204000000009</v>
+        <v>2.8099824000000009</v>
       </c>
       <c r="AJ42" s="6">
         <f t="shared" si="2"/>
@@ -16900,7 +16898,7 @@
     <row r="43" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="6">
         <f t="shared" si="0"/>
-        <v>44.601916947685687</v>
+        <v>43.252133596189523</v>
       </c>
       <c r="B43" s="18">
         <v>91</v>
@@ -17003,7 +17001,7 @@
       </c>
       <c r="AI43" s="6">
         <f t="shared" si="1"/>
-        <v>3.0713164000000011</v>
+        <v>3.0978592000000007</v>
       </c>
       <c r="AJ43" s="6">
         <f t="shared" si="2"/>
@@ -17025,7 +17023,7 @@
     <row r="44" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="6">
         <f t="shared" si="0"/>
-        <v>46.405658181384098</v>
+        <v>45.372618824917616</v>
       </c>
       <c r="B44" s="18">
         <v>69</v>
@@ -17128,7 +17126,7 @@
       </c>
       <c r="AI44" s="6">
         <f t="shared" si="1"/>
-        <v>2.3928444000000004</v>
+        <v>2.4617484000000003</v>
       </c>
       <c r="AJ44" s="6">
         <f t="shared" si="2"/>
@@ -17150,7 +17148,7 @@
     <row r="45" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="6">
         <f t="shared" si="0"/>
-        <v>44.629787221343506</v>
+        <v>43.787828702171431</v>
       </c>
       <c r="B45" s="18">
         <v>161</v>
@@ -17253,7 +17251,7 @@
       </c>
       <c r="AI45" s="6">
         <f t="shared" si="1"/>
-        <v>1.7994404000000004</v>
+        <v>1.8825580000000004</v>
       </c>
       <c r="AJ45" s="6">
         <f t="shared" si="2"/>
@@ -17275,7 +17273,7 @@
     <row r="46" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46" s="6">
         <f t="shared" si="0"/>
-        <v>45.1574083082157</v>
+        <v>44.418490927143729</v>
       </c>
       <c r="B46" s="20">
         <v>66</v>
@@ -17378,7 +17376,7 @@
       </c>
       <c r="AI46" s="6">
         <f t="shared" si="1"/>
-        <v>3.3604800000000008</v>
+        <v>3.4571440000000013</v>
       </c>
       <c r="AJ46" s="6">
         <f t="shared" si="2"/>
@@ -17400,7 +17398,7 @@
     <row r="47" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A47" s="6">
         <f t="shared" si="0"/>
-        <v>44.465297084365389</v>
+        <v>43.718975724173653</v>
       </c>
       <c r="B47" s="18">
         <v>39</v>
@@ -17503,7 +17501,7 @@
       </c>
       <c r="AI47" s="6">
         <f t="shared" si="1"/>
-        <v>2.9526044000000007</v>
+        <v>3.0457044000000009</v>
       </c>
       <c r="AJ47" s="6">
         <f t="shared" si="2"/>
@@ -17525,7 +17523,7 @@
     <row r="48" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="6">
         <f t="shared" si="0"/>
-        <v>42.865443313736598</v>
+        <v>42.688314362597666</v>
       </c>
       <c r="B48" s="18">
         <v>57</v>
@@ -17628,7 +17626,7 @@
       </c>
       <c r="AI48" s="6">
         <f t="shared" si="1"/>
-        <v>2.2956900000000005</v>
+        <v>2.4457424000000008</v>
       </c>
       <c r="AJ48" s="6">
         <f t="shared" si="2"/>
@@ -17650,7 +17648,7 @@
     <row r="49" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="6">
         <f t="shared" si="0"/>
-        <v>42.17689710227102</v>
+        <v>41.427565222396488</v>
       </c>
       <c r="B49" s="18">
         <v>73</v>
@@ -17753,7 +17751,7 @@
       </c>
       <c r="AI49" s="6">
         <f t="shared" si="1"/>
-        <v>1.8890276000000004</v>
+        <v>1.9727308000000006</v>
       </c>
       <c r="AJ49" s="6">
         <f t="shared" si="2"/>
@@ -17775,7 +17773,7 @@
     <row r="50" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A50" s="6">
         <f t="shared" si="0"/>
-        <v>42.947526336208171</v>
+        <v>42.237899068970961</v>
       </c>
       <c r="B50" s="18">
         <v>59</v>
@@ -17878,7 +17876,7 @@
       </c>
       <c r="AI50" s="6">
         <f t="shared" si="1"/>
-        <v>1.5237264000000004</v>
+        <v>1.6148960000000003</v>
       </c>
       <c r="AJ50" s="6">
         <f t="shared" si="2"/>
@@ -17900,7 +17898,7 @@
     <row r="51" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A51" s="6">
         <f t="shared" si="0"/>
-        <v>41.987845653406545</v>
+        <v>42.179099909343385</v>
       </c>
       <c r="B51" s="20">
         <v>58</v>
@@ -18003,7 +18001,7 @@
       </c>
       <c r="AI51" s="6">
         <f t="shared" si="1"/>
-        <v>2.3345820000000006</v>
+        <v>2.5221192000000001</v>
       </c>
       <c r="AJ51" s="6">
         <f t="shared" si="2"/>
@@ -18025,7 +18023,7 @@
     <row r="52" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="6">
         <f t="shared" si="0"/>
-        <v>41.975607448745116</v>
+        <v>41.991240268804056</v>
       </c>
       <c r="B52" s="20">
         <v>176</v>
@@ -18128,7 +18126,7 @@
       </c>
       <c r="AI52" s="6">
         <f t="shared" si="1"/>
-        <v>1.2840096000000003</v>
+        <v>1.4519712000000005</v>
       </c>
       <c r="AJ52" s="6">
         <f t="shared" si="2"/>
@@ -18150,7 +18148,7 @@
     <row r="53" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="6">
         <f t="shared" si="0"/>
-        <v>41.172825360350942</v>
+        <v>40.054385477674003</v>
       </c>
       <c r="B53" s="20">
         <v>120</v>
@@ -18253,7 +18251,7 @@
       </c>
       <c r="AI53" s="6">
         <f t="shared" si="1"/>
-        <v>2.4666304000000006</v>
+        <v>2.5053168000000006</v>
       </c>
       <c r="AJ53" s="6">
         <f t="shared" si="2"/>
@@ -18275,7 +18273,7 @@
     <row r="54" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A54" s="6">
         <f t="shared" si="0"/>
-        <v>41.347325345429574</v>
+        <v>40.785068999755353</v>
       </c>
       <c r="B54" s="18">
         <v>81</v>
@@ -18378,7 +18376,7 @@
       </c>
       <c r="AI54" s="6">
         <f t="shared" si="1"/>
-        <v>1.2562596000000001</v>
+        <v>1.3574784000000002</v>
       </c>
       <c r="AJ54" s="6">
         <f t="shared" si="2"/>
@@ -18400,7 +18398,7 @@
     <row r="55" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A55" s="6">
         <f t="shared" si="0"/>
-        <v>40.916363812707033</v>
+        <v>40.911111478853975</v>
       </c>
       <c r="B55" s="20">
         <v>84</v>
@@ -18503,7 +18501,7 @@
       </c>
       <c r="AI55" s="6">
         <f t="shared" si="1"/>
-        <v>1.1867496000000002</v>
+        <v>1.3481944000000001</v>
       </c>
       <c r="AJ55" s="6">
         <f t="shared" si="2"/>
@@ -18525,7 +18523,7 @@
     <row r="56" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A56" s="6">
         <f t="shared" si="0"/>
-        <v>41.209320779492074</v>
+        <v>41.34259939850056</v>
       </c>
       <c r="B56" s="18">
         <v>67</v>
@@ -18628,7 +18626,7 @@
       </c>
       <c r="AI56" s="6">
         <f t="shared" si="1"/>
-        <v>2.2548724000000009</v>
+        <v>2.4328804000000002</v>
       </c>
       <c r="AJ56" s="6">
         <f t="shared" si="2"/>
@@ -18650,7 +18648,7 @@
     <row r="57" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A57" s="6">
         <f t="shared" si="0"/>
-        <v>38.179837655555211</v>
+        <v>37.637896766580795</v>
       </c>
       <c r="B57" s="18">
         <v>71</v>
@@ -18753,7 +18751,7 @@
       </c>
       <c r="AI57" s="6">
         <f t="shared" si="1"/>
-        <v>1.8055032000000004</v>
+        <v>1.8964376000000005</v>
       </c>
       <c r="AJ57" s="6">
         <f t="shared" si="2"/>
@@ -18775,7 +18773,7 @@
     <row r="58" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A58" s="6">
         <f t="shared" si="0"/>
-        <v>40.605121609119934</v>
+        <v>40.41857510828428</v>
       </c>
       <c r="B58" s="20">
         <v>90</v>
@@ -18878,7 +18876,7 @@
       </c>
       <c r="AI58" s="6">
         <f t="shared" si="1"/>
-        <v>1.4752416000000004</v>
+        <v>1.6152960000000001</v>
       </c>
       <c r="AJ58" s="6">
         <f t="shared" si="2"/>
@@ -18900,7 +18898,7 @@
     <row r="59" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A59" s="6">
         <f t="shared" si="0"/>
-        <v>37.905743979229456</v>
+        <v>37.288265005108421</v>
       </c>
       <c r="B59" s="20">
         <v>78</v>
@@ -19003,7 +19001,7 @@
       </c>
       <c r="AI59" s="6">
         <f t="shared" si="1"/>
-        <v>1.2873408000000004</v>
+        <v>1.3687908000000002</v>
       </c>
       <c r="AJ59" s="6">
         <f t="shared" si="2"/>
@@ -19025,7 +19023,7 @@
     <row r="60" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A60" s="6">
         <f t="shared" si="0"/>
-        <v>35.481799665761429</v>
+        <v>34.389233447973169</v>
       </c>
       <c r="B60" s="18">
         <v>105</v>
@@ -19128,7 +19126,7 @@
       </c>
       <c r="AI60" s="6">
         <f t="shared" si="1"/>
-        <v>1.2798012000000001</v>
+        <v>1.2988280000000001</v>
       </c>
       <c r="AJ60" s="6">
         <f t="shared" si="2"/>
@@ -19150,7 +19148,7 @@
     <row r="61" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A61" s="6">
         <f t="shared" si="0"/>
-        <v>37.975464054433132</v>
+        <v>37.779436777804946</v>
       </c>
       <c r="B61" s="20">
         <v>196</v>
@@ -19253,7 +19251,7 @@
       </c>
       <c r="AI61" s="6">
         <f t="shared" si="1"/>
-        <v>1.4178524000000003</v>
+        <v>1.5464392000000002</v>
       </c>
       <c r="AJ61" s="6">
         <f t="shared" si="2"/>
@@ -19275,7 +19273,7 @@
     <row r="62" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A62" s="6">
         <f t="shared" si="0"/>
-        <v>33.352366976036279</v>
+        <v>32.514820629415901</v>
       </c>
       <c r="B62" s="18">
         <v>167</v>
@@ -19378,7 +19376,7 @@
       </c>
       <c r="AI62" s="6">
         <f t="shared" si="1"/>
-        <v>1.4434372000000004</v>
+        <v>1.4823868000000004</v>
       </c>
       <c r="AJ62" s="6">
         <f t="shared" si="2"/>
@@ -19400,7 +19398,7 @@
     <row r="63" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A63" s="6">
         <f t="shared" si="0"/>
-        <v>34.693909248261654</v>
+        <v>33.841227317859349</v>
       </c>
       <c r="B63" s="20">
         <v>108</v>
@@ -19503,7 +19501,7 @@
       </c>
       <c r="AI63" s="6">
         <f t="shared" si="1"/>
-        <v>1.0639676000000002</v>
+        <v>1.1065468000000003</v>
       </c>
       <c r="AJ63" s="6">
         <f t="shared" si="2"/>
@@ -19525,7 +19523,7 @@
     <row r="64" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A64" s="6">
         <f t="shared" si="0"/>
-        <v>37.201614790056396</v>
+        <v>37.450960096700378</v>
       </c>
       <c r="B64" s="18">
         <v>191</v>
@@ -19628,7 +19626,7 @@
       </c>
       <c r="AI64" s="6">
         <f t="shared" si="1"/>
-        <v>2.8635564000000002</v>
+        <v>3.0385992000000002</v>
       </c>
       <c r="AJ64" s="6">
         <f t="shared" si="2"/>
@@ -19650,7 +19648,7 @@
     <row r="65" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A65" s="6">
         <f t="shared" si="0"/>
-        <v>34.704095914530427</v>
+        <v>34.716667146331275</v>
       </c>
       <c r="B65" s="20">
         <v>188</v>
@@ -19753,7 +19751,7 @@
       </c>
       <c r="AI65" s="6">
         <f t="shared" si="1"/>
-        <v>2.2032152000000007</v>
+        <v>2.3420412000000006</v>
       </c>
       <c r="AJ65" s="6">
         <f t="shared" si="2"/>
@@ -19775,7 +19773,7 @@
     <row r="66" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="6">
         <f t="shared" si="0"/>
-        <v>36.152817004386876</v>
+        <v>35.866856949620818</v>
       </c>
       <c r="B66" s="20">
         <v>80</v>
@@ -19878,7 +19876,7 @@
       </c>
       <c r="AI66" s="6">
         <f t="shared" si="1"/>
-        <v>2.1826136000000003</v>
+        <v>2.2939832000000004</v>
       </c>
       <c r="AJ66" s="6">
         <f t="shared" si="2"/>
@@ -19900,7 +19898,7 @@
     <row r="67" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A67" s="6">
         <f t="shared" si="0"/>
-        <v>35.444357486048517</v>
+        <v>34.698073187227479</v>
       </c>
       <c r="B67" s="20">
         <v>128</v>
@@ -20003,7 +20001,7 @@
       </c>
       <c r="AI67" s="6">
         <f t="shared" si="1"/>
-        <v>1.5785968000000004</v>
+        <v>1.6359780000000004</v>
       </c>
       <c r="AJ67" s="6">
         <f t="shared" si="2"/>
@@ -20025,7 +20023,7 @@
     <row r="68" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A68" s="6">
         <f t="shared" si="0"/>
-        <v>34.865537765973308</v>
+        <v>34.464505201962773</v>
       </c>
       <c r="B68" s="20">
         <v>86</v>
@@ -20128,7 +20126,7 @@
       </c>
       <c r="AI68" s="6">
         <f t="shared" si="1"/>
-        <v>1.0258696000000003</v>
+        <v>1.1193468000000002</v>
       </c>
       <c r="AJ68" s="6">
         <f t="shared" si="2"/>
@@ -20150,7 +20148,7 @@
     <row r="69" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A69" s="6">
         <f t="shared" si="0"/>
-        <v>32.941741323226594</v>
+        <v>32.514298130746973</v>
       </c>
       <c r="B69" s="18">
         <v>185</v>
@@ -20253,7 +20251,7 @@
       </c>
       <c r="AI69" s="6">
         <f t="shared" si="1"/>
-        <v>2.2581396000000007</v>
+        <v>2.3410620000000004</v>
       </c>
       <c r="AJ69" s="6">
         <f t="shared" si="2"/>
@@ -20275,7 +20273,7 @@
     <row r="70" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A70" s="6">
         <f t="shared" si="0"/>
-        <v>34.905998388492634</v>
+        <v>34.035707913027196</v>
       </c>
       <c r="B70" s="20">
         <v>94</v>
@@ -20378,7 +20376,7 @@
       </c>
       <c r="AI70" s="6">
         <f t="shared" si="1"/>
-        <v>0.95798280000000013</v>
+        <v>0.99944400000000011</v>
       </c>
       <c r="AJ70" s="6">
         <f t="shared" si="2"/>
@@ -20400,7 +20398,7 @@
     <row r="71" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A71" s="6">
         <f t="shared" ref="A71:A134" si="6">(AI71*H$3+AJ71*M$3+AK71*W$3+AL71*AB$3+AM71*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>31.95039064132024</v>
+        <v>32.333372138200957</v>
       </c>
       <c r="B71" s="18">
         <v>187</v>
@@ -20503,7 +20501,7 @@
       </c>
       <c r="AI71" s="6">
         <f t="shared" ref="AI71:AI134" si="7">H$1*((-2*10^-6)*H71^3+0.00032*H71^2-0.0021*H71)+I$1*((-2*10^-6)*I71^3+0.00032*I71^2-0.0021*I71)+J$1*((-2*10^-6)*J71^3+0.00032*J71^2-0.0021*J71)+K$1*((-2*10^-6)*K71^3+0.00032*K71^2-0.0021*K71)+L$1*((-2*10^-6)*L71^3+0.00032*L71^2-0.0021*L71)</f>
-        <v>2.1815084000000007</v>
+        <v>2.3506152000000005</v>
       </c>
       <c r="AJ71" s="6">
         <f t="shared" ref="AJ71:AJ134" si="8">(M$1*M71+N$1*N71+O$1*O71)/100</f>
@@ -20525,7 +20523,7 @@
     <row r="72" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A72" s="6">
         <f t="shared" si="6"/>
-        <v>31.414101883076182</v>
+        <v>31.3586336753342</v>
       </c>
       <c r="B72" s="20">
         <v>98</v>
@@ -20628,7 +20626,7 @@
       </c>
       <c r="AI72" s="6">
         <f t="shared" si="7"/>
-        <v>1.6699404000000002</v>
+        <v>1.7881728000000003</v>
       </c>
       <c r="AJ72" s="6">
         <f t="shared" si="8"/>
@@ -20650,7 +20648,7 @@
     <row r="73" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="6">
         <f t="shared" si="6"/>
-        <v>33.69168835238294</v>
+        <v>33.319029542543852</v>
       </c>
       <c r="B73" s="18">
         <v>97</v>
@@ -20753,7 +20751,7 @@
       </c>
       <c r="AI73" s="6">
         <f t="shared" si="7"/>
-        <v>0.85177160000000007</v>
+        <v>0.94375520000000013</v>
       </c>
       <c r="AJ73" s="6">
         <f t="shared" si="8"/>
@@ -20775,7 +20773,7 @@
     <row r="74" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A74" s="6">
         <f t="shared" si="6"/>
-        <v>33.26619206780267</v>
+        <v>32.166400356870469</v>
       </c>
       <c r="B74" s="20">
         <v>170</v>
@@ -20878,7 +20876,7 @@
       </c>
       <c r="AI74" s="6">
         <f t="shared" si="7"/>
-        <v>0.50905160000000005</v>
+        <v>0.5185012</v>
       </c>
       <c r="AJ74" s="6">
         <f t="shared" si="8"/>
@@ -20900,7 +20898,7 @@
     <row r="75" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A75" s="6">
         <f t="shared" si="6"/>
-        <v>33.841638962666742</v>
+        <v>32.967258716705274</v>
       </c>
       <c r="B75" s="20">
         <v>130</v>
@@ -21003,7 +21001,7 @@
       </c>
       <c r="AI75" s="6">
         <f t="shared" si="7"/>
-        <v>1.5267636000000007</v>
+        <v>1.5635552000000006</v>
       </c>
       <c r="AJ75" s="6">
         <f t="shared" si="8"/>
@@ -21025,7 +21023,7 @@
     <row r="76" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A76" s="6">
         <f t="shared" si="6"/>
-        <v>34.253149601599567</v>
+        <v>33.876711755140796</v>
       </c>
       <c r="B76" s="18">
         <v>197</v>
@@ -21128,7 +21126,7 @@
       </c>
       <c r="AI76" s="6">
         <f t="shared" si="7"/>
-        <v>1.5314944000000006</v>
+        <v>1.6252812000000003</v>
       </c>
       <c r="AJ76" s="6">
         <f t="shared" si="8"/>
@@ -21150,7 +21148,7 @@
     <row r="77" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A77" s="6">
         <f t="shared" si="6"/>
-        <v>31.870965859918229</v>
+        <v>30.852001496553601</v>
       </c>
       <c r="B77" s="18">
         <v>201</v>
@@ -21253,7 +21251,7 @@
       </c>
       <c r="AI77" s="6">
         <f t="shared" si="7"/>
-        <v>1.6293848000000004</v>
+        <v>1.6422964000000002</v>
       </c>
       <c r="AJ77" s="6">
         <f t="shared" si="8"/>
@@ -21275,7 +21273,7 @@
     <row r="78" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="6">
         <f t="shared" si="6"/>
-        <v>29.978660210689664</v>
+        <v>29.239845739858687</v>
       </c>
       <c r="B78" s="20">
         <v>200</v>
@@ -21378,7 +21376,7 @@
       </c>
       <c r="AI78" s="6">
         <f t="shared" si="7"/>
-        <v>1.3049724000000005</v>
+        <v>1.3415400000000004</v>
       </c>
       <c r="AJ78" s="6">
         <f t="shared" si="8"/>
@@ -21400,7 +21398,7 @@
     <row r="79" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A79" s="6">
         <f t="shared" si="6"/>
-        <v>32.997932346533759</v>
+        <v>33.291686644698018</v>
       </c>
       <c r="B79" s="18">
         <v>103</v>
@@ -21503,7 +21501,7 @@
       </c>
       <c r="AI79" s="6">
         <f t="shared" si="7"/>
-        <v>1.3023788000000003</v>
+        <v>1.4657128000000001</v>
       </c>
       <c r="AJ79" s="6">
         <f t="shared" si="8"/>
@@ -21525,7 +21523,7 @@
     <row r="80" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A80" s="6">
         <f t="shared" si="6"/>
-        <v>32.095201587633163</v>
+        <v>31.992801001539714</v>
       </c>
       <c r="B80" s="18">
         <v>189</v>
@@ -21628,7 +21626,7 @@
       </c>
       <c r="AI80" s="6">
         <f t="shared" si="7"/>
-        <v>1.7608676000000001</v>
+        <v>1.8765787999999999</v>
       </c>
       <c r="AJ80" s="6">
         <f t="shared" si="8"/>
@@ -21650,7 +21648,7 @@
     <row r="81" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A81" s="6">
         <f t="shared" si="6"/>
-        <v>34.144793040675637</v>
+        <v>34.18752953534888</v>
       </c>
       <c r="B81" s="18">
         <v>145</v>
@@ -21753,7 +21751,7 @@
       </c>
       <c r="AI81" s="6">
         <f t="shared" si="7"/>
-        <v>1.1469128000000004</v>
+        <v>1.2868780000000004</v>
       </c>
       <c r="AJ81" s="6">
         <f t="shared" si="8"/>
@@ -21775,7 +21773,7 @@
     <row r="82" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A82" s="6">
         <f t="shared" si="6"/>
-        <v>31.235067444567125</v>
+        <v>30.550620206351713</v>
       </c>
       <c r="B82" s="20">
         <v>124</v>
@@ -21878,7 +21876,7 @@
       </c>
       <c r="AI82" s="6">
         <f t="shared" si="7"/>
-        <v>0.68838280000000007</v>
+        <v>0.73597080000000004</v>
       </c>
       <c r="AJ82" s="6">
         <f t="shared" si="8"/>
@@ -21900,7 +21898,7 @@
     <row r="83" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A83" s="6">
         <f t="shared" si="6"/>
-        <v>32.355324390462258</v>
+        <v>31.767816614623051</v>
       </c>
       <c r="B83" s="18">
         <v>175</v>
@@ -22003,7 +22001,7 @@
       </c>
       <c r="AI83" s="6">
         <f t="shared" si="7"/>
-        <v>0.41141120000000009</v>
+        <v>0.47421400000000008</v>
       </c>
       <c r="AJ83" s="6">
         <f t="shared" si="8"/>
@@ -22025,7 +22023,7 @@
     <row r="84" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A84" s="6">
         <f t="shared" si="6"/>
-        <v>30.912291623146018</v>
+        <v>30.216452880146196</v>
       </c>
       <c r="B84" s="18">
         <v>129</v>
@@ -22128,7 +22126,7 @@
       </c>
       <c r="AI84" s="6">
         <f t="shared" si="7"/>
-        <v>0.64565280000000014</v>
+        <v>0.6906960000000002</v>
       </c>
       <c r="AJ84" s="6">
         <f t="shared" si="8"/>
@@ -22150,7 +22148,7 @@
     <row r="85" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A85" s="6">
         <f t="shared" si="6"/>
-        <v>32.560699662777168</v>
+        <v>31.780812024232649</v>
       </c>
       <c r="B85" s="20">
         <v>104</v>
@@ -22253,7 +22251,7 @@
       </c>
       <c r="AI85" s="6">
         <f t="shared" si="7"/>
-        <v>0.8192400000000003</v>
+        <v>0.86146560000000028</v>
       </c>
       <c r="AJ85" s="6">
         <f t="shared" si="8"/>
@@ -22275,7 +22273,7 @@
     <row r="86" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A86" s="6">
         <f t="shared" si="6"/>
-        <v>30.821583902832074</v>
+        <v>30.355289885312189</v>
       </c>
       <c r="B86" s="20">
         <v>140</v>
@@ -22378,7 +22376,7 @@
       </c>
       <c r="AI86" s="6">
         <f t="shared" si="7"/>
-        <v>0.89743640000000013</v>
+        <v>0.96764320000000015</v>
       </c>
       <c r="AJ86" s="6">
         <f t="shared" si="8"/>
@@ -22400,7 +22398,7 @@
     <row r="87" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A87" s="6">
         <f t="shared" si="6"/>
-        <v>30.575216210570293</v>
+        <v>29.483557192810778</v>
       </c>
       <c r="B87" s="20">
         <v>180</v>
@@ -22503,7 +22501,7 @@
       </c>
       <c r="AI87" s="6">
         <f t="shared" si="7"/>
-        <v>0.95593920000000021</v>
+        <v>0.95563680000000029</v>
       </c>
       <c r="AJ87" s="6">
         <f t="shared" si="8"/>
@@ -22525,7 +22523,7 @@
     <row r="88" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A88" s="6">
         <f t="shared" si="6"/>
-        <v>30.201106269957322</v>
+        <v>29.442083950901523</v>
       </c>
       <c r="B88" s="18">
         <v>139</v>
@@ -22628,7 +22626,7 @@
       </c>
       <c r="AI88" s="6">
         <f t="shared" si="7"/>
-        <v>0.46957840000000017</v>
+        <v>0.50478000000000012</v>
       </c>
       <c r="AJ88" s="6">
         <f t="shared" si="8"/>
@@ -22650,7 +22648,7 @@
     <row r="89" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A89" s="6">
         <f t="shared" si="6"/>
-        <v>29.295112208660353</v>
+        <v>29.124114371231624</v>
       </c>
       <c r="B89" s="20">
         <v>186</v>
@@ -22753,7 +22751,7 @@
       </c>
       <c r="AI89" s="6">
         <f t="shared" si="7"/>
-        <v>1.5137644000000001</v>
+        <v>1.6107600000000002</v>
       </c>
       <c r="AJ89" s="6">
         <f t="shared" si="8"/>
@@ -22775,7 +22773,7 @@
     <row r="90" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A90" s="6">
         <f t="shared" si="6"/>
-        <v>29.502574979856156</v>
+        <v>28.844280287223164</v>
       </c>
       <c r="B90" s="18">
         <v>109</v>
@@ -22878,7 +22876,7 @@
       </c>
       <c r="AI90" s="6">
         <f t="shared" si="7"/>
-        <v>0.58008320000000013</v>
+        <v>0.62371840000000012</v>
       </c>
       <c r="AJ90" s="6">
         <f t="shared" si="8"/>
@@ -22900,7 +22898,7 @@
     <row r="91" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A91" s="6">
         <f t="shared" si="6"/>
-        <v>29.236296666567185</v>
+        <v>28.418475673808871</v>
       </c>
       <c r="B91" s="20">
         <v>198</v>
@@ -23003,7 +23001,7 @@
       </c>
       <c r="AI91" s="6">
         <f t="shared" si="7"/>
-        <v>1.2400600000000002</v>
+        <v>1.2649032000000004</v>
       </c>
       <c r="AJ91" s="6">
         <f t="shared" si="8"/>
@@ -23025,7 +23023,7 @@
     <row r="92" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A92" s="6">
         <f t="shared" si="6"/>
-        <v>29.015543137664501</v>
+        <v>28.405586461945802</v>
       </c>
       <c r="B92" s="20">
         <v>150</v>
@@ -23128,7 +23126,7 @@
       </c>
       <c r="AI92" s="6">
         <f t="shared" si="7"/>
-        <v>1.0770216000000004</v>
+        <v>1.1241028000000004</v>
       </c>
       <c r="AJ92" s="6">
         <f t="shared" si="8"/>
@@ -23150,7 +23148,7 @@
     <row r="93" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A93" s="6">
         <f t="shared" si="6"/>
-        <v>27.682017368468166</v>
+        <v>27.510341904940063</v>
       </c>
       <c r="B93" s="20">
         <v>192</v>
@@ -23253,7 +23251,7 @@
       </c>
       <c r="AI93" s="6">
         <f t="shared" si="7"/>
-        <v>1.7353328000000001</v>
+        <v>1.8258652000000004</v>
       </c>
       <c r="AJ93" s="6">
         <f t="shared" si="8"/>
@@ -23275,7 +23273,7 @@
     <row r="94" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A94" s="6">
         <f t="shared" si="6"/>
-        <v>26.778284341520184</v>
+        <v>25.855914408645468</v>
       </c>
       <c r="B94" s="20">
         <v>142</v>
@@ -23378,7 +23376,7 @@
       </c>
       <c r="AI94" s="6">
         <f t="shared" si="7"/>
-        <v>0.62760320000000025</v>
+        <v>0.6310880000000002</v>
       </c>
       <c r="AJ94" s="6">
         <f t="shared" si="8"/>
@@ -23400,7 +23398,7 @@
     <row r="95" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A95" s="6">
         <f t="shared" si="6"/>
-        <v>27.409372556626575</v>
+        <v>27.282396500366936</v>
       </c>
       <c r="B95" s="20">
         <v>144</v>
@@ -23503,7 +23501,7 @@
       </c>
       <c r="AI95" s="6">
         <f t="shared" si="7"/>
-        <v>0.53177480000000021</v>
+        <v>0.62619760000000024</v>
       </c>
       <c r="AJ95" s="6">
         <f t="shared" si="8"/>
@@ -23525,7 +23523,7 @@
     <row r="96" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A96" s="6">
         <f t="shared" si="6"/>
-        <v>25.468169596227874</v>
+        <v>24.666215158361268</v>
       </c>
       <c r="B96" s="18">
         <v>147</v>
@@ -23628,7 +23626,7 @@
       </c>
       <c r="AI96" s="6">
         <f t="shared" si="7"/>
-        <v>0.29173720000000003</v>
+        <v>0.3034228000000001</v>
       </c>
       <c r="AJ96" s="6">
         <f t="shared" si="8"/>
@@ -23650,7 +23648,7 @@
     <row r="97" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A97" s="6">
         <f t="shared" si="6"/>
-        <v>26.116848906263982</v>
+        <v>26.509910782380949</v>
       </c>
       <c r="B97" s="20">
         <v>138</v>
@@ -23753,7 +23751,7 @@
       </c>
       <c r="AI97" s="6">
         <f t="shared" si="7"/>
-        <v>1.4485192000000005</v>
+        <v>1.5956460000000003</v>
       </c>
       <c r="AJ97" s="6">
         <f t="shared" si="8"/>
@@ -23775,7 +23773,7 @@
     <row r="98" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A98" s="6">
         <f t="shared" si="6"/>
-        <v>23.411881285624755</v>
+        <v>22.973629862000482</v>
       </c>
       <c r="B98" s="18">
         <v>195</v>
@@ -23878,7 +23876,7 @@
       </c>
       <c r="AI98" s="6">
         <f t="shared" si="7"/>
-        <v>1.7246736000000005</v>
+        <v>1.7686560000000005</v>
       </c>
       <c r="AJ98" s="6">
         <f t="shared" si="8"/>
@@ -23900,7 +23898,7 @@
     <row r="99" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A99" s="6">
         <f t="shared" si="6"/>
-        <v>24.824992837745082</v>
+        <v>24.422274473687992</v>
       </c>
       <c r="B99" s="20">
         <v>148</v>
@@ -24003,7 +24001,7 @@
       </c>
       <c r="AI99" s="6">
         <f t="shared" si="7"/>
-        <v>0.5910044000000001</v>
+        <v>0.64453360000000015</v>
       </c>
       <c r="AJ99" s="6">
         <f t="shared" si="8"/>
@@ -24025,7 +24023,7 @@
     <row r="100" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A100" s="6">
         <f t="shared" si="6"/>
-        <v>24.298918947148525</v>
+        <v>24.149597081720458</v>
       </c>
       <c r="B100" s="18">
         <v>141</v>
@@ -24128,7 +24126,7 @@
       </c>
       <c r="AI100" s="6">
         <f t="shared" si="7"/>
-        <v>0.8092832000000002</v>
+        <v>0.88890400000000025</v>
       </c>
       <c r="AJ100" s="6">
         <f t="shared" si="8"/>
@@ -24150,7 +24148,7 @@
     <row r="101" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A101" s="6">
         <f t="shared" si="6"/>
-        <v>24.659780655943173</v>
+        <v>24.368489344250499</v>
       </c>
       <c r="B101" s="18">
         <v>171</v>
@@ -24253,7 +24251,7 @@
       </c>
       <c r="AI101" s="6">
         <f t="shared" si="7"/>
-        <v>0.77808880000000025</v>
+        <v>0.84335320000000036</v>
       </c>
       <c r="AJ101" s="6">
         <f t="shared" si="8"/>
@@ -24275,7 +24273,7 @@
     <row r="102" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A102" s="6">
         <f t="shared" si="6"/>
-        <v>23.803424154704704</v>
+        <v>23.470430546961559</v>
       </c>
       <c r="B102" s="18">
         <v>169</v>
@@ -24378,7 +24376,7 @@
       </c>
       <c r="AI102" s="6">
         <f t="shared" si="7"/>
-        <v>0.58815720000000016</v>
+        <v>0.64539360000000012</v>
       </c>
       <c r="AJ102" s="6">
         <f t="shared" si="8"/>
@@ -24400,7 +24398,7 @@
     <row r="103" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A103" s="6">
         <f t="shared" si="6"/>
-        <v>23.28365036258915</v>
+        <v>23.15755083245794</v>
       </c>
       <c r="B103" s="18">
         <v>143</v>
@@ -24503,7 +24501,7 @@
       </c>
       <c r="AI103" s="6">
         <f t="shared" si="7"/>
-        <v>0.7182360000000001</v>
+        <v>0.79641840000000008</v>
       </c>
       <c r="AJ103" s="6">
         <f t="shared" si="8"/>
@@ -24525,7 +24523,7 @@
     <row r="104" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A104" s="6">
         <f t="shared" si="6"/>
-        <v>25.135343788235996</v>
+        <v>24.706682255766765</v>
       </c>
       <c r="B104" s="20">
         <v>114</v>
@@ -24628,7 +24626,7 @@
       </c>
       <c r="AI104" s="6">
         <f t="shared" si="7"/>
-        <v>0.91824840000000041</v>
+        <v>0.97012200000000037</v>
       </c>
       <c r="AJ104" s="6">
         <f t="shared" si="8"/>
@@ -24650,7 +24648,7 @@
     <row r="105" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A105" s="6">
         <f t="shared" si="6"/>
-        <v>23.927712256408725</v>
+        <v>23.690694314535275</v>
       </c>
       <c r="B105" s="20">
         <v>156</v>
@@ -24753,7 +24751,7 @@
       </c>
       <c r="AI105" s="6">
         <f t="shared" si="7"/>
-        <v>0.59626720000000011</v>
+        <v>0.66466720000000012</v>
       </c>
       <c r="AJ105" s="6">
         <f t="shared" si="8"/>
@@ -24775,7 +24773,7 @@
     <row r="106" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A106" s="6">
         <f t="shared" si="6"/>
-        <v>23.708954161568531</v>
+        <v>23.153233994790838</v>
       </c>
       <c r="B106" s="18">
         <v>7</v>
@@ -24878,7 +24876,7 @@
       </c>
       <c r="AI106" s="6">
         <f t="shared" si="7"/>
-        <v>0.41552160000000005</v>
+        <v>0.44761920000000011</v>
       </c>
       <c r="AJ106" s="6">
         <f t="shared" si="8"/>
@@ -24900,7 +24898,7 @@
     <row r="107" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A107" s="6">
         <f t="shared" si="6"/>
-        <v>23.142632128681846</v>
+        <v>22.576704416272136</v>
       </c>
       <c r="B107" s="18">
         <v>155</v>
@@ -25003,7 +25001,7 @@
       </c>
       <c r="AI107" s="6">
         <f t="shared" si="7"/>
-        <v>0.15136120000000006</v>
+        <v>0.18008120000000005</v>
       </c>
       <c r="AJ107" s="6">
         <f t="shared" si="8"/>
@@ -25025,7 +25023,7 @@
     <row r="108" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A108" s="6">
         <f t="shared" si="6"/>
-        <v>23.568480408248522</v>
+        <v>22.850501777157408</v>
       </c>
       <c r="B108" s="20">
         <v>102</v>
@@ -25128,7 +25126,7 @@
       </c>
       <c r="AI108" s="6">
         <f t="shared" si="7"/>
-        <v>0.42207480000000003</v>
+        <v>0.43557479999999998</v>
       </c>
       <c r="AJ108" s="6">
         <f t="shared" si="8"/>
@@ -25150,7 +25148,7 @@
     <row r="109" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A109" s="6">
         <f t="shared" si="6"/>
-        <v>22.445803515473457</v>
+        <v>21.883651734707094</v>
       </c>
       <c r="B109" s="18">
         <v>83</v>
@@ -25253,7 +25251,7 @@
       </c>
       <c r="AI109" s="6">
         <f t="shared" si="7"/>
-        <v>0.18315720000000008</v>
+        <v>0.20953760000000007</v>
       </c>
       <c r="AJ109" s="6">
         <f t="shared" si="8"/>
@@ -25275,7 +25273,7 @@
     <row r="110" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A110" s="6">
         <f t="shared" si="6"/>
-        <v>21.723200185024918</v>
+        <v>21.173984142287711</v>
       </c>
       <c r="B110" s="20">
         <v>24</v>
@@ -25378,7 +25376,7 @@
       </c>
       <c r="AI110" s="6">
         <f t="shared" si="7"/>
-        <v>0.77303280000000008</v>
+        <v>0.79799000000000009</v>
       </c>
       <c r="AJ110" s="6">
         <f t="shared" si="8"/>
@@ -25400,7 +25398,7 @@
     <row r="111" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A111" s="6">
         <f t="shared" si="6"/>
-        <v>21.547383538750783</v>
+        <v>21.512509173585823</v>
       </c>
       <c r="B111" s="20">
         <v>194</v>
@@ -25503,7 +25501,7 @@
       </c>
       <c r="AI111" s="6">
         <f t="shared" si="7"/>
-        <v>1.1032588000000003</v>
+        <v>1.1847088000000001</v>
       </c>
       <c r="AJ111" s="6">
         <f t="shared" si="8"/>
@@ -25525,7 +25523,7 @@
     <row r="112" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A112" s="6">
         <f t="shared" si="6"/>
-        <v>22.140750246202515</v>
+        <v>21.994582907630981</v>
       </c>
       <c r="B112" s="18">
         <v>9</v>
@@ -25628,7 +25626,7 @@
       </c>
       <c r="AI112" s="6">
         <f t="shared" si="7"/>
-        <v>0.48152040000000007</v>
+        <v>0.55294560000000004</v>
       </c>
       <c r="AJ112" s="6">
         <f t="shared" si="8"/>
@@ -25650,7 +25648,7 @@
     <row r="113" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A113" s="6">
         <f t="shared" si="6"/>
-        <v>21.817464412545881</v>
+        <v>21.265376800541052</v>
       </c>
       <c r="B113" s="18">
         <v>75</v>
@@ -25753,7 +25751,7 @@
       </c>
       <c r="AI113" s="6">
         <f t="shared" si="7"/>
-        <v>0.39170560000000004</v>
+        <v>0.41671680000000005</v>
       </c>
       <c r="AJ113" s="6">
         <f t="shared" si="8"/>
@@ -25775,7 +25773,7 @@
     <row r="114" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A114" s="6">
         <f t="shared" si="6"/>
-        <v>21.48115536124623</v>
+        <v>21.205417380167788</v>
       </c>
       <c r="B114" s="18">
         <v>33</v>
@@ -25878,7 +25876,7 @@
       </c>
       <c r="AI114" s="6">
         <f t="shared" si="7"/>
-        <v>0.93160040000000033</v>
+        <v>0.98600680000000029</v>
       </c>
       <c r="AJ114" s="6">
         <f t="shared" si="8"/>
@@ -25900,7 +25898,7 @@
     <row r="115" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A115" s="6">
         <f t="shared" si="6"/>
-        <v>21.462887134799605</v>
+        <v>20.988322852661415</v>
       </c>
       <c r="B115" s="18">
         <v>29</v>
@@ -26003,7 +26001,7 @@
       </c>
       <c r="AI115" s="6">
         <f t="shared" si="7"/>
-        <v>0.49443640000000016</v>
+        <v>0.52666320000000011</v>
       </c>
       <c r="AJ115" s="6">
         <f t="shared" si="8"/>
@@ -26025,7 +26023,7 @@
     <row r="116" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A116" s="6">
         <f t="shared" si="6"/>
-        <v>20.926567638544867</v>
+        <v>20.569276186090686</v>
       </c>
       <c r="B116" s="20">
         <v>54</v>
@@ -26128,7 +26126,7 @@
       </c>
       <c r="AI116" s="6">
         <f t="shared" si="7"/>
-        <v>0.57907160000000013</v>
+        <v>0.62221400000000016</v>
       </c>
       <c r="AJ116" s="6">
         <f t="shared" si="8"/>
@@ -26150,7 +26148,7 @@
     <row r="117" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A117" s="6">
         <f t="shared" si="6"/>
-        <v>19.612148378047685</v>
+        <v>19.166203214712272</v>
       </c>
       <c r="B117" s="18">
         <v>199</v>
@@ -26253,7 +26251,7 @@
       </c>
       <c r="AI117" s="6">
         <f t="shared" si="7"/>
-        <v>0.61089480000000018</v>
+        <v>0.63897480000000018</v>
       </c>
       <c r="AJ117" s="6">
         <f t="shared" si="8"/>
@@ -26275,7 +26273,7 @@
     <row r="118" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A118" s="6">
         <f t="shared" si="6"/>
-        <v>20.429120833208991</v>
+        <v>19.843636337472837</v>
       </c>
       <c r="B118" s="20">
         <v>46</v>
@@ -26378,7 +26376,7 @@
       </c>
       <c r="AI118" s="6">
         <f t="shared" si="7"/>
-        <v>0.32567600000000008</v>
+        <v>0.341476</v>
       </c>
       <c r="AJ118" s="6">
         <f t="shared" si="8"/>
@@ -26400,7 +26398,7 @@
     <row r="119" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A119" s="6">
         <f t="shared" si="6"/>
-        <v>20.248017995165473</v>
+        <v>19.874385477674007</v>
       </c>
       <c r="B119" s="18">
         <v>25</v>
@@ -26503,7 +26501,7 @@
       </c>
       <c r="AI119" s="6">
         <f t="shared" si="7"/>
-        <v>0.58732040000000019</v>
+        <v>0.62595880000000026</v>
       </c>
       <c r="AJ119" s="6">
         <f t="shared" si="8"/>
@@ -26525,7 +26523,7 @@
     <row r="120" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A120" s="6">
         <f t="shared" si="6"/>
-        <v>19.634224984332558</v>
+        <v>19.361349200638905</v>
       </c>
       <c r="B120" s="20">
         <v>160</v>
@@ -26628,7 +26626,7 @@
       </c>
       <c r="AI120" s="6">
         <f t="shared" si="7"/>
-        <v>0.53071960000000007</v>
+        <v>0.57813040000000004</v>
       </c>
       <c r="AJ120" s="6">
         <f t="shared" si="8"/>
@@ -26650,7 +26648,7 @@
     <row r="121" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A121" s="6">
         <f t="shared" si="6"/>
-        <v>20.090288280760387</v>
+        <v>20.032527592707169</v>
       </c>
       <c r="B121" s="20">
         <v>62</v>
@@ -26753,7 +26751,7 @@
       </c>
       <c r="AI121" s="6">
         <f t="shared" si="7"/>
-        <v>0.61185640000000008</v>
+        <v>0.68499160000000014</v>
       </c>
       <c r="AJ121" s="6">
         <f t="shared" si="8"/>
@@ -26775,7 +26773,7 @@
     <row r="122" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A122" s="6">
         <f t="shared" si="6"/>
-        <v>18.576597182846395</v>
+        <v>18.766550443929603</v>
       </c>
       <c r="B122" s="18">
         <v>157</v>
@@ -26878,7 +26876,7 @@
       </c>
       <c r="AI122" s="6">
         <f t="shared" si="7"/>
-        <v>0.93559080000000017</v>
+        <v>1.0302748000000004</v>
       </c>
       <c r="AJ122" s="6">
         <f t="shared" si="8"/>
@@ -26900,7 +26898,7 @@
     <row r="123" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A123" s="6">
         <f t="shared" si="6"/>
-        <v>19.664758721537488</v>
+        <v>19.264239563697057</v>
       </c>
       <c r="B123" s="20">
         <v>92</v>
@@ -27003,7 +27001,7 @@
       </c>
       <c r="AI123" s="6">
         <f t="shared" si="7"/>
-        <v>0.21471280000000004</v>
+        <v>0.24805200000000002</v>
       </c>
       <c r="AJ123" s="6">
         <f t="shared" si="8"/>
@@ -27025,7 +27023,7 @@
     <row r="124" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A124" s="6">
         <f t="shared" si="6"/>
-        <v>19.731164015637589</v>
+        <v>19.416446980271395</v>
       </c>
       <c r="B124" s="18">
         <v>11</v>
@@ -27128,7 +27126,7 @@
       </c>
       <c r="AI124" s="6">
         <f t="shared" si="7"/>
-        <v>0.49652280000000015</v>
+        <v>0.53966520000000018</v>
       </c>
       <c r="AJ124" s="6">
         <f t="shared" si="8"/>
@@ -27150,7 +27148,7 @@
     <row r="125" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A125" s="6">
         <f t="shared" si="6"/>
-        <v>19.0267917574383</v>
+        <v>18.813916941274655</v>
       </c>
       <c r="B125" s="18">
         <v>193</v>
@@ -27253,7 +27251,7 @@
       </c>
       <c r="AI125" s="6">
         <f t="shared" si="7"/>
-        <v>0.49512480000000014</v>
+        <v>0.54680160000000011</v>
       </c>
       <c r="AJ125" s="6">
         <f t="shared" si="8"/>
@@ -27275,7 +27273,7 @@
     <row r="126" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A126" s="6">
         <f t="shared" si="6"/>
-        <v>19.010634307201048</v>
+        <v>18.55886118026276</v>
       </c>
       <c r="B126" s="18">
         <v>61</v>
@@ -27378,7 +27376,7 @@
       </c>
       <c r="AI126" s="6">
         <f t="shared" si="7"/>
-        <v>0.43319400000000008</v>
+        <v>0.4582440000000001</v>
       </c>
       <c r="AJ126" s="6">
         <f t="shared" si="8"/>
@@ -27400,7 +27398,7 @@
     <row r="127" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A127" s="6">
         <f t="shared" si="6"/>
-        <v>17.015352144200062</v>
+        <v>16.453281193789298</v>
       </c>
       <c r="B127" s="18">
         <v>179</v>
@@ -27503,7 +27501,7 @@
       </c>
       <c r="AI127" s="6">
         <f t="shared" si="7"/>
-        <v>0.71644240000000026</v>
+        <v>0.72132720000000028</v>
       </c>
       <c r="AJ127" s="6">
         <f t="shared" si="8"/>
@@ -27525,7 +27523,7 @@
     <row r="128" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A128" s="6">
         <f t="shared" si="6"/>
-        <v>18.900312751798019</v>
+        <v>18.322664297123449</v>
       </c>
       <c r="B128" s="20">
         <v>52</v>
@@ -27628,7 +27626,7 @@
       </c>
       <c r="AI128" s="6">
         <f t="shared" si="7"/>
-        <v>0.36460880000000007</v>
+        <v>0.37522600000000006</v>
       </c>
       <c r="AJ128" s="6">
         <f t="shared" si="8"/>
@@ -27650,7 +27648,7 @@
     <row r="129" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A129" s="6">
         <f t="shared" si="6"/>
-        <v>18.949831090154881</v>
+        <v>18.538266875800435</v>
       </c>
       <c r="B129" s="18">
         <v>125</v>
@@ -27753,7 +27751,7 @@
       </c>
       <c r="AI129" s="6">
         <f t="shared" si="7"/>
-        <v>0.71071680000000015</v>
+        <v>0.73999680000000012</v>
       </c>
       <c r="AJ129" s="6">
         <f t="shared" si="8"/>
@@ -27775,7 +27773,7 @@
     <row r="130" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A130" s="6">
         <f t="shared" si="6"/>
-        <v>18.547702706735507</v>
+        <v>18.363690443641808</v>
       </c>
       <c r="B130" s="18">
         <v>17</v>
@@ -27878,7 +27876,7 @@
       </c>
       <c r="AI130" s="6">
         <f t="shared" si="7"/>
-        <v>0.47585280000000013</v>
+        <v>0.52884160000000013</v>
       </c>
       <c r="AJ130" s="6">
         <f t="shared" si="8"/>
@@ -27900,7 +27898,7 @@
     <row r="131" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A131" s="6">
         <f t="shared" si="6"/>
-        <v>20.359881524366585</v>
+        <v>20.172949649604995</v>
       </c>
       <c r="B131" s="20">
         <v>178</v>
@@ -28003,7 +28001,7 @@
       </c>
       <c r="AI131" s="6">
         <f t="shared" si="7"/>
-        <v>1.0902192000000004</v>
+        <v>1.1500596000000003</v>
       </c>
       <c r="AJ131" s="6">
         <f t="shared" si="8"/>
@@ -28025,7 +28023,7 @@
     <row r="132" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A132" s="6">
         <f t="shared" si="6"/>
-        <v>17.940330508221667</v>
+        <v>17.571195228296371</v>
       </c>
       <c r="B132" s="18">
         <v>93</v>
@@ -28128,7 +28126,7 @@
       </c>
       <c r="AI132" s="6">
         <f t="shared" si="7"/>
-        <v>0.79655400000000021</v>
+        <v>0.82655400000000023</v>
       </c>
       <c r="AJ132" s="6">
         <f t="shared" si="8"/>
@@ -28150,7 +28148,7 @@
     <row r="133" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A133" s="6">
         <f t="shared" si="6"/>
-        <v>19.207620490017607</v>
+        <v>18.631305455225704</v>
       </c>
       <c r="B133" s="18">
         <v>95</v>
@@ -28253,7 +28251,7 @@
       </c>
       <c r="AI133" s="6">
         <f t="shared" si="7"/>
-        <v>0.26733480000000009</v>
+        <v>0.2793172000000001</v>
       </c>
       <c r="AJ133" s="6">
         <f t="shared" si="8"/>
@@ -28275,7 +28273,7 @@
     <row r="134" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A134" s="6">
         <f t="shared" si="6"/>
-        <v>18.53377779104121</v>
+        <v>18.060314995754961</v>
       </c>
       <c r="B134" s="18">
         <v>151</v>
@@ -28378,7 +28376,7 @@
       </c>
       <c r="AI134" s="6">
         <f t="shared" si="7"/>
-        <v>0.24687960000000003</v>
+        <v>0.26762960000000002</v>
       </c>
       <c r="AJ134" s="6">
         <f t="shared" si="8"/>
@@ -28400,7 +28398,7 @@
     <row r="135" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A135" s="6">
         <f t="shared" ref="A135:A198" si="12">(AI135*H$3+AJ135*M$3+AK135*W$3+AL135*AB$3+AM135*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>18.629672923692141</v>
+        <v>18.535581569366695</v>
       </c>
       <c r="B135" s="18">
         <v>133</v>
@@ -28503,7 +28501,7 @@
       </c>
       <c r="AI135" s="6">
         <f t="shared" ref="AI135:AI198" si="13">H$1*((-2*10^-6)*H135^3+0.00032*H135^2-0.0021*H135)+I$1*((-2*10^-6)*I135^3+0.00032*I135^2-0.0021*I135)+J$1*((-2*10^-6)*J135^3+0.00032*J135^2-0.0021*J135)+K$1*((-2*10^-6)*K135^3+0.00032*K135^2-0.0021*K135)+L$1*((-2*10^-6)*L135^3+0.00032*L135^2-0.0021*L135)</f>
-        <v>0.2922340000000001</v>
+        <v>0.35554560000000007</v>
       </c>
       <c r="AJ135" s="6">
         <f t="shared" ref="AJ135:AJ198" si="14">(M$1*M135+N$1*N135+O$1*O135)/100</f>
@@ -28525,7 +28523,7 @@
     <row r="136" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A136" s="6">
         <f t="shared" si="12"/>
-        <v>17.889171267420689</v>
+        <v>17.379581108888662</v>
       </c>
       <c r="B136" s="20">
         <v>96</v>
@@ -28628,7 +28626,7 @@
       </c>
       <c r="AI136" s="6">
         <f t="shared" si="13"/>
-        <v>0.4731588000000001</v>
+        <v>0.48733920000000008</v>
       </c>
       <c r="AJ136" s="6">
         <f t="shared" si="14"/>
@@ -28650,7 +28648,7 @@
     <row r="137" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A137" s="6">
         <f t="shared" si="12"/>
-        <v>17.854923751827865</v>
+        <v>17.533381491661029</v>
       </c>
       <c r="B137" s="18">
         <v>63</v>
@@ -28753,7 +28751,7 @@
       </c>
       <c r="AI137" s="6">
         <f t="shared" si="13"/>
-        <v>0.6585504000000002</v>
+        <v>0.69350400000000012</v>
       </c>
       <c r="AJ137" s="6">
         <f t="shared" si="14"/>
@@ -28775,7 +28773,7 @@
     <row r="138" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="6">
         <f t="shared" si="12"/>
-        <v>17.163295383329846</v>
+        <v>16.851866087231802</v>
       </c>
       <c r="B138" s="18">
         <v>101</v>
@@ -28878,7 +28876,7 @@
       </c>
       <c r="AI138" s="6">
         <f t="shared" si="13"/>
-        <v>0.41785280000000002</v>
+        <v>0.45119200000000004</v>
       </c>
       <c r="AJ138" s="6">
         <f t="shared" si="14"/>
@@ -28900,7 +28898,7 @@
     <row r="139" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A139" s="6">
         <f t="shared" si="12"/>
-        <v>17.651764600555072</v>
+        <v>17.062592059631903</v>
       </c>
       <c r="B139" s="20">
         <v>22</v>
@@ -29003,7 +29001,7 @@
       </c>
       <c r="AI139" s="6">
         <f t="shared" si="13"/>
-        <v>0.14823680000000006</v>
+        <v>0.15262840000000005</v>
       </c>
       <c r="AJ139" s="6">
         <f t="shared" si="14"/>
@@ -29025,7 +29023,7 @@
     <row r="140" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A140" s="6">
         <f t="shared" si="12"/>
-        <v>17.19819451490644</v>
+        <v>16.795311758018787</v>
       </c>
       <c r="B140" s="20">
         <v>110</v>
@@ -29128,7 +29126,7 @@
       </c>
       <c r="AI140" s="6">
         <f t="shared" si="13"/>
-        <v>0.74547479999999999</v>
+        <v>0.76878360000000012</v>
       </c>
       <c r="AJ140" s="6">
         <f t="shared" si="14"/>
@@ -29150,7 +29148,7 @@
     <row r="141" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A141" s="6">
         <f t="shared" si="12"/>
-        <v>17.281182070488523</v>
+        <v>16.973231260702512</v>
       </c>
       <c r="B141" s="20">
         <v>136</v>
@@ -29253,7 +29251,7 @@
       </c>
       <c r="AI141" s="6">
         <f t="shared" si="13"/>
-        <v>0.59553560000000016</v>
+        <v>0.62972840000000008</v>
       </c>
       <c r="AJ141" s="6">
         <f t="shared" si="14"/>
@@ -29275,7 +29273,7 @@
     <row r="142" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A142" s="6">
         <f t="shared" si="12"/>
-        <v>16.242026172073171</v>
+        <v>15.963318032032001</v>
       </c>
       <c r="B142" s="20">
         <v>88</v>
@@ -29378,7 +29376,7 @@
       </c>
       <c r="AI142" s="6">
         <f t="shared" si="13"/>
-        <v>0.62736600000000009</v>
+        <v>0.66069520000000015</v>
       </c>
       <c r="AJ142" s="6">
         <f t="shared" si="14"/>
@@ -29400,7 +29398,7 @@
     <row r="143" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A143" s="6">
         <f t="shared" si="12"/>
-        <v>17.066101345907065</v>
+        <v>16.491603183054401</v>
       </c>
       <c r="B143" s="20">
         <v>158</v>
@@ -29503,7 +29501,7 @@
       </c>
       <c r="AI143" s="6">
         <f t="shared" si="13"/>
-        <v>0.14952280000000007</v>
+        <v>0.15322680000000005</v>
       </c>
       <c r="AJ143" s="6">
         <f t="shared" si="14"/>
@@ -29525,7 +29523,7 @@
     <row r="144" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A144" s="6">
         <f t="shared" si="12"/>
-        <v>16.188242412486193</v>
+        <v>15.980557466219617</v>
       </c>
       <c r="B144" s="20">
         <v>74</v>
@@ -29628,7 +29626,7 @@
       </c>
       <c r="AI144" s="6">
         <f t="shared" si="13"/>
-        <v>0.73074680000000014</v>
+        <v>0.77176000000000011</v>
       </c>
       <c r="AJ144" s="6">
         <f t="shared" si="14"/>
@@ -29650,7 +29648,7 @@
     <row r="145" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A145" s="6">
         <f t="shared" si="12"/>
-        <v>16.481303978035754</v>
+        <v>16.209359647734303</v>
       </c>
       <c r="B145" s="20">
         <v>126</v>
@@ -29753,7 +29751,7 @@
       </c>
       <c r="AI145" s="6">
         <f t="shared" si="13"/>
-        <v>0.5020300000000002</v>
+        <v>0.53705880000000017</v>
       </c>
       <c r="AJ145" s="6">
         <f t="shared" si="14"/>
@@ -29775,7 +29773,7 @@
     <row r="146" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A146" s="6">
         <f t="shared" si="12"/>
-        <v>16.620946312930851</v>
+        <v>16.234172218784625</v>
       </c>
       <c r="B146" s="18">
         <v>173</v>
@@ -29878,7 +29876,7 @@
       </c>
       <c r="AI146" s="6">
         <f t="shared" si="13"/>
-        <v>0.61509400000000014</v>
+        <v>0.63790800000000014</v>
       </c>
       <c r="AJ146" s="6">
         <f t="shared" si="14"/>
@@ -29900,7 +29898,7 @@
     <row r="147" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A147" s="6">
         <f t="shared" si="12"/>
-        <v>16.826596138350887</v>
+        <v>16.353756061761612</v>
       </c>
       <c r="B147" s="18">
         <v>35</v>
@@ -30003,7 +30001,7 @@
       </c>
       <c r="AI147" s="6">
         <f t="shared" si="13"/>
-        <v>0.14326720000000001</v>
+        <v>0.15732600000000005</v>
       </c>
       <c r="AJ147" s="6">
         <f t="shared" si="14"/>
@@ -30025,7 +30023,7 @@
     <row r="148" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A148" s="6">
         <f t="shared" si="12"/>
-        <v>16.634447163448623</v>
+        <v>16.042009698818585</v>
       </c>
       <c r="B148" s="18">
         <v>159</v>
@@ -30150,7 +30148,7 @@
     <row r="149" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A149" s="6">
         <f t="shared" si="12"/>
-        <v>16.307627950699811</v>
+        <v>16.175004820629411</v>
       </c>
       <c r="B149" s="20">
         <v>20</v>
@@ -30253,7 +30251,7 @@
       </c>
       <c r="AI149" s="6">
         <f t="shared" si="13"/>
-        <v>0.34971440000000015</v>
+        <v>0.39954640000000013</v>
       </c>
       <c r="AJ149" s="6">
         <f t="shared" si="14"/>
@@ -30275,7 +30273,7 @@
     <row r="150" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A150" s="6">
         <f t="shared" si="12"/>
-        <v>17.04584231102092</v>
+        <v>17.517210510411118</v>
       </c>
       <c r="B150" s="18">
         <v>177</v>
@@ -30378,7 +30376,7 @@
       </c>
       <c r="AI150" s="6">
         <f t="shared" si="13"/>
-        <v>0.50149480000000024</v>
+        <v>0.62140720000000016</v>
       </c>
       <c r="AJ150" s="6">
         <f t="shared" si="14"/>
@@ -30400,7 +30398,7 @@
     <row r="151" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A151" s="6">
         <f t="shared" si="12"/>
-        <v>15.813078874332271</v>
+        <v>15.573668139237045</v>
       </c>
       <c r="B151" s="18">
         <v>3</v>
@@ -30503,7 +30501,7 @@
       </c>
       <c r="AI151" s="6">
         <f t="shared" si="13"/>
-        <v>0.20153760000000001</v>
+        <v>0.23753760000000004</v>
       </c>
       <c r="AJ151" s="6">
         <f t="shared" si="14"/>
@@ -30525,7 +30523,7 @@
     <row r="152" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A152" s="6">
         <f t="shared" si="12"/>
-        <v>15.025219940911395</v>
+        <v>14.856380354855885</v>
       </c>
       <c r="B152" s="18">
         <v>53</v>
@@ -30628,7 +30626,7 @@
       </c>
       <c r="AI152" s="6">
         <f t="shared" si="13"/>
-        <v>0.27023160000000013</v>
+        <v>0.31095840000000008</v>
       </c>
       <c r="AJ152" s="6">
         <f t="shared" si="14"/>
@@ -30650,7 +30648,7 @@
     <row r="153" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A153" s="6">
         <f t="shared" si="12"/>
-        <v>14.997102121818017</v>
+        <v>14.87668959463543</v>
       </c>
       <c r="B153" s="20">
         <v>76</v>
@@ -30753,7 +30751,7 @@
       </c>
       <c r="AI153" s="6">
         <f t="shared" si="13"/>
-        <v>0.4948140000000002</v>
+        <v>0.54081400000000013</v>
       </c>
       <c r="AJ153" s="6">
         <f t="shared" si="14"/>
@@ -30775,7 +30773,7 @@
     <row r="154" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A154" s="6">
         <f t="shared" si="12"/>
-        <v>15.286872332806109</v>
+        <v>15.05746780251248</v>
       </c>
       <c r="B154" s="20">
         <v>146</v>
@@ -30878,7 +30876,7 @@
       </c>
       <c r="AI154" s="6">
         <f t="shared" si="13"/>
-        <v>0.17703560000000004</v>
+        <v>0.21206440000000007</v>
       </c>
       <c r="AJ154" s="6">
         <f t="shared" si="14"/>
@@ -30900,7 +30898,7 @@
     <row r="155" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A155" s="6">
         <f t="shared" si="12"/>
-        <v>14.978774508341036</v>
+        <v>14.556074136963428</v>
       </c>
       <c r="B155" s="20">
         <v>82</v>
@@ -31003,7 +31001,7 @@
       </c>
       <c r="AI155" s="6">
         <f t="shared" si="13"/>
-        <v>0.38768360000000002</v>
+        <v>0.4</v>
       </c>
       <c r="AJ155" s="6">
         <f t="shared" si="14"/>
@@ -31025,7 +31023,7 @@
     <row r="156" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A156" s="6">
         <f t="shared" si="12"/>
-        <v>14.918303739293917</v>
+        <v>14.58889211863065</v>
       </c>
       <c r="B156" s="18">
         <v>121</v>
@@ -31128,7 +31126,7 @@
       </c>
       <c r="AI156" s="6">
         <f t="shared" si="13"/>
-        <v>0.42554760000000008</v>
+        <v>0.4479972000000001</v>
       </c>
       <c r="AJ156" s="6">
         <f t="shared" si="14"/>
@@ -31150,7 +31148,7 @@
     <row r="157" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A157" s="6">
         <f t="shared" si="12"/>
-        <v>14.751632844907336</v>
+        <v>14.546701538284427</v>
       </c>
       <c r="B157" s="20">
         <v>70</v>
@@ -31253,7 +31251,7 @@
       </c>
       <c r="AI157" s="6">
         <f t="shared" si="13"/>
-        <v>0.2960484000000001</v>
+        <v>0.33167880000000005</v>
       </c>
       <c r="AJ157" s="6">
         <f t="shared" si="14"/>
@@ -31275,7 +31273,7 @@
     <row r="158" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A158" s="6">
         <f t="shared" si="12"/>
-        <v>15.056213852994714</v>
+        <v>14.583560070798494</v>
       </c>
       <c r="B158" s="20">
         <v>116</v>
@@ -31378,7 +31376,7 @@
       </c>
       <c r="AI158" s="6">
         <f t="shared" si="13"/>
-        <v>0.2918092000000001</v>
+        <v>0.29887800000000009</v>
       </c>
       <c r="AJ158" s="6">
         <f t="shared" si="14"/>
@@ -31400,7 +31398,7 @@
     <row r="159" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A159" s="6">
         <f t="shared" si="12"/>
-        <v>14.630422871467363</v>
+        <v>14.590785115047556</v>
       </c>
       <c r="B159" s="20">
         <v>16</v>
@@ -31503,7 +31501,7 @@
       </c>
       <c r="AI159" s="6">
         <f t="shared" si="13"/>
-        <v>0.5707928000000001</v>
+        <v>0.62432200000000015</v>
       </c>
       <c r="AJ159" s="6">
         <f t="shared" si="14"/>
@@ -31525,7 +31523,7 @@
     <row r="160" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A160" s="6">
         <f t="shared" si="12"/>
-        <v>13.43037094511922</v>
+        <v>13.012754522038188</v>
       </c>
       <c r="B160" s="18">
         <v>181</v>
@@ -31628,7 +31626,7 @@
       </c>
       <c r="AI160" s="6">
         <f t="shared" si="13"/>
-        <v>0.48338760000000003</v>
+        <v>0.49013760000000006</v>
       </c>
       <c r="AJ160" s="6">
         <f t="shared" si="14"/>
@@ -31650,7 +31648,7 @@
     <row r="161" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A161" s="6">
         <f t="shared" si="12"/>
-        <v>15.28738503088722</v>
+        <v>15.197713726562384</v>
       </c>
       <c r="B161" s="18">
         <v>65</v>
@@ -31753,7 +31751,7 @@
       </c>
       <c r="AI161" s="6">
         <f t="shared" si="13"/>
-        <v>0.42905520000000003</v>
+        <v>0.47962280000000007</v>
       </c>
       <c r="AJ161" s="6">
         <f t="shared" si="14"/>
@@ -31775,7 +31773,7 @@
     <row r="162" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A162" s="6">
         <f t="shared" si="12"/>
-        <v>15.127650034319135</v>
+        <v>14.730977940224193</v>
       </c>
       <c r="B162" s="20">
         <v>64</v>
@@ -31878,7 +31876,7 @@
       </c>
       <c r="AI162" s="6">
         <f t="shared" si="13"/>
-        <v>0.33982640000000008</v>
+        <v>0.35562640000000012</v>
       </c>
       <c r="AJ162" s="6">
         <f t="shared" si="14"/>
@@ -31900,7 +31898,7 @@
     <row r="163" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A163" s="6">
         <f t="shared" si="12"/>
-        <v>13.986965442120026</v>
+        <v>13.565775689637801</v>
       </c>
       <c r="B163" s="20">
         <v>168</v>
@@ -32003,7 +32001,7 @@
       </c>
       <c r="AI163" s="6">
         <f t="shared" si="13"/>
-        <v>0.20062480000000005</v>
+        <v>0.20918160000000002</v>
       </c>
       <c r="AJ163" s="6">
         <f t="shared" si="14"/>
@@ -32025,7 +32023,7 @@
     <row r="164" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A164" s="6">
         <f t="shared" si="12"/>
-        <v>14.694966277716432</v>
+        <v>14.529761990416297</v>
       </c>
       <c r="B164" s="20">
         <v>38</v>
@@ -32128,7 +32126,7 @@
       </c>
       <c r="AI164" s="6">
         <f t="shared" si="13"/>
-        <v>0.38960280000000003</v>
+        <v>0.42942600000000009</v>
       </c>
       <c r="AJ164" s="6">
         <f t="shared" si="14"/>
@@ -32150,7 +32148,7 @@
     <row r="165" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A165" s="6">
         <f t="shared" si="12"/>
-        <v>14.274481333373124</v>
+        <v>14.199591181845651</v>
       </c>
       <c r="B165" s="18">
         <v>163</v>
@@ -32253,7 +32251,7 @@
       </c>
       <c r="AI165" s="6">
         <f t="shared" si="13"/>
-        <v>0.60440640000000023</v>
+        <v>0.65260640000000025</v>
       </c>
       <c r="AJ165" s="6">
         <f t="shared" si="14"/>
@@ -32275,7 +32273,7 @@
     <row r="166" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A166" s="6">
         <f t="shared" si="12"/>
-        <v>14.567267898176606</v>
+        <v>14.255697120573291</v>
       </c>
       <c r="B166" s="20">
         <v>100</v>
@@ -32378,7 +32376,7 @@
       </c>
       <c r="AI166" s="6">
         <f t="shared" si="13"/>
-        <v>0.46874720000000009</v>
+        <v>0.49179040000000007</v>
       </c>
       <c r="AJ166" s="6">
         <f t="shared" si="14"/>
@@ -32400,7 +32398,7 @@
     <row r="167" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A167" s="6">
         <f t="shared" si="12"/>
-        <v>14.441133426840548</v>
+        <v>13.926811045716832</v>
       </c>
       <c r="B167" s="18">
         <v>115</v>
@@ -32525,7 +32523,7 @@
     <row r="168" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A168" s="6">
         <f t="shared" si="12"/>
-        <v>14.097046912769699</v>
+        <v>13.590032665160514</v>
       </c>
       <c r="B168" s="20">
         <v>122</v>
@@ -32628,7 +32626,7 @@
       </c>
       <c r="AI168" s="6">
         <f t="shared" si="13"/>
-        <v>0.8037084000000001</v>
+        <v>0.80315840000000005</v>
       </c>
       <c r="AJ168" s="6">
         <f t="shared" si="14"/>
@@ -32650,7 +32648,7 @@
     <row r="169" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A169" s="6">
         <f t="shared" si="12"/>
-        <v>14.28922080635053</v>
+        <v>14.080151957751138</v>
       </c>
       <c r="B169" s="18">
         <v>37</v>
@@ -32753,7 +32751,7 @@
       </c>
       <c r="AI169" s="6">
         <f t="shared" si="13"/>
-        <v>0.69917040000000008</v>
+        <v>0.73250960000000009</v>
       </c>
       <c r="AJ169" s="6">
         <f t="shared" si="14"/>
@@ -32775,7 +32773,7 @@
     <row r="170" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A170" s="6">
         <f t="shared" si="12"/>
-        <v>14.18821376346653</v>
+        <v>14.137689551465613</v>
       </c>
       <c r="B170" s="20">
         <v>6</v>
@@ -32878,7 +32876,7 @@
       </c>
       <c r="AI170" s="6">
         <f t="shared" si="13"/>
-        <v>0.39645040000000004</v>
+        <v>0.44701800000000008</v>
       </c>
       <c r="AJ170" s="6">
         <f t="shared" si="14"/>
@@ -32900,7 +32898,7 @@
     <row r="171" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A171" s="6">
         <f t="shared" si="12"/>
-        <v>13.854752156137156</v>
+        <v>13.854939058610219</v>
       </c>
       <c r="B171" s="18">
         <v>19</v>
@@ -33003,7 +33001,7 @@
       </c>
       <c r="AI171" s="6">
         <f t="shared" si="13"/>
-        <v>0.36264200000000008</v>
+        <v>0.41752760000000011</v>
       </c>
       <c r="AJ171" s="6">
         <f t="shared" si="14"/>
@@ -33025,7 +33023,7 @@
     <row r="172" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A172" s="6">
         <f t="shared" si="12"/>
-        <v>13.426288907457696</v>
+        <v>13.595513648856718</v>
       </c>
       <c r="B172" s="18">
         <v>137</v>
@@ -33128,7 +33126,7 @@
       </c>
       <c r="AI172" s="6">
         <f t="shared" si="13"/>
-        <v>0.74857760000000018</v>
+        <v>0.82056160000000022</v>
       </c>
       <c r="AJ172" s="6">
         <f t="shared" si="14"/>
@@ -33150,7 +33148,7 @@
     <row r="173" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A173" s="6">
         <f t="shared" si="12"/>
-        <v>13.642244620848128</v>
+        <v>13.468496107521617</v>
       </c>
       <c r="B173" s="20">
         <v>154</v>
@@ -33253,7 +33251,7 @@
       </c>
       <c r="AI173" s="6">
         <f t="shared" si="13"/>
-        <v>0.18676600000000007</v>
+        <v>0.22147040000000004</v>
       </c>
       <c r="AJ173" s="6">
         <f t="shared" si="14"/>
@@ -33275,7 +33273,7 @@
     <row r="174" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A174" s="6">
         <f t="shared" si="12"/>
-        <v>13.951376794294067</v>
+        <v>13.742867914754003</v>
       </c>
       <c r="B174" s="18">
         <v>135</v>
@@ -33378,7 +33376,7 @@
       </c>
       <c r="AI174" s="6">
         <f t="shared" si="13"/>
-        <v>0.37277680000000007</v>
+        <v>0.40484040000000004</v>
       </c>
       <c r="AJ174" s="6">
         <f t="shared" si="14"/>
@@ -33400,7 +33398,7 @@
     <row r="175" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A175" s="6">
         <f t="shared" si="12"/>
-        <v>13.194436718493536</v>
+        <v>13.448959031844932</v>
       </c>
       <c r="B175" s="18">
         <v>79</v>
@@ -33503,7 +33501,7 @@
       </c>
       <c r="AI175" s="6">
         <f t="shared" si="13"/>
-        <v>0.56366880000000008</v>
+        <v>0.64421880000000009</v>
       </c>
       <c r="AJ175" s="6">
         <f t="shared" si="14"/>
@@ -33525,7 +33523,7 @@
     <row r="176" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A176" s="6">
         <f t="shared" si="12"/>
-        <v>13.47523322092572</v>
+        <v>13.343648712819993</v>
       </c>
       <c r="B176" s="20">
         <v>166</v>
@@ -33628,7 +33626,7 @@
       </c>
       <c r="AI176" s="6">
         <f t="shared" si="13"/>
-        <v>0.17483760000000004</v>
+        <v>0.21356880000000003</v>
       </c>
       <c r="AJ176" s="6">
         <f t="shared" si="14"/>
@@ -33650,7 +33648,7 @@
     <row r="177" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A177" s="6">
         <f t="shared" si="12"/>
-        <v>13.2499279298099</v>
+        <v>13.150755040075975</v>
       </c>
       <c r="B177" s="20">
         <v>50</v>
@@ -33753,7 +33751,7 @@
       </c>
       <c r="AI177" s="6">
         <f t="shared" si="13"/>
-        <v>0.46526240000000008</v>
+        <v>0.50670520000000008</v>
       </c>
       <c r="AJ177" s="6">
         <f t="shared" si="14"/>
@@ -33775,7 +33773,7 @@
     <row r="178" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A178" s="6">
         <f t="shared" si="12"/>
-        <v>12.75139216329941</v>
+        <v>12.387579324536283</v>
       </c>
       <c r="B178" s="20">
         <v>112</v>
@@ -33878,7 +33876,7 @@
       </c>
       <c r="AI178" s="6">
         <f t="shared" si="13"/>
-        <v>0.40732480000000015</v>
+        <v>0.41736840000000014</v>
       </c>
       <c r="AJ178" s="6">
         <f t="shared" si="14"/>
@@ -33900,7 +33898,7 @@
     <row r="179" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A179" s="6">
         <f t="shared" si="12"/>
-        <v>13.513182577814913</v>
+        <v>13.307523347675303</v>
       </c>
       <c r="B179" s="18">
         <v>45</v>
@@ -34003,7 +34001,7 @@
       </c>
       <c r="AI179" s="6">
         <f t="shared" si="13"/>
-        <v>0.38200680000000004</v>
+        <v>0.41265200000000007</v>
       </c>
       <c r="AJ179" s="6">
         <f t="shared" si="14"/>
@@ -34025,7 +34023,7 @@
     <row r="180" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A180" s="6">
         <f t="shared" si="12"/>
-        <v>12.199195738458322</v>
+        <v>12.081313225792524</v>
       </c>
       <c r="B180" s="18">
         <v>119</v>
@@ -34128,7 +34126,7 @@
       </c>
       <c r="AI180" s="6">
         <f t="shared" si="13"/>
-        <v>0.58797840000000012</v>
+        <v>0.62318000000000007</v>
       </c>
       <c r="AJ180" s="6">
         <f t="shared" si="14"/>
@@ -34150,7 +34148,7 @@
     <row r="181" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A181" s="6">
         <f t="shared" si="12"/>
-        <v>12.654398072159717</v>
+        <v>12.38568920610709</v>
       </c>
       <c r="B181" s="18">
         <v>107</v>
@@ -34253,7 +34251,7 @@
       </c>
       <c r="AI181" s="6">
         <f t="shared" si="13"/>
-        <v>0.43921720000000009</v>
+        <v>0.45945120000000006</v>
       </c>
       <c r="AJ181" s="6">
         <f t="shared" si="14"/>
@@ -34275,7 +34273,7 @@
     <row r="182" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A182" s="6">
         <f t="shared" si="12"/>
-        <v>12.615742934733952</v>
+        <v>12.216494610968009</v>
       </c>
       <c r="B182" s="18">
         <v>131</v>
@@ -34378,7 +34376,7 @@
       </c>
       <c r="AI182" s="6">
         <f t="shared" si="13"/>
-        <v>1.7568000000000011E-2</v>
+        <v>2.3134400000000013E-2</v>
       </c>
       <c r="AJ182" s="6">
         <f t="shared" si="14"/>
@@ -34400,7 +34398,7 @@
     <row r="183" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A183" s="6">
         <f t="shared" si="12"/>
-        <v>12.599458802112862</v>
+        <v>12.714773862115605</v>
       </c>
       <c r="B183" s="18">
         <v>99</v>
@@ -34503,7 +34501,7 @@
       </c>
       <c r="AI183" s="6">
         <f t="shared" si="13"/>
-        <v>0.52176240000000007</v>
+        <v>0.58447800000000005</v>
       </c>
       <c r="AJ183" s="6">
         <f t="shared" si="14"/>
@@ -34525,7 +34523,7 @@
     <row r="184" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A184" s="6">
         <f t="shared" si="12"/>
-        <v>11.809287057208511</v>
+        <v>11.688451354812713</v>
       </c>
       <c r="B184" s="18">
         <v>87</v>
@@ -34628,7 +34626,7 @@
       </c>
       <c r="AI184" s="6">
         <f t="shared" si="13"/>
-        <v>0.45561200000000013</v>
+        <v>0.48894120000000019</v>
       </c>
       <c r="AJ184" s="6">
         <f t="shared" si="14"/>
@@ -34650,7 +34648,7 @@
     <row r="185" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A185" s="6">
         <f t="shared" si="12"/>
-        <v>11.367810588200184</v>
+        <v>11.297960657907987</v>
       </c>
       <c r="B185" s="18">
         <v>23</v>
@@ -34753,7 +34751,7 @@
       </c>
       <c r="AI185" s="6">
         <f t="shared" si="13"/>
-        <v>0.46860920000000017</v>
+        <v>0.50585920000000018</v>
       </c>
       <c r="AJ185" s="6">
         <f t="shared" si="14"/>
@@ -34775,7 +34773,7 @@
     <row r="186" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A186" s="6">
         <f t="shared" si="12"/>
-        <v>12.263833895371389</v>
+        <v>12.050960096700381</v>
       </c>
       <c r="B186" s="20">
         <v>152</v>
@@ -34878,7 +34876,7 @@
       </c>
       <c r="AI186" s="6">
         <f t="shared" si="13"/>
-        <v>0.50145480000000009</v>
+        <v>0.52635040000000011</v>
       </c>
       <c r="AJ186" s="6">
         <f t="shared" si="14"/>
@@ -34900,7 +34898,7 @@
     <row r="187" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A187" s="6">
         <f t="shared" si="12"/>
-        <v>11.90084962248948</v>
+        <v>11.638408041097662</v>
       </c>
       <c r="B187" s="20">
         <v>164</v>
@@ -35003,7 +35001,7 @@
       </c>
       <c r="AI187" s="6">
         <f t="shared" si="13"/>
-        <v>0.17054600000000003</v>
+        <v>0.18849280000000004</v>
       </c>
       <c r="AJ187" s="6">
         <f t="shared" si="14"/>
@@ -35025,7 +35023,7 @@
     <row r="188" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A188" s="6">
         <f t="shared" si="12"/>
-        <v>11.750657435315883</v>
+        <v>11.453506971925226</v>
       </c>
       <c r="B188" s="20">
         <v>172</v>
@@ -35128,7 +35126,7 @@
       </c>
       <c r="AI188" s="6">
         <f t="shared" si="13"/>
-        <v>0.13986360000000006</v>
+        <v>0.15335640000000009</v>
       </c>
       <c r="AJ188" s="6">
         <f t="shared" si="14"/>
@@ -35150,7 +35148,7 @@
     <row r="189" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A189" s="6">
         <f t="shared" si="12"/>
-        <v>12.316603002178519</v>
+        <v>12.160341329342522</v>
       </c>
       <c r="B189" s="18">
         <v>111</v>
@@ -35253,7 +35251,7 @@
       </c>
       <c r="AI189" s="6">
         <f t="shared" si="13"/>
-        <v>0.42922920000000009</v>
+        <v>0.4606284000000001</v>
       </c>
       <c r="AJ189" s="6">
         <f t="shared" si="14"/>
@@ -35275,7 +35273,7 @@
     <row r="190" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A190" s="6">
         <f t="shared" si="12"/>
-        <v>11.79908382822525</v>
+        <v>12.186576345819001</v>
       </c>
       <c r="B190" s="18">
         <v>165</v>
@@ -35378,7 +35376,7 @@
       </c>
       <c r="AI190" s="6">
         <f t="shared" si="13"/>
-        <v>0.44943240000000012</v>
+        <v>0.5392416000000001</v>
       </c>
       <c r="AJ190" s="6">
         <f t="shared" si="14"/>
@@ -35400,7 +35398,7 @@
     <row r="191" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A191" s="6">
         <f t="shared" si="12"/>
-        <v>11.455953773613059</v>
+        <v>11.405596391003407</v>
       </c>
       <c r="B191" s="20">
         <v>132</v>
@@ -35503,7 +35501,7 @@
       </c>
       <c r="AI191" s="6">
         <f t="shared" si="13"/>
-        <v>0.16873120000000005</v>
+        <v>0.20849760000000009</v>
       </c>
       <c r="AJ191" s="6">
         <f t="shared" si="14"/>
@@ -35525,7 +35523,7 @@
     <row r="192" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A192" s="6">
         <f t="shared" si="12"/>
-        <v>10.992880867826553</v>
+        <v>10.949705581857163</v>
       </c>
       <c r="B192" s="18">
         <v>41</v>
@@ -35628,7 +35626,7 @@
       </c>
       <c r="AI192" s="6">
         <f t="shared" si="13"/>
-        <v>0.34400480000000011</v>
+        <v>0.38273600000000013</v>
       </c>
       <c r="AJ192" s="6">
         <f t="shared" si="14"/>
@@ -35650,7 +35648,7 @@
     <row r="193" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A193" s="6">
         <f t="shared" si="12"/>
-        <v>11.328554865856933</v>
+        <v>11.159636078453943</v>
       </c>
       <c r="B193" s="18">
         <v>89</v>
@@ -35753,7 +35751,7 @@
       </c>
       <c r="AI193" s="6">
         <f t="shared" si="13"/>
-        <v>0.19036920000000004</v>
+        <v>0.21644840000000001</v>
       </c>
       <c r="AJ193" s="6">
         <f t="shared" si="14"/>
@@ -35775,7 +35773,7 @@
     <row r="194" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A194" s="6">
         <f t="shared" si="12"/>
-        <v>10.594728878808677</v>
+        <v>10.409081346322647</v>
       </c>
       <c r="B194" s="18">
         <v>123</v>
@@ -35878,7 +35876,7 @@
       </c>
       <c r="AI194" s="6">
         <f t="shared" si="13"/>
-        <v>0.3302172000000001</v>
+        <v>0.35153040000000008</v>
       </c>
       <c r="AJ194" s="6">
         <f t="shared" si="14"/>
@@ -35900,7 +35898,7 @@
     <row r="195" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A195" s="6">
         <f t="shared" si="12"/>
-        <v>11.312678235697868</v>
+        <v>11.439847466651315</v>
       </c>
       <c r="B195" s="18">
         <v>51</v>
@@ -36003,7 +36001,7 @@
       </c>
       <c r="AI195" s="6">
         <f t="shared" si="13"/>
-        <v>0.38655600000000012</v>
+        <v>0.44549400000000011</v>
       </c>
       <c r="AJ195" s="6">
         <f t="shared" si="14"/>
@@ -36025,7 +36023,7 @@
     <row r="196" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A196" s="6">
         <f t="shared" si="12"/>
-        <v>10.706393506222206</v>
+        <v>10.855087274977334</v>
       </c>
       <c r="B196" s="20">
         <v>14</v>
@@ -36128,7 +36126,7 @@
       </c>
       <c r="AI196" s="6">
         <f t="shared" si="13"/>
-        <v>0.61402600000000007</v>
+        <v>0.67295640000000012</v>
       </c>
       <c r="AJ196" s="6">
         <f t="shared" si="14"/>
@@ -36150,7 +36148,7 @@
     <row r="197" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A197" s="6">
         <f t="shared" si="12"/>
-        <v>10.970096839655017</v>
+        <v>10.977536586418775</v>
       </c>
       <c r="B197" s="20">
         <v>162</v>
@@ -36253,7 +36251,7 @@
       </c>
       <c r="AI197" s="6">
         <f t="shared" si="13"/>
-        <v>0.23529560000000008</v>
+        <v>0.27956440000000005</v>
       </c>
       <c r="AJ197" s="6">
         <f t="shared" si="14"/>
@@ -36275,7 +36273,7 @@
     <row r="198" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A198" s="6">
         <f t="shared" si="12"/>
-        <v>10.862664806469903</v>
+        <v>10.644350078425163</v>
       </c>
       <c r="B198" s="20">
         <v>134</v>
@@ -36378,7 +36376,7 @@
       </c>
       <c r="AI198" s="6">
         <f t="shared" si="13"/>
-        <v>0.31639680000000009</v>
+        <v>0.33513880000000007</v>
       </c>
       <c r="AJ198" s="6">
         <f t="shared" si="14"/>
@@ -36400,7 +36398,7 @@
     <row r="199" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A199" s="6">
         <f t="shared" ref="A199:A207" si="18">(AI199*H$3+AJ199*M$3+AK199*W$3+AL199*AB$3+AM199*AD$3)*100/(AI$5*H$3+AJ$5*M$3+AK$5*W$3+AL$5*AB$3+AM$5*AD$3)</f>
-        <v>10.244364648303439</v>
+        <v>10.316277610694602</v>
       </c>
       <c r="B199" s="18">
         <v>127</v>
@@ -36503,7 +36501,7 @@
       </c>
       <c r="AI199" s="6">
         <f t="shared" ref="AI199:AI207" si="19">H$1*((-2*10^-6)*H199^3+0.00032*H199^2-0.0021*H199)+I$1*((-2*10^-6)*I199^3+0.00032*I199^2-0.0021*I199)+J$1*((-2*10^-6)*J199^3+0.00032*J199^2-0.0021*J199)+K$1*((-2*10^-6)*K199^3+0.00032*K199^2-0.0021*K199)+L$1*((-2*10^-6)*L199^3+0.00032*L199^2-0.0021*L199)</f>
-        <v>0.52138480000000009</v>
+        <v>0.56994840000000013</v>
       </c>
       <c r="AJ199" s="6">
         <f t="shared" ref="AJ199:AJ207" si="20">(M$1*M199+N$1*N199+O$1*O199)/100</f>
@@ -36525,7 +36523,7 @@
     <row r="200" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A200" s="6">
         <f t="shared" si="18"/>
-        <v>10.688792861619266</v>
+        <v>10.626246816226095</v>
       </c>
       <c r="B200" s="20">
         <v>106</v>
@@ -36628,7 +36626,7 @@
       </c>
       <c r="AI200" s="6">
         <f t="shared" si="19"/>
-        <v>0.4353512000000001</v>
+        <v>0.4707244000000001</v>
       </c>
       <c r="AJ200" s="6">
         <f t="shared" si="20"/>
@@ -36650,7 +36648,7 @@
     <row r="201" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A201" s="6">
         <f t="shared" si="18"/>
-        <v>10.493818974006981</v>
+        <v>10.232527161009019</v>
       </c>
       <c r="B201" s="18">
         <v>113</v>
@@ -36753,7 +36751,7 @@
       </c>
       <c r="AI201" s="6">
         <f t="shared" si="19"/>
-        <v>0.43459280000000006</v>
+        <v>0.44709560000000009</v>
       </c>
       <c r="AJ201" s="6">
         <f t="shared" si="20"/>
@@ -36775,7 +36773,7 @@
     <row r="202" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A202" s="6">
         <f t="shared" si="18"/>
-        <v>10.676501984541463</v>
+        <v>10.822860719784721</v>
       </c>
       <c r="B202" s="18">
         <v>153</v>
@@ -36878,7 +36876,7 @@
       </c>
       <c r="AI202" s="6">
         <f t="shared" si="19"/>
-        <v>0.39900520000000012</v>
+        <v>0.45755760000000006</v>
       </c>
       <c r="AJ202" s="6">
         <f t="shared" si="20"/>
@@ -36900,7 +36898,7 @@
     <row r="203" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A203" s="6">
         <f t="shared" si="18"/>
-        <v>9.7371204750962406</v>
+        <v>9.4984723641230033</v>
       </c>
       <c r="B203" s="20">
         <v>118</v>
@@ -37003,7 +37001,7 @@
       </c>
       <c r="AI203" s="6">
         <f t="shared" si="19"/>
-        <v>6.847240000000003E-2</v>
+        <v>8.0496400000000037E-2</v>
       </c>
       <c r="AJ203" s="6">
         <f t="shared" si="20"/>
@@ -37025,7 +37023,7 @@
     <row r="204" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A204" s="6">
         <f t="shared" si="18"/>
-        <v>10.106443642006621</v>
+        <v>10.105476666714631</v>
       </c>
       <c r="B204" s="18">
         <v>77</v>
@@ -37128,7 +37126,7 @@
       </c>
       <c r="AI204" s="6">
         <f t="shared" si="19"/>
-        <v>0.36021680000000006</v>
+        <v>0.40013080000000006</v>
       </c>
       <c r="AJ204" s="6">
         <f t="shared" si="20"/>
@@ -37150,7 +37148,7 @@
     <row r="205" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A205" s="6">
         <f t="shared" si="18"/>
-        <v>9.684640544331371</v>
+        <v>9.6872237491545885</v>
       </c>
       <c r="B205" s="18">
         <v>149</v>
@@ -37253,7 +37251,7 @@
       </c>
       <c r="AI205" s="6">
         <f t="shared" si="19"/>
-        <v>0.37557560000000006</v>
+        <v>0.41421400000000008</v>
       </c>
       <c r="AJ205" s="6">
         <f t="shared" si="20"/>
@@ -37275,7 +37273,7 @@
     <row r="206" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A206" s="6">
         <f t="shared" si="18"/>
-        <v>9.1882228654988189</v>
+        <v>9.1593623818226284</v>
       </c>
       <c r="B206" s="18">
         <v>117</v>
@@ -37378,7 +37376,7 @@
       </c>
       <c r="AI206" s="6">
         <f t="shared" si="19"/>
-        <v>0.55998520000000007</v>
+        <v>0.59316160000000018</v>
       </c>
       <c r="AJ206" s="6">
         <f t="shared" si="20"/>
@@ -37400,7 +37398,7 @@
     <row r="207" spans="1:39" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A207" s="6">
         <f t="shared" si="18"/>
-        <v>8.6968869557432313</v>
+        <v>8.88134013497762</v>
       </c>
       <c r="B207" s="20">
         <v>174</v>
@@ -37503,7 +37501,7 @@
       </c>
       <c r="AI207" s="6">
         <f t="shared" si="19"/>
-        <v>0.31070480000000011</v>
+        <v>0.36565360000000002</v>
       </c>
       <c r="AJ207" s="6">
         <f t="shared" si="20"/>

</xml_diff>

<commit_message>
Update amateur draft template for Hardball Dynasty Draft Optimizer
This commit modifies the Season x amateur draft-template.xlsx file, reflecting changes in the draft process. The updates ensure compatibility with recent enhancements in the algorithm and improve data handling for player evaluations. No specific details on the changes are provided due to the binary nature of the file.
</commit_message>
<xml_diff>
--- a/Season x amateur draft-template.xlsx
+++ b/Season x amateur draft-template.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13362ca80da55a94/Documents/hardball-dynasty-draft-optimizer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F4D1FAA-7EEC-4AD7-A890-F7367C1FBE05}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{7F539934-F661-4AA3-BA5B-9B5C3F8FDDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAF8A9A5-5815-4B9A-B6F7-D0A4D79C5A39}"/>
   <bookViews>
-    <workbookView xWindow="-30828" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hitters" sheetId="1" r:id="rId1"/>
     <sheet name="Pitchers" sheetId="3" r:id="rId2"/>
-    <sheet name="Algorithm" sheetId="2" r:id="rId3"/>
+    <sheet name="Algorithm Analysis" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hitters!$A$6:$AM$6</definedName>
@@ -1406,7 +1406,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Algorithm!$A$1:$A$14</c:f>
+              <c:f>'Algorithm Analysis'!$A$1:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -1457,7 +1457,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Algorithm!$B$1:$B$14</c:f>
+              <c:f>'Algorithm Analysis'!$B$1:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -11403,10 +11403,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -73369,9 +73365,9 @@
         <f>MAX(0, (((LOG(A1+0.000001, 100)*2.6-0.92))))</f>
         <v>0</v>
       </c>
-      <c r="E1" t="e">
-        <f ca="1">Hitters!AF2(-2*10^-6)*A1^3+0.00032*A1^2-0.0021*A1</f>
-        <v>#REF!</v>
+      <c r="E1">
+        <f t="shared" ref="E1:E14" si="0">(-2*10^-6)*A1^3+0.00032*A1^2-0.0021*A1</f>
+        <v>0</v>
       </c>
       <c r="G1">
         <f>-2*10^-6*A1^3</f>
@@ -73401,15 +73397,15 @@
         <v>0.05</v>
       </c>
       <c r="C2">
-        <f t="shared" ref="C2:C14" si="0">1/LOG10(111-A2)</f>
+        <f t="shared" ref="C2:C14" si="1">1/LOG10(111-A2)</f>
         <v>0.49892198580547809</v>
       </c>
       <c r="D2">
-        <f t="shared" ref="D2:D14" si="1">MAX(0, (((LOG(A2+0.000001, 100)*2.6-0.92))))</f>
+        <f t="shared" ref="D2:D14" si="2">MAX(0, (((LOG(A2+0.000001, 100)*2.6-0.92))))</f>
         <v>0.38000005645827961</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E14" si="2">(-2*10^-6)*A2^3+0.00032*A2^2-0.0021*A2</f>
+        <f t="shared" si="0"/>
         <v>9.0000000000000011E-3</v>
       </c>
       <c r="G2">
@@ -73440,15 +73436,15 @@
         <v>0.1</v>
       </c>
       <c r="C3">
+        <f t="shared" si="1"/>
+        <v>0.51045373717968723</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="2"/>
+        <v>0.7713390225923159</v>
+      </c>
+      <c r="E3">
         <f t="shared" si="0"/>
-        <v>0.51045373717968723</v>
-      </c>
-      <c r="D3">
-        <f t="shared" si="1"/>
-        <v>0.7713390225923159</v>
-      </c>
-      <c r="E3">
-        <f t="shared" si="2"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G3">
@@ -73483,11 +73479,11 @@
         <v>0.51298098204632536</v>
       </c>
       <c r="D4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.82514951073172316</v>
       </c>
       <c r="E4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>8.7384000000000017E-2</v>
       </c>
       <c r="G4">
@@ -73522,11 +73518,11 @@
         <v>0.51559168523326704</v>
       </c>
       <c r="D5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.87427463774937164</v>
       </c>
       <c r="E5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0.10627200000000001</v>
       </c>
       <c r="G5">
@@ -73561,11 +73557,11 @@
         <v>0.5182907592915772</v>
       </c>
       <c r="D6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.91946537407678675</v>
       </c>
       <c r="E6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0.12656800000000001</v>
       </c>
       <c r="G6">
@@ -73596,15 +73592,15 @@
         <v>0.15</v>
       </c>
       <c r="C7">
+        <f t="shared" si="1"/>
+        <v>0.52397581857234621</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="2"/>
+        <v>1.000257649954988</v>
+      </c>
+      <c r="E7">
         <f t="shared" si="0"/>
-        <v>0.52397581857234621</v>
-      </c>
-      <c r="D7">
-        <f t="shared" si="1"/>
-        <v>1.000257649954988</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="2"/>
         <v>0.17100000000000004</v>
       </c>
       <c r="G7">
@@ -73635,15 +73631,15 @@
         <v>0.3</v>
       </c>
       <c r="C8">
+        <f t="shared" si="1"/>
+        <v>0.54017312099735892</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="2"/>
+        <v>1.1626780028409214</v>
+      </c>
+      <c r="E8">
         <f t="shared" si="0"/>
-        <v>0.54017312099735892</v>
-      </c>
-      <c r="D8">
-        <f t="shared" si="1"/>
-        <v>1.1626780028409214</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="2"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="G8">
@@ -73674,15 +73670,15 @@
         <v>0.45</v>
       </c>
       <c r="C9">
+        <f t="shared" si="1"/>
+        <v>0.5601205897026692</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="2"/>
+        <v>1.2886610169284807</v>
+      </c>
+      <c r="E9">
         <f t="shared" si="0"/>
-        <v>0.5601205897026692</v>
-      </c>
-      <c r="D9">
-        <f t="shared" si="1"/>
-        <v>1.2886610169284807</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="2"/>
         <v>0.44500000000000006</v>
       </c>
       <c r="G9">
@@ -73713,15 +73709,15 @@
         <v>0.6</v>
       </c>
       <c r="C10">
+        <f t="shared" si="1"/>
+        <v>0.58562746878441962</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="2"/>
+        <v>1.3915966349084505</v>
+      </c>
+      <c r="E10">
         <f t="shared" si="0"/>
-        <v>0.58562746878441962</v>
-      </c>
-      <c r="D10">
-        <f t="shared" si="1"/>
-        <v>1.3915966349084505</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="2"/>
         <v>0.59400000000000019</v>
       </c>
       <c r="G10">
@@ -73752,15 +73748,15 @@
         <v>0.75</v>
       </c>
       <c r="C11">
+        <f t="shared" si="1"/>
+        <v>0.62004588887311562</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="2"/>
+        <v>1.4786274600840028</v>
+      </c>
+      <c r="E11">
         <f t="shared" si="0"/>
-        <v>0.62004588887311562</v>
-      </c>
-      <c r="D11">
-        <f t="shared" si="1"/>
-        <v>1.4786274600840028</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="2"/>
         <v>0.7350000000000001</v>
       </c>
       <c r="G11">
@@ -73791,15 +73787,15 @@
         <v>0.85</v>
       </c>
       <c r="C12">
+        <f t="shared" si="1"/>
+        <v>0.67052815164442925</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="2"/>
+        <v>1.5540169901468119</v>
+      </c>
+      <c r="E12">
         <f t="shared" si="0"/>
-        <v>0.67052815164442925</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="1"/>
-        <v>1.5540169901468119</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="2"/>
         <v>0.85600000000000009</v>
       </c>
       <c r="G12">
@@ -73830,15 +73826,15 @@
         <v>0.95</v>
       </c>
       <c r="C13">
+        <f t="shared" si="1"/>
+        <v>0.75630419551640105</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>1.6205152685442648</v>
+      </c>
+      <c r="E13">
         <f t="shared" si="0"/>
-        <v>0.75630419551640105</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="1"/>
-        <v>1.6205152685442648</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="2"/>
         <v>0.94500000000000006</v>
       </c>
       <c r="G13">
@@ -73869,15 +73865,15 @@
         <v>1</v>
       </c>
       <c r="C14">
+        <f t="shared" si="1"/>
+        <v>0.96025256778912738</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>1.6800000056458275</v>
+      </c>
+      <c r="E14">
         <f t="shared" si="0"/>
-        <v>0.96025256778912738</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="1"/>
-        <v>1.6800000056458275</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="2"/>
         <v>0.99000000000000021</v>
       </c>
       <c r="G14">

</xml_diff>